<commit_message>
adding 3rd dive to deployment 23 in log, fixing some plotting routines, fix error in beamform_from_spec vectorized calculation, add option to not time average in beamform_from_spec_avg
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/sio_research/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D84052-5AB9-0244-A77D-E7BF8B2EC36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B29694A-1671-CB47-8DD0-FB7F851069D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10340" yWindow="3600" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1640" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="101">
   <si>
     <t>Deployment</t>
   </si>
@@ -667,11 +667,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1620,7 +1620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD1005"/>
+  <dimension ref="A1:AD1006"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="55" customWidth="1"/>
@@ -1954,7 +1954,7 @@
         <v>-63.696891999999998</v>
       </c>
       <c r="Y4" s="52">
-        <f t="shared" ref="Y4:Y38" si="0">(V4-S4)*1440/60</f>
+        <f t="shared" ref="Y4:Y39" si="0">(V4-S4)*1440/60</f>
         <v>9.1666666666860692</v>
       </c>
       <c r="Z4" s="24">
@@ -3117,7 +3117,7 @@
         <v>0.37708333333333338</v>
       </c>
       <c r="G20" s="53">
-        <f t="shared" ref="G20:G38" si="1">$F20+TIME(AC20,0,0)</f>
+        <f t="shared" ref="G20:G39" si="1">$F20+TIME(AC20,0,0)</f>
         <v>0.66875000000000007</v>
       </c>
       <c r="H20" s="33">
@@ -3317,7 +3317,7 @@
         <v>0.37847222222222227</v>
       </c>
       <c r="L22" s="36">
-        <f t="shared" ref="L22:L38" si="2">$K22 +TIME($AC22,0,0)</f>
+        <f t="shared" ref="L22:L39" si="2">$K22 +TIME($AC22,0,0)</f>
         <v>0.54513888888888895</v>
       </c>
       <c r="M22" s="33">
@@ -4691,7 +4691,7 @@
         <v>5</v>
       </c>
       <c r="D37" s="25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" s="26">
         <v>45317</v>
@@ -4765,26 +4765,26 @@
     </row>
     <row r="38" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="25">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B38" s="25" t="s">
         <v>98</v>
       </c>
       <c r="C38" s="25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D38" s="25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E38" s="26">
         <v>45317</v>
       </c>
       <c r="F38" s="27">
-        <v>0.63472222222222219</v>
+        <v>0.50972222222222219</v>
       </c>
       <c r="G38" s="27">
-        <f t="shared" si="1"/>
-        <v>0.96805555555555545</v>
+        <f t="shared" ref="G38" si="4">$F38+TIME(AC38,0,0)</f>
+        <v>0.84305555555555545</v>
       </c>
       <c r="H38" s="25"/>
       <c r="I38" s="25"/>
@@ -4792,45 +4792,45 @@
         <v>45320</v>
       </c>
       <c r="K38" s="28">
-        <v>0.51388888888888895</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="L38" s="28">
         <f t="shared" si="2"/>
-        <v>0.84722222222222232</v>
+        <v>0.90625</v>
       </c>
       <c r="M38" s="25"/>
       <c r="N38" s="25"/>
       <c r="O38" s="25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P38" s="25" t="s">
         <v>29</v>
       </c>
       <c r="Q38" s="29"/>
       <c r="R38" s="29" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="S38" s="30">
-        <v>45317.875324074077</v>
-      </c>
-      <c r="T38" s="63">
-        <v>32.909129</v>
-      </c>
-      <c r="U38" s="63">
-        <v>-117.680663</v>
+        <v>45319.910034722219</v>
+      </c>
+      <c r="T38" s="61">
+        <v>33.123451000000003</v>
+      </c>
+      <c r="U38" s="61">
+        <v>-117.600043</v>
       </c>
       <c r="V38" s="30">
-        <v>45318.878796296296</v>
-      </c>
-      <c r="W38" s="63">
-        <v>32.999972</v>
-      </c>
-      <c r="X38" s="63">
-        <v>-117.66408699999999</v>
+        <v>45320.89980324074</v>
+      </c>
+      <c r="W38" s="61">
+        <v>33.200189999999999</v>
+      </c>
+      <c r="X38" s="61">
+        <v>-117.597759</v>
       </c>
       <c r="Y38" s="52">
-        <f t="shared" si="0"/>
-        <v>24.083333333255723</v>
+        <f t="shared" ref="Y38" si="5">(V38-S38)*1440/60</f>
+        <v>23.754444444493856</v>
       </c>
       <c r="Z38" s="31">
         <v>0.6166666666666667</v>
@@ -4843,40 +4843,91 @@
         <v>8</v>
       </c>
       <c r="AD38" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="25"/>
-      <c r="B39" s="25"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
+      <c r="A39" s="25">
+        <v>24</v>
+      </c>
+      <c r="B39" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" s="25">
+        <v>6</v>
+      </c>
+      <c r="D39" s="25">
+        <v>1</v>
+      </c>
+      <c r="E39" s="26">
+        <v>45317</v>
+      </c>
+      <c r="F39" s="27">
+        <v>0.63472222222222219</v>
+      </c>
+      <c r="G39" s="27">
+        <f t="shared" si="1"/>
+        <v>0.96805555555555545</v>
+      </c>
       <c r="H39" s="25"/>
       <c r="I39" s="25"/>
-      <c r="J39" s="26"/>
-      <c r="K39" s="28"/>
-      <c r="L39" s="28"/>
+      <c r="J39" s="26">
+        <v>45320</v>
+      </c>
+      <c r="K39" s="28">
+        <v>0.51388888888888895</v>
+      </c>
+      <c r="L39" s="28">
+        <f t="shared" si="2"/>
+        <v>0.84722222222222232</v>
+      </c>
       <c r="M39" s="25"/>
       <c r="N39" s="25"/>
-      <c r="O39" s="25"/>
-      <c r="P39" s="25"/>
+      <c r="O39" s="25">
+        <v>4</v>
+      </c>
+      <c r="P39" s="25" t="s">
+        <v>29</v>
+      </c>
       <c r="Q39" s="29"/>
-      <c r="R39" s="29"/>
-      <c r="S39" s="30"/>
-      <c r="T39" s="25"/>
-      <c r="U39" s="25"/>
-      <c r="V39" s="30"/>
-      <c r="W39" s="25"/>
-      <c r="X39" s="25"/>
-      <c r="Y39" s="52"/>
-      <c r="Z39" s="31"/>
-      <c r="AA39" s="31"/>
+      <c r="R39" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="S39" s="30">
+        <v>45317.875324074077</v>
+      </c>
+      <c r="T39" s="61">
+        <v>32.909129</v>
+      </c>
+      <c r="U39" s="61">
+        <v>-117.680663</v>
+      </c>
+      <c r="V39" s="30">
+        <v>45318.878796296296</v>
+      </c>
+      <c r="W39" s="61">
+        <v>32.999972</v>
+      </c>
+      <c r="X39" s="61">
+        <v>-117.66408699999999</v>
+      </c>
+      <c r="Y39" s="52">
+        <f t="shared" si="0"/>
+        <v>24.083333333255723</v>
+      </c>
+      <c r="Z39" s="31">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AA39" s="31">
+        <v>5.2777777777777778E-2</v>
+      </c>
       <c r="AB39" s="25"/>
-      <c r="AC39" s="25"/>
-      <c r="AD39" s="25"/>
+      <c r="AC39" s="25">
+        <v>8</v>
+      </c>
+      <c r="AD39" s="25" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="40" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25"/>
@@ -4947,7 +4998,7 @@
       <c r="B42" s="25"/>
       <c r="C42" s="25"/>
       <c r="D42" s="25"/>
-      <c r="E42" s="57"/>
+      <c r="E42" s="26"/>
       <c r="F42" s="27"/>
       <c r="G42" s="27"/>
       <c r="H42" s="25"/>
@@ -4979,7 +5030,7 @@
       <c r="B43" s="25"/>
       <c r="C43" s="25"/>
       <c r="D43" s="25"/>
-      <c r="E43" s="26"/>
+      <c r="E43" s="57"/>
       <c r="F43" s="27"/>
       <c r="G43" s="27"/>
       <c r="H43" s="25"/>
@@ -35790,6 +35841,38 @@
       <c r="AC1005" s="25"/>
       <c r="AD1005" s="25"/>
     </row>
+    <row r="1006" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1006" s="25"/>
+      <c r="B1006" s="25"/>
+      <c r="C1006" s="25"/>
+      <c r="D1006" s="25"/>
+      <c r="E1006" s="26"/>
+      <c r="F1006" s="27"/>
+      <c r="G1006" s="27"/>
+      <c r="H1006" s="25"/>
+      <c r="I1006" s="25"/>
+      <c r="J1006" s="26"/>
+      <c r="K1006" s="28"/>
+      <c r="L1006" s="28"/>
+      <c r="M1006" s="25"/>
+      <c r="N1006" s="25"/>
+      <c r="O1006" s="25"/>
+      <c r="P1006" s="25"/>
+      <c r="Q1006" s="29"/>
+      <c r="R1006" s="29"/>
+      <c r="S1006" s="30"/>
+      <c r="T1006" s="25"/>
+      <c r="U1006" s="25"/>
+      <c r="V1006" s="30"/>
+      <c r="W1006" s="25"/>
+      <c r="X1006" s="25"/>
+      <c r="Y1006" s="52"/>
+      <c r="Z1006" s="31"/>
+      <c r="AA1006" s="31"/>
+      <c r="AB1006" s="25"/>
+      <c r="AC1006" s="25"/>
+      <c r="AD1006" s="25"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AD35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -35818,11 +35901,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
       <c r="D1" s="9" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Adding drift track fcn and script to plot tracks over bathymetry.  Fixing entries for deployment 24.
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/ThodeLab/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0EC4C3-CA19-9D44-934E-BCE3F67BB599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E929733D-E30F-3E4B-99ED-D6A71D920939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1460" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="113">
   <si>
     <t>Deployment</t>
   </si>
@@ -3328,7 +3328,7 @@
         <v>0.61805555555555558</v>
       </c>
       <c r="L21" s="32">
-        <f t="shared" ref="L21:L39" si="2">$J21+$K21 +TIME($AC21,0,0)</f>
+        <f t="shared" ref="L21:L40" si="2">$J21+$K21 +TIME($AC21,0,0)</f>
         <v>45204.784722222219</v>
       </c>
       <c r="M21" s="21">
@@ -4999,27 +4999,27 @@
       <c r="R39" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="S39" s="26">
-        <v>45317.875324074077</v>
+      <c r="S39" s="30">
+        <v>45317.993379629632</v>
       </c>
       <c r="T39" s="37">
-        <v>32.909129</v>
+        <v>32.907333000000001</v>
       </c>
       <c r="U39" s="37">
-        <v>-117.680663</v>
-      </c>
-      <c r="V39" s="26">
-        <v>45318.878796296296</v>
+        <v>-117.67442</v>
+      </c>
+      <c r="V39" s="30">
+        <v>45318.882280092592</v>
       </c>
       <c r="W39" s="37">
-        <v>32.999972</v>
+        <v>33.012383</v>
       </c>
       <c r="X39" s="37">
-        <v>-117.66408699999999</v>
+        <v>-117.66186500000001</v>
       </c>
       <c r="Y39" s="27">
         <f t="shared" si="0"/>
-        <v>24.083333333255723</v>
+        <v>21.333611111040227</v>
       </c>
       <c r="Z39" s="28">
         <v>0.6166666666666667</v>
@@ -5036,36 +5036,87 @@
       </c>
     </row>
     <row r="40" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
+      <c r="A40" s="21">
+        <v>24</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C40" s="21">
+        <v>6</v>
+      </c>
+      <c r="D40" s="21">
+        <v>1</v>
+      </c>
+      <c r="E40" s="22">
+        <v>45317</v>
+      </c>
+      <c r="F40" s="23">
+        <v>0.63472222222222219</v>
+      </c>
+      <c r="G40" s="10">
+        <f t="shared" ref="G40" si="4">$E40+$F40+TIME(AC40,0,0)</f>
+        <v>45317.968055555561</v>
+      </c>
       <c r="H40" s="21"/>
       <c r="I40" s="21"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="24"/>
-      <c r="L40" s="24"/>
+      <c r="J40" s="22">
+        <v>45320</v>
+      </c>
+      <c r="K40" s="24">
+        <v>0.51388888888888895</v>
+      </c>
+      <c r="L40" s="32">
+        <f t="shared" si="2"/>
+        <v>45320.847222222226</v>
+      </c>
       <c r="M40" s="21"/>
       <c r="N40" s="21"/>
-      <c r="O40" s="21"/>
-      <c r="P40" s="21"/>
+      <c r="O40" s="21">
+        <v>4</v>
+      </c>
+      <c r="P40" s="21" t="s">
+        <v>29</v>
+      </c>
       <c r="Q40" s="25"/>
-      <c r="R40" s="25"/>
-      <c r="S40" s="26"/>
-      <c r="T40" s="21"/>
-      <c r="U40" s="21"/>
-      <c r="V40" s="26"/>
-      <c r="W40" s="21"/>
-      <c r="X40" s="21"/>
-      <c r="Y40" s="27"/>
-      <c r="Z40" s="28"/>
-      <c r="AA40" s="28"/>
+      <c r="R40" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="S40" s="30">
+        <v>45318.882280092592</v>
+      </c>
+      <c r="T40" s="37">
+        <v>33.012383</v>
+      </c>
+      <c r="U40" s="37">
+        <v>-117.66186500000001</v>
+      </c>
+      <c r="V40" s="30">
+        <v>45320.848263888889</v>
+      </c>
+      <c r="W40" s="37">
+        <v>33.115271</v>
+      </c>
+      <c r="X40" s="37">
+        <v>-117.89773700000001</v>
+      </c>
+      <c r="Y40" s="27">
+        <f t="shared" ref="Y40" si="5">(V40-S40)*1440/60</f>
+        <v>47.183611111133359</v>
+      </c>
+      <c r="Z40" s="28">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AA40" s="28">
+        <v>5.2777777777777778E-2</v>
+      </c>
       <c r="AB40" s="21"/>
-      <c r="AC40" s="21"/>
-      <c r="AD40" s="21"/>
+      <c r="AC40" s="21">
+        <v>8</v>
+      </c>
+      <c r="AD40" s="21" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="41" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="21"/>
@@ -5089,7 +5140,7 @@
       <c r="S41" s="26"/>
       <c r="T41" s="21"/>
       <c r="U41" s="21"/>
-      <c r="V41" s="26"/>
+      <c r="V41" s="30"/>
       <c r="W41" s="21"/>
       <c r="X41" s="21"/>
       <c r="Y41" s="27"/>

</xml_diff>

<commit_message>
Added May 2024 metadata to spreadsheet.
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B96820-84EE-F547-BF9E-00DD42E4B758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927293E7-A575-C240-BC8F-70A92E324272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4760" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="124">
   <si>
     <t>Deployment</t>
   </si>
@@ -385,6 +385,36 @@
   <si>
     <t>Drifter</t>
   </si>
+  <si>
+    <t>2024_May_CA</t>
+  </si>
+  <si>
+    <t>acoustic_config_Drifter5_VS209_2024.txt</t>
+  </si>
+  <si>
+    <t>20240517T172653</t>
+  </si>
+  <si>
+    <t>20240520T193304</t>
+  </si>
+  <si>
+    <t>2024-05-19T19:21:43</t>
+  </si>
+  <si>
+    <t>2024-05-17T18:20:27</t>
+  </si>
+  <si>
+    <t>33.001117 </t>
+  </si>
+  <si>
+    <t> -117.872970</t>
+  </si>
+  <si>
+    <t>2024-05-19T21:43:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-05-20T10:14:28 </t>
+  </si>
 </sst>
 </file>
 
@@ -397,7 +427,7 @@
     <numFmt numFmtId="167" formatCode="0.00000000"/>
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -472,6 +502,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -548,7 +584,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -719,22 +755,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -747,6 +767,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1695,7 +1721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD1006"/>
+  <dimension ref="A1:AD1005"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="27" customWidth="1"/>
@@ -5141,67 +5167,155 @@
       </c>
     </row>
     <row r="41" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="20"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
+      <c r="A41" s="20">
+        <v>25</v>
+      </c>
+      <c r="B41" s="48" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" s="20">
+        <v>5</v>
+      </c>
+      <c r="D41" s="20">
+        <v>1</v>
+      </c>
+      <c r="E41" s="21">
+        <v>45429</v>
+      </c>
+      <c r="F41" s="22">
+        <v>0.43533564814814812</v>
+      </c>
+      <c r="G41" s="22" t="s">
+        <v>116</v>
+      </c>
       <c r="H41" s="20"/>
       <c r="I41" s="20"/>
-      <c r="J41" s="21"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
+      <c r="J41" s="21">
+        <v>45432</v>
+      </c>
+      <c r="K41" s="22">
+        <v>0.52296296296296296</v>
+      </c>
+      <c r="L41" s="22" t="s">
+        <v>117</v>
+      </c>
       <c r="M41" s="20"/>
       <c r="N41" s="20"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="20"/>
+      <c r="O41" s="20">
+        <v>3</v>
+      </c>
+      <c r="P41" s="20" t="s">
+        <v>29</v>
+      </c>
       <c r="Q41" s="23"/>
-      <c r="R41" s="23"/>
-      <c r="S41" s="24"/>
-      <c r="T41" s="20"/>
-      <c r="U41" s="20"/>
-      <c r="V41" s="28"/>
-      <c r="W41" s="20"/>
-      <c r="X41" s="20"/>
+      <c r="R41" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="S41" s="70" t="s">
+        <v>119</v>
+      </c>
+      <c r="T41" s="71">
+        <v>32.917650000000002</v>
+      </c>
+      <c r="U41" s="71">
+        <v>-117.794504</v>
+      </c>
+      <c r="V41" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="W41" s="71" t="s">
+        <v>120</v>
+      </c>
+      <c r="X41" s="71" t="s">
+        <v>121</v>
+      </c>
       <c r="Y41" s="25"/>
-      <c r="Z41" s="26"/>
-      <c r="AA41" s="26"/>
+      <c r="Z41" s="26">
+        <v>0.53263888888888888</v>
+      </c>
+      <c r="AA41" s="26">
+        <v>0.1125</v>
+      </c>
       <c r="AB41" s="20"/>
-      <c r="AC41" s="20"/>
+      <c r="AC41" s="20">
+        <v>7</v>
+      </c>
       <c r="AD41" s="20"/>
     </row>
     <row r="42" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="20"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
+      <c r="A42" s="20">
+        <v>26</v>
+      </c>
+      <c r="B42" s="48" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="20">
+        <v>5</v>
+      </c>
+      <c r="D42" s="20">
+        <v>2</v>
+      </c>
+      <c r="E42" s="21">
+        <v>45429</v>
+      </c>
+      <c r="F42" s="22">
+        <v>0.43533564814814812</v>
+      </c>
+      <c r="G42" s="22" t="s">
+        <v>116</v>
+      </c>
       <c r="H42" s="20"/>
       <c r="I42" s="20"/>
-      <c r="J42" s="21"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
+      <c r="J42" s="21">
+        <v>45432</v>
+      </c>
+      <c r="K42" s="22">
+        <v>0.52296296296296296</v>
+      </c>
+      <c r="L42" s="22" t="s">
+        <v>117</v>
+      </c>
       <c r="M42" s="20"/>
       <c r="N42" s="20"/>
-      <c r="O42" s="20"/>
-      <c r="P42" s="20"/>
+      <c r="O42" s="20">
+        <v>3</v>
+      </c>
+      <c r="P42" s="20" t="s">
+        <v>29</v>
+      </c>
       <c r="Q42" s="23"/>
-      <c r="R42" s="23"/>
-      <c r="S42" s="24"/>
-      <c r="T42" s="20"/>
-      <c r="U42" s="20"/>
-      <c r="V42" s="24"/>
-      <c r="W42" s="20"/>
-      <c r="X42" s="20"/>
+      <c r="R42" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="S42" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="T42" s="71">
+        <v>32.998700999999997</v>
+      </c>
+      <c r="U42" s="71">
+        <v>-117.874388</v>
+      </c>
+      <c r="V42" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="W42" s="71">
+        <v>33.012540000000001</v>
+      </c>
+      <c r="X42" s="20">
+        <v>-117.890097</v>
+      </c>
       <c r="Y42" s="25"/>
-      <c r="Z42" s="26"/>
-      <c r="AA42" s="26"/>
+      <c r="Z42" s="26">
+        <v>0.53263888888888888</v>
+      </c>
+      <c r="AA42" s="26">
+        <v>0.1125</v>
+      </c>
       <c r="AB42" s="20"/>
-      <c r="AC42" s="20"/>
+      <c r="AC42" s="20">
+        <v>7</v>
+      </c>
       <c r="AD42" s="20"/>
     </row>
     <row r="43" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5209,7 +5323,7 @@
       <c r="B43" s="20"/>
       <c r="C43" s="20"/>
       <c r="D43" s="20"/>
-      <c r="E43" s="36"/>
+      <c r="E43" s="21"/>
       <c r="F43" s="22"/>
       <c r="G43" s="22"/>
       <c r="H43" s="20"/>
@@ -5337,12 +5451,12 @@
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
       <c r="D47" s="20"/>
-      <c r="E47" s="21"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="20"/>
-      <c r="I47" s="20"/>
-      <c r="J47" s="21"/>
+      <c r="E47" s="70"/>
+      <c r="F47" s="71"/>
+      <c r="G47" s="71"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="71"/>
+      <c r="J47" s="71"/>
       <c r="K47" s="22"/>
       <c r="L47" s="22"/>
       <c r="M47" s="20"/>
@@ -5369,12 +5483,12 @@
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
       <c r="D48" s="20"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20"/>
-      <c r="J48" s="21"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="71"/>
+      <c r="G48" s="71"/>
+      <c r="H48" s="24"/>
+      <c r="I48" s="71"/>
+      <c r="J48" s="20"/>
       <c r="K48" s="22"/>
       <c r="L48" s="22"/>
       <c r="M48" s="20"/>
@@ -36020,38 +36134,6 @@
       <c r="AC1005" s="20"/>
       <c r="AD1005" s="20"/>
     </row>
-    <row r="1006" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1006" s="20"/>
-      <c r="B1006" s="20"/>
-      <c r="C1006" s="20"/>
-      <c r="D1006" s="20"/>
-      <c r="E1006" s="21"/>
-      <c r="F1006" s="22"/>
-      <c r="G1006" s="22"/>
-      <c r="H1006" s="20"/>
-      <c r="I1006" s="20"/>
-      <c r="J1006" s="21"/>
-      <c r="K1006" s="22"/>
-      <c r="L1006" s="22"/>
-      <c r="M1006" s="20"/>
-      <c r="N1006" s="20"/>
-      <c r="O1006" s="20"/>
-      <c r="P1006" s="20"/>
-      <c r="Q1006" s="23"/>
-      <c r="R1006" s="23"/>
-      <c r="S1006" s="24"/>
-      <c r="T1006" s="20"/>
-      <c r="U1006" s="20"/>
-      <c r="V1006" s="24"/>
-      <c r="W1006" s="20"/>
-      <c r="X1006" s="20"/>
-      <c r="Y1006" s="25"/>
-      <c r="Z1006" s="26"/>
-      <c r="AA1006" s="26"/>
-      <c r="AB1006" s="20"/>
-      <c r="AC1006" s="20"/>
-      <c r="AD1006" s="20"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:AD35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -36443,133 +36525,133 @@
       </c>
       <c r="H15" s="48"/>
     </row>
-    <row r="16" spans="1:8" s="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="66">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="20">
         <v>11</v>
       </c>
-      <c r="B16" s="66" t="s">
+      <c r="B16" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C16" s="66">
+      <c r="C16" s="20">
         <v>5</v>
       </c>
-      <c r="D16" s="66">
+      <c r="D16" s="20">
         <v>1</v>
       </c>
-      <c r="E16" s="67">
+      <c r="E16" s="21">
         <v>45317</v>
       </c>
-      <c r="F16" s="68">
+      <c r="F16" s="25">
         <v>24.083333333255723</v>
       </c>
-      <c r="G16" s="66" t="s">
+      <c r="G16" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="H16" s="66" t="s">
+      <c r="H16" s="20" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="66">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="20">
         <v>11</v>
       </c>
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C17" s="66">
+      <c r="C17" s="20">
         <v>5</v>
       </c>
-      <c r="D17" s="66">
+      <c r="D17" s="20">
         <v>2</v>
       </c>
-      <c r="E17" s="67">
+      <c r="E17" s="21">
         <v>45317</v>
       </c>
-      <c r="F17" s="68">
+      <c r="F17" s="25">
         <v>22.744166666641831</v>
       </c>
-      <c r="G17" s="66" t="s">
+      <c r="G17" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="H17" s="66" t="s">
+      <c r="H17" s="20" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="66">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="20">
         <v>11</v>
       </c>
-      <c r="B18" s="66" t="s">
+      <c r="B18" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="66">
+      <c r="C18" s="20">
         <v>5</v>
       </c>
-      <c r="D18" s="66">
+      <c r="D18" s="20">
         <v>3</v>
       </c>
-      <c r="E18" s="67">
+      <c r="E18" s="21">
         <v>45317</v>
       </c>
-      <c r="F18" s="68">
+      <c r="F18" s="25">
         <v>23.754444444493856</v>
       </c>
-      <c r="G18" s="66" t="s">
+      <c r="G18" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="H18" s="66" t="s">
+      <c r="H18" s="20" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="70">
+    <row r="19" spans="1:8" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="64">
         <v>12</v>
       </c>
-      <c r="B19" s="70" t="s">
+      <c r="B19" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="70">
+      <c r="C19" s="64">
         <v>6</v>
       </c>
-      <c r="D19" s="70">
+      <c r="D19" s="64">
         <v>1</v>
       </c>
-      <c r="E19" s="71">
+      <c r="E19" s="65">
         <v>45317</v>
       </c>
-      <c r="F19" s="72">
+      <c r="F19" s="66">
         <v>21.333611111040227</v>
       </c>
-      <c r="G19" s="70" t="s">
+      <c r="G19" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="H19" s="70" t="s">
+      <c r="H19" s="64" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="70">
+    <row r="20" spans="1:8" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="64">
         <v>12</v>
       </c>
-      <c r="B20" s="70" t="s">
+      <c r="B20" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="70">
+      <c r="C20" s="64">
         <v>6</v>
       </c>
-      <c r="D20" s="70">
+      <c r="D20" s="64">
         <v>1</v>
       </c>
-      <c r="E20" s="71">
+      <c r="E20" s="65">
         <v>45317</v>
       </c>
-      <c r="F20" s="72">
+      <c r="F20" s="66">
         <v>47.183611111133359</v>
       </c>
-      <c r="G20" s="70" t="s">
+      <c r="G20" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="70" t="s">
+      <c r="H20" s="64" t="s">
         <v>98</v>
       </c>
     </row>
@@ -46261,11 +46343,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
Updated XLS log for May 2024
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927293E7-A575-C240-BC8F-70A92E324272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA7BA71-7088-1648-B86C-A932AF568467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -767,12 +767,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -5211,22 +5211,22 @@
       <c r="R41" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="S41" s="70" t="s">
+      <c r="S41" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="T41" s="71">
+      <c r="T41" s="69">
         <v>32.917650000000002</v>
       </c>
-      <c r="U41" s="71">
+      <c r="U41" s="69">
         <v>-117.794504</v>
       </c>
       <c r="V41" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="W41" s="71" t="s">
+      <c r="W41" s="69" t="s">
         <v>120</v>
       </c>
-      <c r="X41" s="71" t="s">
+      <c r="X41" s="69" t="s">
         <v>121</v>
       </c>
       <c r="Y41" s="25"/>
@@ -5244,7 +5244,7 @@
     </row>
     <row r="42" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="20">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B42" s="48" t="s">
         <v>114</v>
@@ -5290,16 +5290,16 @@
       <c r="S42" s="24" t="s">
         <v>122</v>
       </c>
-      <c r="T42" s="71">
+      <c r="T42" s="69">
         <v>32.998700999999997</v>
       </c>
-      <c r="U42" s="71">
+      <c r="U42" s="69">
         <v>-117.874388</v>
       </c>
       <c r="V42" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="W42" s="71">
+      <c r="W42" s="69">
         <v>33.012540000000001</v>
       </c>
       <c r="X42" s="20">
@@ -5451,12 +5451,12 @@
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
       <c r="D47" s="20"/>
-      <c r="E47" s="70"/>
-      <c r="F47" s="71"/>
-      <c r="G47" s="71"/>
+      <c r="E47" s="68"/>
+      <c r="F47" s="69"/>
+      <c r="G47" s="69"/>
       <c r="H47" s="28"/>
-      <c r="I47" s="71"/>
-      <c r="J47" s="71"/>
+      <c r="I47" s="69"/>
+      <c r="J47" s="69"/>
       <c r="K47" s="22"/>
       <c r="L47" s="22"/>
       <c r="M47" s="20"/>
@@ -5484,10 +5484,10 @@
       <c r="C48" s="20"/>
       <c r="D48" s="20"/>
       <c r="E48" s="24"/>
-      <c r="F48" s="71"/>
-      <c r="G48" s="71"/>
+      <c r="F48" s="69"/>
+      <c r="G48" s="69"/>
       <c r="H48" s="24"/>
-      <c r="I48" s="71"/>
+      <c r="I48" s="69"/>
       <c r="J48" s="20"/>
       <c r="K48" s="22"/>
       <c r="L48" s="22"/>
@@ -46343,11 +46343,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="70" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
update deployment log, update getLinearDriftTrack to estimate speed and fix bug, update getDeployLog to calculate sunset/sunrise rather than read it in from the excel spreadsheet, estimate speed using readLatestGPS
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA7BA71-7088-1648-B86C-A932AF568467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49037BF2-BDF3-DC4B-8838-214863E3BF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="960" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="127">
   <si>
     <t>Deployment</t>
   </si>
@@ -415,19 +415,29 @@
   <si>
     <t xml:space="preserve">2024-05-20T10:14:28 </t>
   </si>
+  <si>
+    <t>2024_Seamounts</t>
+  </si>
+  <si>
+    <t>20240513T171747</t>
+  </si>
+  <si>
+    <t>20240513T211836</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\Thh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
     <numFmt numFmtId="167" formatCode="0.00000000"/>
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
+    <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,8 +519,15 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -541,8 +558,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -565,26 +588,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -668,13 +678,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="22" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -753,8 +759,6 @@
     <xf numFmtId="22" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -767,12 +771,67 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="168" fontId="2" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1743,8 +1802,8 @@
     <col min="20" max="21" width="10.83203125" style="27" customWidth="1"/>
     <col min="22" max="22" width="18.83203125" style="27" customWidth="1"/>
     <col min="23" max="24" width="10.83203125" style="27" customWidth="1"/>
-    <col min="25" max="25" width="14.1640625" style="37" customWidth="1"/>
-    <col min="26" max="27" width="15.1640625" style="38" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.1640625" style="35" customWidth="1"/>
+    <col min="26" max="27" width="15.1640625" style="36" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12.6640625" style="27" customWidth="1"/>
     <col min="29" max="29" width="45.1640625" style="27" customWidth="1"/>
     <col min="30" max="30" width="134" style="27" customWidth="1"/>
@@ -1843,67 +1902,67 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="39" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="39">
+    <row r="2" spans="1:30" s="37" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="37">
         <v>1</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="39">
+      <c r="C2" s="37">
         <v>4</v>
       </c>
-      <c r="D2" s="39">
+      <c r="D2" s="37">
         <v>1</v>
       </c>
-      <c r="E2" s="41">
+      <c r="E2" s="39">
         <v>44818</v>
       </c>
-      <c r="F2" s="42">
+      <c r="F2" s="40">
         <v>0.55138888888888882</v>
       </c>
-      <c r="G2" s="43"/>
-      <c r="H2" s="39">
+      <c r="G2" s="41"/>
+      <c r="H2" s="37">
         <v>39.865239000000003</v>
       </c>
-      <c r="I2" s="39">
+      <c r="I2" s="37">
         <v>-70.443644000000006</v>
       </c>
-      <c r="J2" s="41">
+      <c r="J2" s="39">
         <v>44818</v>
       </c>
-      <c r="K2" s="42">
+      <c r="K2" s="40">
         <v>0.66666666666666663</v>
       </c>
-      <c r="L2" s="42"/>
-      <c r="M2" s="39">
+      <c r="L2" s="40"/>
+      <c r="M2" s="37">
         <v>39.869919000000003</v>
       </c>
-      <c r="N2" s="39">
+      <c r="N2" s="37">
         <v>-70.432182999999995</v>
       </c>
-      <c r="O2" s="39">
+      <c r="O2" s="37">
         <v>1</v>
       </c>
-      <c r="P2" s="39" t="s">
+      <c r="P2" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="44">
+      <c r="Q2" s="42">
         <v>300434066482170</v>
       </c>
-      <c r="R2" s="44" t="s">
+      <c r="R2" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="S2" s="45"/>
-      <c r="V2" s="45"/>
-      <c r="Y2" s="46"/>
-      <c r="Z2" s="47">
+      <c r="S2" s="43"/>
+      <c r="V2" s="43"/>
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="45">
         <v>0.43124999999999997</v>
       </c>
-      <c r="AA2" s="47">
+      <c r="AA2" s="45">
         <v>0.45208333333333334</v>
       </c>
-      <c r="AD2" s="39" t="s">
+      <c r="AD2" s="37" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1992,83 +2051,83 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="39" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="39">
+    <row r="4" spans="1:30" s="37" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="37">
         <v>3</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="39">
+      <c r="C4" s="37">
         <v>4</v>
       </c>
-      <c r="D4" s="39">
+      <c r="D4" s="37">
         <v>1</v>
       </c>
-      <c r="E4" s="41">
+      <c r="E4" s="39">
         <v>44822</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="39">
+      <c r="F4" s="40"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="37">
         <v>38.944544999999998</v>
       </c>
-      <c r="I4" s="39">
+      <c r="I4" s="37">
         <v>-63.757482000000003</v>
       </c>
-      <c r="J4" s="41"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="39">
+      <c r="J4" s="39"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="37">
         <v>38.974831000000002</v>
       </c>
-      <c r="N4" s="39">
+      <c r="N4" s="37">
         <v>-63.683495000000001</v>
       </c>
-      <c r="O4" s="39">
+      <c r="O4" s="37">
         <v>1</v>
       </c>
-      <c r="P4" s="39" t="s">
+      <c r="P4" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" s="44">
+      <c r="Q4" s="42">
         <v>300434066482170</v>
       </c>
-      <c r="R4" s="44" t="s">
+      <c r="R4" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="S4" s="45">
+      <c r="S4" s="43">
         <v>44822.083333333336</v>
       </c>
-      <c r="T4" s="39">
+      <c r="T4" s="37">
         <v>38.941955</v>
       </c>
-      <c r="U4" s="39">
+      <c r="U4" s="37">
         <v>-63.756053000000001</v>
       </c>
-      <c r="V4" s="45">
+      <c r="V4" s="43">
         <v>44822.465277777781</v>
       </c>
-      <c r="W4" s="39">
+      <c r="W4" s="37">
         <v>38.973402999999998</v>
       </c>
-      <c r="X4" s="39">
+      <c r="X4" s="37">
         <v>-63.696891999999998</v>
       </c>
-      <c r="Y4" s="53">
+      <c r="Y4" s="51">
         <f t="shared" ref="Y4:Y39" si="0">(V4-S4)*1440/60</f>
         <v>9.1666666666860692</v>
       </c>
-      <c r="Z4" s="47">
+      <c r="Z4" s="45">
         <v>0.41597222222222219</v>
       </c>
-      <c r="AA4" s="47">
+      <c r="AA4" s="45">
         <v>0.92986111111111114</v>
       </c>
-      <c r="AB4" s="39">
+      <c r="AB4" s="37">
         <v>250</v>
       </c>
-      <c r="AD4" s="39" t="s">
+      <c r="AD4" s="37" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2151,84 +2210,84 @@
       <c r="AC5" s="20"/>
       <c r="AD5" s="20"/>
     </row>
-    <row r="6" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="48">
+    <row r="6" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="46">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="46">
         <v>4</v>
       </c>
-      <c r="D6" s="48">
+      <c r="D6" s="46">
         <v>1</v>
       </c>
-      <c r="E6" s="49">
+      <c r="E6" s="47">
         <v>44823</v>
       </c>
-      <c r="F6" s="50"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="48">
+      <c r="F6" s="48"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="46">
         <v>38.885973999999997</v>
       </c>
-      <c r="I6" s="48">
+      <c r="I6" s="46">
         <v>-64.015152</v>
       </c>
-      <c r="J6" s="49"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="50"/>
-      <c r="M6" s="48">
+      <c r="J6" s="47"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="46">
         <v>38.879128999999999</v>
       </c>
-      <c r="N6" s="48">
+      <c r="N6" s="46">
         <v>-63.895172000000002</v>
       </c>
-      <c r="O6" s="48">
+      <c r="O6" s="46">
         <v>1</v>
       </c>
-      <c r="P6" s="48" t="s">
+      <c r="P6" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q6" s="51">
+      <c r="Q6" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R6" s="51" t="s">
+      <c r="R6" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="S6" s="52">
+      <c r="S6" s="50">
         <v>44823.822916666664</v>
       </c>
-      <c r="T6" s="48">
+      <c r="T6" s="46">
         <v>38.886195999999998</v>
       </c>
-      <c r="U6" s="48">
+      <c r="U6" s="46">
         <v>-64.012355999999997</v>
       </c>
-      <c r="V6" s="52">
+      <c r="V6" s="50">
         <v>44824.329861111109</v>
       </c>
-      <c r="W6" s="48">
+      <c r="W6" s="46">
         <v>38.854120000000002</v>
       </c>
-      <c r="X6" s="48">
+      <c r="X6" s="46">
         <v>-63.966763999999998</v>
       </c>
-      <c r="Y6" s="53">
+      <c r="Y6" s="51">
         <f t="shared" si="0"/>
         <v>12.166666666686069</v>
       </c>
-      <c r="Z6" s="54">
+      <c r="Z6" s="52">
         <v>0.41666666666666669</v>
       </c>
-      <c r="AA6" s="54">
+      <c r="AA6" s="52">
         <v>0.92847222222222225</v>
       </c>
-      <c r="AB6" s="48">
+      <c r="AB6" s="46">
         <v>400</v>
       </c>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="48" t="s">
+      <c r="AC6" s="46"/>
+      <c r="AD6" s="46" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2319,305 +2378,305 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="48">
+    <row r="8" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="46">
         <v>7</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="48">
+      <c r="C8" s="46">
         <v>4</v>
       </c>
-      <c r="D8" s="48">
+      <c r="D8" s="46">
         <v>1</v>
       </c>
-      <c r="E8" s="49">
+      <c r="E8" s="47">
         <v>44983</v>
       </c>
-      <c r="F8" s="50"/>
-      <c r="G8" s="43" t="s">
+      <c r="F8" s="48"/>
+      <c r="G8" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="48"/>
-      <c r="I8" s="48"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50" t="s">
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="M8" s="48"/>
-      <c r="N8" s="48"/>
-      <c r="O8" s="48">
+      <c r="M8" s="46"/>
+      <c r="N8" s="46"/>
+      <c r="O8" s="46">
         <v>1</v>
       </c>
-      <c r="P8" s="48" t="s">
+      <c r="P8" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q8" s="51">
+      <c r="Q8" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R8" s="51" t="s">
+      <c r="R8" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S8" s="52">
+      <c r="S8" s="50">
         <v>44983.875324074077</v>
       </c>
-      <c r="T8" s="48">
+      <c r="T8" s="46">
         <v>32.910995</v>
       </c>
-      <c r="U8" s="48">
+      <c r="U8" s="46">
         <v>-117.74101400000001</v>
       </c>
-      <c r="V8" s="52">
+      <c r="V8" s="50">
         <v>44984.385752314818</v>
       </c>
-      <c r="W8" s="48">
+      <c r="W8" s="46">
         <v>32.911644000000003</v>
       </c>
-      <c r="X8" s="48">
+      <c r="X8" s="46">
         <v>-117.73635299999999</v>
       </c>
-      <c r="Y8" s="53">
+      <c r="Y8" s="51">
         <f t="shared" si="0"/>
         <v>12.250277777784504</v>
       </c>
-      <c r="Z8" s="54">
+      <c r="Z8" s="52">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA8" s="54">
+      <c r="AA8" s="52">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB8" s="48">
+      <c r="AB8" s="46">
         <v>250</v>
       </c>
-      <c r="AC8" s="48"/>
-      <c r="AD8" s="48"/>
-    </row>
-    <row r="9" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="48">
+      <c r="AC8" s="46"/>
+      <c r="AD8" s="46"/>
+    </row>
+    <row r="9" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="46">
         <v>7</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="48">
+      <c r="C9" s="46">
         <v>4</v>
       </c>
-      <c r="D9" s="48">
+      <c r="D9" s="46">
         <v>2</v>
       </c>
-      <c r="E9" s="49">
+      <c r="E9" s="47">
         <v>44983</v>
       </c>
-      <c r="F9" s="50"/>
-      <c r="G9" s="43" t="s">
+      <c r="F9" s="48"/>
+      <c r="G9" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H9" s="48"/>
-      <c r="I9" s="48"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50" t="s">
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="M9" s="48"/>
-      <c r="N9" s="48"/>
-      <c r="O9" s="48">
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46">
         <v>1</v>
       </c>
-      <c r="P9" s="48" t="s">
+      <c r="P9" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q9" s="51">
+      <c r="Q9" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R9" s="51" t="s">
+      <c r="R9" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S9" s="52">
+      <c r="S9" s="50">
         <v>44984.416990740741</v>
       </c>
-      <c r="T9" s="48">
+      <c r="T9" s="46">
         <v>32.908870999999998</v>
       </c>
-      <c r="U9" s="48">
+      <c r="U9" s="46">
         <v>-117.73746199999999</v>
       </c>
-      <c r="V9" s="52">
+      <c r="V9" s="50">
         <v>44984.896157407406</v>
       </c>
-      <c r="W9" s="48">
+      <c r="W9" s="46">
         <v>32.92512</v>
       </c>
-      <c r="X9" s="48">
+      <c r="X9" s="46">
         <v>-117.753174</v>
       </c>
-      <c r="Y9" s="53">
+      <c r="Y9" s="51">
         <f t="shared" si="0"/>
         <v>11.499999999941792</v>
       </c>
-      <c r="Z9" s="54">
+      <c r="Z9" s="52">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA9" s="54">
+      <c r="AA9" s="52">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB9" s="48">
+      <c r="AB9" s="46">
         <v>250</v>
       </c>
-      <c r="AC9" s="48"/>
-      <c r="AD9" s="48"/>
-    </row>
-    <row r="10" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="48">
+      <c r="AC9" s="46"/>
+      <c r="AD9" s="46"/>
+    </row>
+    <row r="10" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="46">
         <v>7</v>
       </c>
-      <c r="B10" s="48" t="s">
+      <c r="B10" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="48">
+      <c r="C10" s="46">
         <v>4</v>
       </c>
-      <c r="D10" s="48">
+      <c r="D10" s="46">
         <v>3</v>
       </c>
-      <c r="E10" s="49">
+      <c r="E10" s="47">
         <v>44983</v>
       </c>
-      <c r="F10" s="50"/>
-      <c r="G10" s="43" t="s">
+      <c r="F10" s="48"/>
+      <c r="G10" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="48"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="50"/>
-      <c r="L10" s="50" t="s">
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="M10" s="48"/>
-      <c r="N10" s="48"/>
-      <c r="O10" s="48">
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46">
         <v>1</v>
       </c>
-      <c r="P10" s="48" t="s">
+      <c r="P10" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q10" s="51">
+      <c r="Q10" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R10" s="51" t="s">
+      <c r="R10" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S10" s="52">
+      <c r="S10" s="50">
         <v>44984.896157407406</v>
       </c>
-      <c r="T10" s="48">
+      <c r="T10" s="46">
         <v>32.92512</v>
       </c>
-      <c r="U10" s="48">
+      <c r="U10" s="46">
         <v>-117.753174</v>
       </c>
-      <c r="V10" s="52">
+      <c r="V10" s="50">
         <v>44985.399629629632</v>
       </c>
-      <c r="W10" s="48">
+      <c r="W10" s="46">
         <v>32.922975999999998</v>
       </c>
-      <c r="X10" s="48">
+      <c r="X10" s="46">
         <v>-117.769451</v>
       </c>
-      <c r="Y10" s="53">
+      <c r="Y10" s="51">
         <f t="shared" si="0"/>
         <v>12.083333333430346</v>
       </c>
-      <c r="Z10" s="54">
+      <c r="Z10" s="52">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA10" s="54">
+      <c r="AA10" s="52">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB10" s="48">
+      <c r="AB10" s="46">
         <v>250</v>
       </c>
-      <c r="AC10" s="48"/>
-      <c r="AD10" s="48"/>
-    </row>
-    <row r="11" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="48">
+      <c r="AC10" s="46"/>
+      <c r="AD10" s="46"/>
+    </row>
+    <row r="11" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="46">
         <v>7</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="46">
         <v>4</v>
       </c>
-      <c r="D11" s="48">
+      <c r="D11" s="46">
         <v>4</v>
       </c>
-      <c r="E11" s="49">
+      <c r="E11" s="47">
         <v>44983</v>
       </c>
-      <c r="F11" s="50"/>
-      <c r="G11" s="43" t="s">
+      <c r="F11" s="48"/>
+      <c r="G11" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="48"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="50"/>
-      <c r="L11" s="50" t="s">
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48" t="s">
         <v>108</v>
       </c>
-      <c r="M11" s="48"/>
-      <c r="N11" s="48"/>
-      <c r="O11" s="48">
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46">
         <v>1</v>
       </c>
-      <c r="P11" s="48" t="s">
+      <c r="P11" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q11" s="51">
+      <c r="Q11" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R11" s="51" t="s">
+      <c r="R11" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S11" s="52">
+      <c r="S11" s="50">
         <v>44985.403113425928</v>
       </c>
-      <c r="T11" s="48">
+      <c r="T11" s="46">
         <v>32.922437000000002</v>
       </c>
-      <c r="U11" s="48">
+      <c r="U11" s="46">
         <v>-117.76988799999999</v>
       </c>
-      <c r="V11" s="52">
+      <c r="V11" s="50">
         <v>44985.885740740741</v>
       </c>
-      <c r="W11" s="48">
+      <c r="W11" s="46">
         <v>32.938851</v>
       </c>
-      <c r="X11" s="48">
+      <c r="X11" s="46">
         <v>-117.768916</v>
       </c>
-      <c r="Y11" s="53">
+      <c r="Y11" s="51">
         <f t="shared" si="0"/>
         <v>11.583055555529427</v>
       </c>
-      <c r="Z11" s="54">
+      <c r="Z11" s="52">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA11" s="54">
+      <c r="AA11" s="52">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB11" s="48">
+      <c r="AB11" s="46">
         <v>250</v>
       </c>
-      <c r="AC11" s="48"/>
-      <c r="AD11" s="48"/>
+      <c r="AC11" s="46"/>
+      <c r="AD11" s="46"/>
     </row>
     <row r="12" spans="1:30" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="20">
@@ -2779,84 +2838,84 @@
       <c r="AC13" s="20"/>
       <c r="AD13" s="20"/>
     </row>
-    <row r="14" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="48">
+    <row r="14" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="46">
         <v>9</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="48">
+      <c r="C14" s="46">
         <v>6</v>
       </c>
-      <c r="D14" s="48">
+      <c r="D14" s="46">
         <v>1</v>
       </c>
-      <c r="E14" s="49">
+      <c r="E14" s="47">
         <v>44985</v>
       </c>
-      <c r="F14" s="50"/>
-      <c r="G14" s="43" t="s">
+      <c r="F14" s="48"/>
+      <c r="G14" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="48">
+      <c r="H14" s="46">
         <v>32.912492</v>
       </c>
-      <c r="I14" s="48">
+      <c r="I14" s="46">
         <v>-117.69094200000001</v>
       </c>
-      <c r="J14" s="49"/>
-      <c r="K14" s="50"/>
-      <c r="L14" s="50" t="s">
+      <c r="J14" s="47"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="M14" s="48"/>
-      <c r="N14" s="48"/>
-      <c r="O14" s="48">
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46">
         <v>4</v>
       </c>
-      <c r="P14" s="48" t="s">
+      <c r="P14" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="51">
+      <c r="Q14" s="49">
         <v>300434066489180</v>
       </c>
-      <c r="R14" s="51" t="s">
+      <c r="R14" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="S14" s="52">
+      <c r="S14" s="50">
         <v>44985.715925925928</v>
       </c>
-      <c r="T14" s="48">
+      <c r="T14" s="46">
         <v>32.911934000000002</v>
       </c>
-      <c r="U14" s="48">
+      <c r="U14" s="46">
         <v>-117.691322</v>
       </c>
-      <c r="V14" s="52">
+      <c r="V14" s="50">
         <v>44985.788761574076</v>
       </c>
-      <c r="W14" s="48">
+      <c r="W14" s="46">
         <v>32.910586000000002</v>
       </c>
-      <c r="X14" s="48">
+      <c r="X14" s="46">
         <v>-117.69389</v>
       </c>
-      <c r="Y14" s="53">
+      <c r="Y14" s="51">
         <f t="shared" si="0"/>
         <v>1.7480555555666797</v>
       </c>
-      <c r="Z14" s="54">
+      <c r="Z14" s="52">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA14" s="54">
+      <c r="AA14" s="52">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB14" s="48">
+      <c r="AB14" s="46">
         <v>250</v>
       </c>
-      <c r="AC14" s="48"/>
-      <c r="AD14" s="48" t="s">
+      <c r="AC14" s="46"/>
+      <c r="AD14" s="46" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2951,155 +3010,155 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="48">
+    <row r="16" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="46">
         <v>11</v>
       </c>
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="48">
+      <c r="C16" s="46">
         <v>4</v>
       </c>
-      <c r="D16" s="48">
+      <c r="D16" s="46">
         <v>1</v>
       </c>
-      <c r="E16" s="49">
+      <c r="E16" s="47">
         <v>45084</v>
       </c>
-      <c r="F16" s="50"/>
-      <c r="G16" s="43" t="s">
+      <c r="F16" s="48"/>
+      <c r="G16" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="H16" s="48"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="50"/>
-      <c r="L16" s="50" t="s">
+      <c r="H16" s="46"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="47"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="M16" s="48"/>
-      <c r="N16" s="48"/>
-      <c r="O16" s="48">
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46">
         <v>1</v>
       </c>
-      <c r="P16" s="48" t="s">
+      <c r="P16" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q16" s="51">
+      <c r="Q16" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R16" s="51" t="s">
+      <c r="R16" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S16" s="52">
+      <c r="S16" s="50">
         <v>45084.72278935185</v>
       </c>
-      <c r="T16" s="48">
+      <c r="T16" s="46">
         <v>32.907145</v>
       </c>
-      <c r="U16" s="48">
+      <c r="U16" s="46">
         <v>-117.747221</v>
       </c>
-      <c r="V16" s="52">
+      <c r="V16" s="50">
         <v>45085.253900462965</v>
       </c>
-      <c r="W16" s="48">
+      <c r="W16" s="46">
         <v>32.939883999999999</v>
       </c>
-      <c r="X16" s="48">
+      <c r="X16" s="46">
         <v>-117.83437499999999</v>
       </c>
-      <c r="Y16" s="53">
+      <c r="Y16" s="51">
         <f t="shared" si="0"/>
         <v>12.746666666760575</v>
       </c>
-      <c r="Z16" s="54">
+      <c r="Z16" s="52">
         <v>0.52916666666666667</v>
       </c>
-      <c r="AA16" s="54">
+      <c r="AA16" s="52">
         <v>0.12291666666666667</v>
       </c>
-      <c r="AB16" s="48">
+      <c r="AB16" s="46">
         <v>250</v>
       </c>
-      <c r="AC16" s="48"/>
-      <c r="AD16" s="48"/>
-    </row>
-    <row r="17" spans="1:30" s="55" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="48">
+      <c r="AC16" s="46"/>
+      <c r="AD16" s="46"/>
+    </row>
+    <row r="17" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="46">
         <v>11</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="48">
+      <c r="C17" s="46">
         <v>4</v>
       </c>
-      <c r="D17" s="48">
+      <c r="D17" s="46">
         <v>2</v>
       </c>
-      <c r="E17" s="49">
+      <c r="E17" s="47">
         <v>45084</v>
       </c>
-      <c r="F17" s="50"/>
-      <c r="G17" s="43" t="s">
+      <c r="F17" s="48"/>
+      <c r="G17" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="H17" s="48"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="50"/>
-      <c r="L17" s="50" t="s">
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="M17" s="48"/>
-      <c r="N17" s="48"/>
-      <c r="O17" s="48">
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+      <c r="O17" s="46">
         <v>1</v>
       </c>
-      <c r="P17" s="48" t="s">
+      <c r="P17" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q17" s="51">
+      <c r="Q17" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R17" s="51" t="s">
+      <c r="R17" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="S17" s="56">
+      <c r="S17" s="54">
         <v>45085.26767361111</v>
       </c>
-      <c r="T17" s="57">
+      <c r="T17" s="55">
         <v>32.939607000000002</v>
       </c>
-      <c r="U17" s="57">
+      <c r="U17" s="55">
         <v>-117.834576</v>
       </c>
-      <c r="V17" s="56">
+      <c r="V17" s="54">
         <v>45085.753796296296</v>
       </c>
-      <c r="W17" s="57">
+      <c r="W17" s="55">
         <v>32.963126000000003</v>
       </c>
-      <c r="X17" s="57">
+      <c r="X17" s="55">
         <v>-117.875584</v>
       </c>
-      <c r="Y17" s="53">
+      <c r="Y17" s="51">
         <f t="shared" si="0"/>
         <v>11.666944444470573</v>
       </c>
-      <c r="Z17" s="54">
+      <c r="Z17" s="52">
         <v>0.52916666666666667</v>
       </c>
-      <c r="AA17" s="54">
+      <c r="AA17" s="52">
         <v>0.12291666666666667</v>
       </c>
-      <c r="AB17" s="48">
+      <c r="AB17" s="46">
         <v>250</v>
       </c>
-      <c r="AC17" s="48"/>
-      <c r="AD17" s="48"/>
+      <c r="AC17" s="46"/>
+      <c r="AD17" s="46"/>
     </row>
     <row r="18" spans="1:30" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="20">
@@ -3251,94 +3310,94 @@
       <c r="AC19" s="20"/>
       <c r="AD19" s="20"/>
     </row>
-    <row r="20" spans="1:30" s="59" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="48">
+    <row r="20" spans="1:30" s="57" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="46">
         <v>13</v>
       </c>
-      <c r="B20" s="48" t="s">
+      <c r="B20" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="48">
+      <c r="C20" s="46">
         <v>6</v>
       </c>
-      <c r="D20" s="48">
+      <c r="D20" s="46">
         <v>1</v>
       </c>
-      <c r="E20" s="49">
+      <c r="E20" s="47">
         <v>45176</v>
       </c>
-      <c r="F20" s="50">
+      <c r="F20" s="48">
         <v>0.37708333333333338</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="41">
         <f>$E20+$F20+TIME(AC20,0,0)</f>
         <v>45176.668749999997</v>
       </c>
-      <c r="H20" s="48">
+      <c r="H20" s="46">
         <v>32.910367999999998</v>
       </c>
-      <c r="I20" s="48">
+      <c r="I20" s="46">
         <v>-117.737223</v>
       </c>
-      <c r="J20" s="49">
+      <c r="J20" s="47">
         <v>45180</v>
       </c>
-      <c r="K20" s="50">
+      <c r="K20" s="48">
         <v>0.25</v>
       </c>
-      <c r="L20" s="58">
+      <c r="L20" s="56">
         <f>$J20+$K20 +TIME($AC20,0,0)</f>
         <v>45180.541666666664</v>
       </c>
-      <c r="M20" s="48"/>
-      <c r="N20" s="48"/>
-      <c r="O20" s="48">
+      <c r="M20" s="46"/>
+      <c r="N20" s="46"/>
+      <c r="O20" s="46">
         <v>4</v>
       </c>
-      <c r="P20" s="48" t="s">
+      <c r="P20" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="51">
+      <c r="Q20" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R20" s="51" t="s">
+      <c r="R20" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="S20" s="56">
+      <c r="S20" s="54">
         <v>45176.681122685186</v>
       </c>
-      <c r="T20" s="57">
+      <c r="T20" s="55">
         <v>32.911997999999997</v>
       </c>
-      <c r="U20" s="57">
+      <c r="U20" s="55">
         <v>-117.736034</v>
       </c>
-      <c r="V20" s="56">
+      <c r="V20" s="54">
         <v>45180.389189814814</v>
       </c>
-      <c r="W20" s="57">
+      <c r="W20" s="55">
         <v>32.880761</v>
       </c>
-      <c r="X20" s="57">
+      <c r="X20" s="55">
         <v>-117.434878</v>
       </c>
-      <c r="Y20" s="53">
+      <c r="Y20" s="51">
         <f t="shared" si="0"/>
         <v>88.993611111072823</v>
       </c>
-      <c r="Z20" s="54">
+      <c r="Z20" s="52">
         <v>0.57361111111111118</v>
       </c>
-      <c r="AA20" s="54">
+      <c r="AA20" s="52">
         <v>6.2847222222222221E-2</v>
       </c>
-      <c r="AB20" s="48">
+      <c r="AB20" s="46">
         <v>250</v>
       </c>
-      <c r="AC20" s="48">
+      <c r="AC20" s="46">
         <v>7</v>
       </c>
-      <c r="AD20" s="48"/>
+      <c r="AD20" s="46"/>
     </row>
     <row r="21" spans="1:30" s="31" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="20">
@@ -3435,193 +3494,193 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="48">
+    <row r="22" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="46">
         <v>15</v>
       </c>
-      <c r="B22" s="48" t="s">
+      <c r="B22" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="48">
+      <c r="C22" s="46">
         <v>5</v>
       </c>
-      <c r="D22" s="48">
+      <c r="D22" s="46">
         <v>1</v>
       </c>
-      <c r="E22" s="49">
+      <c r="E22" s="47">
         <v>45203</v>
       </c>
-      <c r="F22" s="50">
+      <c r="F22" s="48">
         <v>0.29444444444444445</v>
       </c>
-      <c r="G22" s="43">
+      <c r="G22" s="41">
         <f t="shared" si="1"/>
         <v>45203.461111111108</v>
       </c>
-      <c r="H22" s="48">
+      <c r="H22" s="46">
         <v>38.708799999999997</v>
       </c>
-      <c r="I22" s="48">
+      <c r="I22" s="46">
         <v>-64.031542999999999</v>
       </c>
-      <c r="J22" s="49">
+      <c r="J22" s="47">
         <v>45205</v>
       </c>
-      <c r="K22" s="50">
+      <c r="K22" s="48">
         <v>0.37847222222222227</v>
       </c>
-      <c r="L22" s="58">
+      <c r="L22" s="56">
         <f t="shared" si="2"/>
         <v>45205.545138888883</v>
       </c>
-      <c r="M22" s="48">
+      <c r="M22" s="46">
         <v>38.943779999999997</v>
       </c>
-      <c r="N22" s="48">
+      <c r="N22" s="46">
         <v>-64.196479999999994</v>
       </c>
-      <c r="O22" s="48">
+      <c r="O22" s="46">
         <v>3</v>
       </c>
-      <c r="P22" s="48" t="s">
+      <c r="P22" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q22" s="51">
+      <c r="Q22" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R22" s="51" t="s">
+      <c r="R22" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S22" s="52">
+      <c r="S22" s="50">
         <v>45203.535277777781</v>
       </c>
-      <c r="T22" s="57">
+      <c r="T22" s="55">
         <v>38.722087999999999</v>
       </c>
-      <c r="U22" s="57">
+      <c r="U22" s="55">
         <v>-64.021294999999995</v>
       </c>
-      <c r="V22" s="52">
+      <c r="V22" s="50">
         <v>45204.719074074077</v>
       </c>
-      <c r="W22" s="57">
+      <c r="W22" s="55">
         <v>38.866824999999999</v>
       </c>
-      <c r="X22" s="57">
+      <c r="X22" s="55">
         <v>-64.043930000000003</v>
       </c>
-      <c r="Y22" s="53">
+      <c r="Y22" s="51">
         <f t="shared" si="0"/>
         <v>28.411111111112405</v>
       </c>
-      <c r="Z22" s="54">
+      <c r="Z22" s="52">
         <v>0.42708333333333331</v>
       </c>
-      <c r="AA22" s="54">
+      <c r="AA22" s="52">
         <v>0.91180555555555554</v>
       </c>
-      <c r="AB22" s="48">
+      <c r="AB22" s="46">
         <v>300</v>
       </c>
-      <c r="AC22" s="48">
+      <c r="AC22" s="46">
         <v>4</v>
       </c>
-      <c r="AD22" s="48" t="s">
+      <c r="AD22" s="46" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="48">
+    <row r="23" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="46">
         <v>15</v>
       </c>
-      <c r="B23" s="48" t="s">
+      <c r="B23" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="48">
+      <c r="C23" s="46">
         <v>5</v>
       </c>
-      <c r="D23" s="48">
+      <c r="D23" s="46">
         <v>2</v>
       </c>
-      <c r="E23" s="49">
+      <c r="E23" s="47">
         <v>45203</v>
       </c>
-      <c r="F23" s="50">
+      <c r="F23" s="48">
         <v>0.29444444444444445</v>
       </c>
-      <c r="G23" s="43">
+      <c r="G23" s="41">
         <f t="shared" si="1"/>
         <v>45203.461111111108</v>
       </c>
-      <c r="H23" s="48">
+      <c r="H23" s="46">
         <v>38.708799999999997</v>
       </c>
-      <c r="I23" s="48">
+      <c r="I23" s="46">
         <v>-64.031542999999999</v>
       </c>
-      <c r="J23" s="49">
+      <c r="J23" s="47">
         <v>45205</v>
       </c>
-      <c r="K23" s="50">
+      <c r="K23" s="48">
         <v>0.37847222222222227</v>
       </c>
-      <c r="L23" s="58">
+      <c r="L23" s="56">
         <f t="shared" si="2"/>
         <v>45205.545138888883</v>
       </c>
-      <c r="M23" s="48">
+      <c r="M23" s="46">
         <v>38.943779999999997</v>
       </c>
-      <c r="N23" s="48">
+      <c r="N23" s="46">
         <v>-64.196479999999994</v>
       </c>
-      <c r="O23" s="48">
+      <c r="O23" s="46">
         <v>3</v>
       </c>
-      <c r="P23" s="48" t="s">
+      <c r="P23" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q23" s="51">
+      <c r="Q23" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R23" s="51" t="s">
+      <c r="R23" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S23" s="56">
+      <c r="S23" s="54">
         <v>45204.812939814816</v>
       </c>
-      <c r="T23" s="57">
+      <c r="T23" s="55">
         <v>38.887227000000003</v>
       </c>
-      <c r="U23" s="57">
+      <c r="U23" s="55">
         <v>-64.073801000000003</v>
       </c>
-      <c r="V23" s="56">
+      <c r="V23" s="54">
         <v>45205.389224537037</v>
       </c>
-      <c r="W23" s="57">
+      <c r="W23" s="55">
         <v>38.930204000000003</v>
       </c>
-      <c r="X23" s="57">
+      <c r="X23" s="55">
         <v>-64.167721999999998</v>
       </c>
-      <c r="Y23" s="53">
+      <c r="Y23" s="51">
         <f t="shared" si="0"/>
         <v>13.830833333311602</v>
       </c>
-      <c r="Z23" s="54">
+      <c r="Z23" s="52">
         <v>0.42708333333333331</v>
       </c>
-      <c r="AA23" s="54">
+      <c r="AA23" s="52">
         <v>0.91180555555555554</v>
       </c>
-      <c r="AB23" s="48">
+      <c r="AB23" s="46">
         <v>300</v>
       </c>
-      <c r="AC23" s="48">
+      <c r="AC23" s="46">
         <v>4</v>
       </c>
-      <c r="AD23" s="48" t="s">
+      <c r="AD23" s="46" t="s">
         <v>49</v>
       </c>
     </row>
@@ -3811,284 +3870,284 @@
       </c>
       <c r="AD25" s="20"/>
     </row>
-    <row r="26" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="48">
+    <row r="26" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="46">
         <v>17</v>
       </c>
-      <c r="B26" s="48" t="s">
+      <c r="B26" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="48">
+      <c r="C26" s="46">
         <v>6</v>
       </c>
-      <c r="D26" s="48">
+      <c r="D26" s="46">
         <v>1</v>
       </c>
-      <c r="E26" s="49">
+      <c r="E26" s="47">
         <v>45207</v>
       </c>
-      <c r="F26" s="50">
+      <c r="F26" s="48">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G26" s="43">
+      <c r="G26" s="41">
         <f t="shared" si="1"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H26" s="48">
+      <c r="H26" s="46">
         <v>38.767780000000002</v>
       </c>
-      <c r="I26" s="48">
+      <c r="I26" s="46">
         <v>-63.738374</v>
       </c>
-      <c r="J26" s="49">
+      <c r="J26" s="47">
         <v>45210</v>
       </c>
-      <c r="K26" s="50">
+      <c r="K26" s="48">
         <v>0.40625</v>
       </c>
-      <c r="L26" s="58">
+      <c r="L26" s="56">
         <f t="shared" si="2"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M26" s="59">
+      <c r="M26" s="57">
         <v>38.954067000000002</v>
       </c>
-      <c r="N26" s="48">
+      <c r="N26" s="46">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O26" s="48">
+      <c r="O26" s="46">
         <v>4</v>
       </c>
-      <c r="P26" s="48" t="s">
+      <c r="P26" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q26" s="51">
+      <c r="Q26" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R26" s="51" t="s">
+      <c r="R26" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="S26" s="56">
+      <c r="S26" s="54">
         <v>45208.132511574076</v>
       </c>
-      <c r="T26" s="60">
+      <c r="T26" s="58">
         <v>38.769841999999997</v>
       </c>
-      <c r="U26" s="60">
+      <c r="U26" s="58">
         <v>-63.7483</v>
       </c>
-      <c r="V26" s="56">
+      <c r="V26" s="54">
         <v>45208.63921296296</v>
       </c>
-      <c r="W26" s="60">
+      <c r="W26" s="58">
         <v>38.832385000000002</v>
       </c>
-      <c r="X26" s="60">
+      <c r="X26" s="58">
         <v>-63.796340000000001</v>
       </c>
-      <c r="Y26" s="53">
+      <c r="Y26" s="51">
         <f t="shared" si="0"/>
         <v>12.160833333211485</v>
       </c>
-      <c r="Z26" s="54">
+      <c r="Z26" s="52">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA26" s="54">
+      <c r="AA26" s="52">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB26" s="48">
+      <c r="AB26" s="46">
         <v>200</v>
       </c>
-      <c r="AC26" s="48">
+      <c r="AC26" s="46">
         <v>4</v>
       </c>
-      <c r="AD26" s="48"/>
-    </row>
-    <row r="27" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="48">
+      <c r="AD26" s="46"/>
+    </row>
+    <row r="27" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="46">
         <v>17</v>
       </c>
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="48">
+      <c r="C27" s="46">
         <v>6</v>
       </c>
-      <c r="D27" s="48">
+      <c r="D27" s="46">
         <v>2</v>
       </c>
-      <c r="E27" s="49">
+      <c r="E27" s="47">
         <v>45207</v>
       </c>
-      <c r="F27" s="50">
+      <c r="F27" s="48">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G27" s="43">
+      <c r="G27" s="41">
         <f t="shared" si="1"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H27" s="48">
+      <c r="H27" s="46">
         <v>38.767780000000002</v>
       </c>
-      <c r="I27" s="48">
+      <c r="I27" s="46">
         <v>-63.738374</v>
       </c>
-      <c r="J27" s="49">
+      <c r="J27" s="47">
         <v>45210</v>
       </c>
-      <c r="K27" s="50">
+      <c r="K27" s="48">
         <v>0.40625</v>
       </c>
-      <c r="L27" s="58">
+      <c r="L27" s="56">
         <f t="shared" si="2"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M27" s="59">
+      <c r="M27" s="57">
         <v>38.954067000000002</v>
       </c>
-      <c r="N27" s="48">
+      <c r="N27" s="46">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O27" s="48">
+      <c r="O27" s="46">
         <v>4</v>
       </c>
-      <c r="P27" s="48" t="s">
+      <c r="P27" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q27" s="51">
+      <c r="Q27" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R27" s="51" t="s">
+      <c r="R27" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="S27" s="56">
+      <c r="S27" s="54">
         <v>45208.771828703706</v>
       </c>
-      <c r="T27" s="60">
+      <c r="T27" s="58">
         <v>38.857106999999999</v>
       </c>
-      <c r="U27" s="60">
+      <c r="U27" s="58">
         <v>-63.781923999999997</v>
       </c>
-      <c r="V27" s="56">
+      <c r="V27" s="54">
         <v>45209.656574074077</v>
       </c>
-      <c r="W27" s="60">
+      <c r="W27" s="58">
         <v>38.923247000000003</v>
       </c>
-      <c r="X27" s="60">
+      <c r="X27" s="58">
         <v>-63.812421999999998</v>
       </c>
-      <c r="Y27" s="53">
+      <c r="Y27" s="51">
         <f t="shared" si="0"/>
         <v>21.233888888906222</v>
       </c>
-      <c r="Z27" s="54">
+      <c r="Z27" s="52">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA27" s="54">
+      <c r="AA27" s="52">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB27" s="48">
+      <c r="AB27" s="46">
         <v>300</v>
       </c>
-      <c r="AC27" s="48">
+      <c r="AC27" s="46">
         <v>4</v>
       </c>
-      <c r="AD27" s="48"/>
-    </row>
-    <row r="28" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="48">
+      <c r="AD27" s="46"/>
+    </row>
+    <row r="28" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="46">
         <v>17</v>
       </c>
-      <c r="B28" s="48" t="s">
+      <c r="B28" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="48">
+      <c r="C28" s="46">
         <v>6</v>
       </c>
-      <c r="D28" s="48">
+      <c r="D28" s="46">
         <v>3</v>
       </c>
-      <c r="E28" s="49">
+      <c r="E28" s="47">
         <v>45207</v>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="48">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G28" s="43">
+      <c r="G28" s="41">
         <f t="shared" si="1"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H28" s="48">
+      <c r="H28" s="46">
         <v>38.767780000000002</v>
       </c>
-      <c r="I28" s="48">
+      <c r="I28" s="46">
         <v>-63.738374</v>
       </c>
-      <c r="J28" s="49">
+      <c r="J28" s="47">
         <v>45210</v>
       </c>
-      <c r="K28" s="50">
+      <c r="K28" s="48">
         <v>0.40625</v>
       </c>
-      <c r="L28" s="58">
+      <c r="L28" s="56">
         <f t="shared" si="2"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M28" s="59">
+      <c r="M28" s="57">
         <v>38.954067000000002</v>
       </c>
-      <c r="N28" s="48">
+      <c r="N28" s="46">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O28" s="48">
+      <c r="O28" s="46">
         <v>4</v>
       </c>
-      <c r="P28" s="48" t="s">
+      <c r="P28" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q28" s="51">
+      <c r="Q28" s="49">
         <v>300434066480130</v>
       </c>
-      <c r="R28" s="51" t="s">
+      <c r="R28" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="S28" s="56">
+      <c r="S28" s="54">
         <v>45209.750567129631</v>
       </c>
-      <c r="T28" s="60">
+      <c r="T28" s="58">
         <v>38.923658000000003</v>
       </c>
-      <c r="U28" s="60">
+      <c r="U28" s="58">
         <v>-63.819659000000001</v>
       </c>
-      <c r="V28" s="56">
+      <c r="V28" s="54">
         <v>45210.542002314818</v>
       </c>
-      <c r="W28" s="60">
+      <c r="W28" s="58">
         <v>38.940576999999998</v>
       </c>
-      <c r="X28" s="60">
+      <c r="X28" s="58">
         <v>-63.867663</v>
       </c>
-      <c r="Y28" s="53">
+      <c r="Y28" s="51">
         <f t="shared" si="0"/>
         <v>18.994444444484543</v>
       </c>
-      <c r="Z28" s="54">
+      <c r="Z28" s="52">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA28" s="54">
+      <c r="AA28" s="52">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB28" s="48">
+      <c r="AB28" s="46">
         <v>200</v>
       </c>
-      <c r="AC28" s="48">
+      <c r="AC28" s="46">
         <v>4</v>
       </c>
-      <c r="AD28" s="48"/>
+      <c r="AD28" s="46"/>
     </row>
     <row r="29" spans="1:30" s="31" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20">
@@ -4278,98 +4337,98 @@
       </c>
       <c r="AD30" s="20"/>
     </row>
-    <row r="31" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="48">
+    <row r="31" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="46">
         <v>19</v>
       </c>
-      <c r="B31" s="48" t="s">
+      <c r="B31" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="48">
+      <c r="C31" s="46">
         <v>5</v>
       </c>
-      <c r="D31" s="48">
+      <c r="D31" s="46">
         <v>1</v>
       </c>
-      <c r="E31" s="49">
+      <c r="E31" s="47">
         <v>45208</v>
       </c>
-      <c r="F31" s="50">
+      <c r="F31" s="48">
         <v>0.59722222222222221</v>
       </c>
-      <c r="G31" s="43">
+      <c r="G31" s="41">
         <f t="shared" si="1"/>
         <v>45208.763888888883</v>
       </c>
-      <c r="H31" s="48">
+      <c r="H31" s="46">
         <v>38.826842999999997</v>
       </c>
-      <c r="I31" s="48">
+      <c r="I31" s="46">
         <v>-63.845635000000001</v>
       </c>
-      <c r="J31" s="49">
+      <c r="J31" s="47">
         <v>45209</v>
       </c>
-      <c r="K31" s="50">
+      <c r="K31" s="48">
         <v>0.36805555555555558</v>
       </c>
-      <c r="L31" s="58">
+      <c r="L31" s="56">
         <f t="shared" si="2"/>
         <v>45209.534722222219</v>
       </c>
-      <c r="M31" s="48">
+      <c r="M31" s="46">
         <v>38.862192</v>
       </c>
-      <c r="N31" s="48">
+      <c r="N31" s="46">
         <v>-63.908256999999999</v>
       </c>
-      <c r="O31" s="48">
+      <c r="O31" s="46">
         <v>3</v>
       </c>
-      <c r="P31" s="48" t="s">
+      <c r="P31" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q31" s="51">
+      <c r="Q31" s="49">
         <v>300434066482170</v>
       </c>
-      <c r="R31" s="51" t="s">
+      <c r="R31" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S31" s="56">
+      <c r="S31" s="54">
         <v>45208.77138888889</v>
       </c>
-      <c r="T31" s="60">
+      <c r="T31" s="58">
         <v>38.827702000000002</v>
       </c>
-      <c r="U31" s="60">
+      <c r="U31" s="58">
         <v>-63.844456999999998</v>
       </c>
-      <c r="V31" s="52">
+      <c r="V31" s="50">
         <v>45209.26421296296</v>
       </c>
-      <c r="W31" s="60">
+      <c r="W31" s="58">
         <v>38.862524999999998</v>
       </c>
-      <c r="X31" s="60">
+      <c r="X31" s="58">
         <v>-63.894246000000003</v>
       </c>
-      <c r="Y31" s="53">
+      <c r="Y31" s="51">
         <f t="shared" si="0"/>
         <v>11.827777777682059</v>
       </c>
-      <c r="Z31" s="54">
+      <c r="Z31" s="52">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA31" s="54">
+      <c r="AA31" s="52">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB31" s="48">
+      <c r="AB31" s="46">
         <v>100</v>
       </c>
-      <c r="AC31" s="48">
+      <c r="AC31" s="46">
         <v>4</v>
       </c>
-      <c r="AD31" s="48" t="s">
+      <c r="AD31" s="46" t="s">
         <v>47</v>
       </c>
     </row>
@@ -4439,7 +4498,7 @@
       <c r="U32" s="32">
         <v>-63.895504000000003</v>
       </c>
-      <c r="V32" s="33">
+      <c r="V32" s="28">
         <v>45211.541979166665</v>
       </c>
       <c r="W32" s="32">
@@ -4534,7 +4593,7 @@
       <c r="U33" s="32">
         <v>-63.899909000000001</v>
       </c>
-      <c r="V33" s="34">
+      <c r="V33" s="33">
         <v>45212.556122685186</v>
       </c>
       <c r="W33" s="32">
@@ -4561,98 +4620,98 @@
       </c>
       <c r="AD33" s="20"/>
     </row>
-    <row r="34" spans="1:30" s="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="48">
+    <row r="34" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="46">
         <v>21</v>
       </c>
-      <c r="B34" s="48" t="s">
+      <c r="B34" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="48">
+      <c r="C34" s="46">
         <v>4</v>
       </c>
-      <c r="D34" s="48">
+      <c r="D34" s="46">
         <v>1</v>
       </c>
-      <c r="E34" s="49">
+      <c r="E34" s="47">
         <v>45211</v>
       </c>
-      <c r="F34" s="50">
+      <c r="F34" s="48">
         <v>0.60416666666666663</v>
       </c>
-      <c r="G34" s="43">
+      <c r="G34" s="41">
         <f t="shared" si="1"/>
         <v>45211.770833333328</v>
       </c>
-      <c r="H34" s="48">
+      <c r="H34" s="46">
         <v>38.834505</v>
       </c>
-      <c r="I34" s="48">
+      <c r="I34" s="46">
         <v>-63.75074</v>
       </c>
-      <c r="J34" s="49">
+      <c r="J34" s="47">
         <v>45212</v>
       </c>
-      <c r="K34" s="50">
+      <c r="K34" s="48">
         <v>0.54166666666666663</v>
       </c>
-      <c r="L34" s="58">
+      <c r="L34" s="56">
         <f t="shared" si="2"/>
         <v>45212.708333333328</v>
       </c>
-      <c r="M34" s="48">
+      <c r="M34" s="46">
         <v>38.856884999999998</v>
       </c>
-      <c r="N34" s="48">
+      <c r="N34" s="46">
         <v>-63.746738999999998</v>
       </c>
-      <c r="O34" s="48">
+      <c r="O34" s="46">
         <v>1</v>
       </c>
-      <c r="P34" s="48" t="s">
+      <c r="P34" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q34" s="51">
+      <c r="Q34" s="49">
         <v>300434066489180</v>
       </c>
-      <c r="R34" s="51" t="s">
+      <c r="R34" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="S34" s="56">
+      <c r="S34" s="54">
         <v>45211.834328703706</v>
       </c>
-      <c r="T34" s="60">
+      <c r="T34" s="58">
         <v>38.831561999999998</v>
       </c>
-      <c r="U34" s="60">
+      <c r="U34" s="58">
         <v>-63.740231999999999</v>
       </c>
-      <c r="V34" s="61">
+      <c r="V34" s="59">
         <v>45212.541990740741</v>
       </c>
-      <c r="W34" s="60">
+      <c r="W34" s="58">
         <v>38.884850999999998</v>
       </c>
-      <c r="X34" s="60">
+      <c r="X34" s="58">
         <v>-63.740850999999999</v>
       </c>
-      <c r="Y34" s="53">
+      <c r="Y34" s="51">
         <f t="shared" si="0"/>
         <v>16.983888888848014</v>
       </c>
-      <c r="Z34" s="54">
+      <c r="Z34" s="52">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA34" s="54">
+      <c r="AA34" s="52">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB34" s="48">
+      <c r="AB34" s="46">
         <v>125</v>
       </c>
-      <c r="AC34" s="48">
+      <c r="AC34" s="46">
         <v>4</v>
       </c>
-      <c r="AD34" s="48" t="s">
+      <c r="AD34" s="46" t="s">
         <v>52</v>
       </c>
     </row>
@@ -4722,7 +4781,7 @@
       <c r="U35" s="32">
         <v>-63.738950000000003</v>
       </c>
-      <c r="V35" s="34">
+      <c r="V35" s="33">
         <v>45212.535046296296</v>
       </c>
       <c r="W35" s="32">
@@ -4751,252 +4810,252 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="48">
+    <row r="36" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="46">
         <v>23</v>
       </c>
-      <c r="B36" s="48" t="s">
+      <c r="B36" s="46" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="48">
+      <c r="C36" s="46">
         <v>5</v>
       </c>
-      <c r="D36" s="48">
+      <c r="D36" s="46">
         <v>1</v>
       </c>
-      <c r="E36" s="49">
+      <c r="E36" s="47">
         <v>45317</v>
       </c>
-      <c r="F36" s="50">
+      <c r="F36" s="48">
         <v>0.50972222222222219</v>
       </c>
-      <c r="G36" s="43">
+      <c r="G36" s="41">
         <f t="shared" si="1"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H36" s="48"/>
-      <c r="I36" s="48"/>
-      <c r="J36" s="49">
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="47">
         <v>45320</v>
       </c>
-      <c r="K36" s="50">
+      <c r="K36" s="48">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L36" s="58">
+      <c r="L36" s="56">
         <f t="shared" si="2"/>
         <v>45320.90625</v>
       </c>
-      <c r="M36" s="48"/>
-      <c r="N36" s="48"/>
-      <c r="O36" s="48">
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46">
         <v>3</v>
       </c>
-      <c r="P36" s="48" t="s">
+      <c r="P36" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q36" s="51"/>
-      <c r="R36" s="51" t="s">
+      <c r="Q36" s="49"/>
+      <c r="R36" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S36" s="52">
+      <c r="S36" s="50">
         <v>45317.875324074077</v>
       </c>
-      <c r="T36" s="62">
+      <c r="T36" s="72">
         <v>32.909129</v>
       </c>
-      <c r="U36" s="62">
+      <c r="U36" s="72">
         <v>-117.680663</v>
       </c>
-      <c r="V36" s="52">
+      <c r="V36" s="50">
         <v>45318.878796296296</v>
       </c>
-      <c r="W36" s="48">
+      <c r="W36" s="46">
         <v>32.999972</v>
       </c>
-      <c r="X36" s="48">
+      <c r="X36" s="46">
         <v>-117.66408699999999</v>
       </c>
-      <c r="Y36" s="53">
+      <c r="Y36" s="51">
         <f t="shared" si="0"/>
         <v>24.083333333255723</v>
       </c>
-      <c r="Z36" s="54">
+      <c r="Z36" s="52">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA36" s="54">
+      <c r="AA36" s="52">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB36" s="48"/>
-      <c r="AC36" s="48">
+      <c r="AB36" s="46"/>
+      <c r="AC36" s="46">
         <v>8</v>
       </c>
-      <c r="AD36" s="48" t="s">
+      <c r="AD36" s="46" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="48">
+    <row r="37" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="46">
         <v>23</v>
       </c>
-      <c r="B37" s="48" t="s">
+      <c r="B37" s="46" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="48">
+      <c r="C37" s="46">
         <v>5</v>
       </c>
-      <c r="D37" s="48">
+      <c r="D37" s="46">
         <v>2</v>
       </c>
-      <c r="E37" s="49">
+      <c r="E37" s="47">
         <v>45317</v>
       </c>
-      <c r="F37" s="50">
+      <c r="F37" s="48">
         <v>0.50972222222222219</v>
       </c>
-      <c r="G37" s="43">
+      <c r="G37" s="41">
         <f t="shared" si="1"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
-      <c r="J37" s="49">
+      <c r="H37" s="46"/>
+      <c r="I37" s="46"/>
+      <c r="J37" s="47">
         <v>45320</v>
       </c>
-      <c r="K37" s="50">
+      <c r="K37" s="48">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L37" s="58">
+      <c r="L37" s="56">
         <f t="shared" si="2"/>
         <v>45320.90625</v>
       </c>
-      <c r="M37" s="48"/>
-      <c r="N37" s="48"/>
-      <c r="O37" s="48">
+      <c r="M37" s="46"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="46">
         <v>3</v>
       </c>
-      <c r="P37" s="48" t="s">
+      <c r="P37" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q37" s="51"/>
-      <c r="R37" s="51" t="s">
+      <c r="Q37" s="49"/>
+      <c r="R37" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S37" s="52">
+      <c r="S37" s="50">
         <v>45318.931122685186</v>
       </c>
-      <c r="T37" s="62">
+      <c r="T37" s="72">
         <v>33.001423000000003</v>
       </c>
-      <c r="U37" s="62">
+      <c r="U37" s="72">
         <v>-117.65347800000001</v>
       </c>
-      <c r="V37" s="52">
+      <c r="V37" s="50">
         <v>45319.878796296296</v>
       </c>
-      <c r="W37" s="48">
+      <c r="W37" s="46">
         <v>33.117448000000003</v>
       </c>
-      <c r="X37" s="48">
+      <c r="X37" s="46">
         <v>-117.6035</v>
       </c>
-      <c r="Y37" s="53">
+      <c r="Y37" s="51">
         <f t="shared" si="0"/>
         <v>22.744166666641831</v>
       </c>
-      <c r="Z37" s="54">
+      <c r="Z37" s="52">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA37" s="54">
+      <c r="AA37" s="52">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB37" s="48"/>
-      <c r="AC37" s="48">
+      <c r="AB37" s="46"/>
+      <c r="AC37" s="46">
         <v>8</v>
       </c>
-      <c r="AD37" s="48" t="s">
+      <c r="AD37" s="46" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="48">
+    <row r="38" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="46">
         <v>23</v>
       </c>
-      <c r="B38" s="48" t="s">
+      <c r="B38" s="46" t="s">
         <v>96</v>
       </c>
-      <c r="C38" s="48">
+      <c r="C38" s="46">
         <v>5</v>
       </c>
-      <c r="D38" s="48">
+      <c r="D38" s="46">
         <v>3</v>
       </c>
-      <c r="E38" s="49">
+      <c r="E38" s="47">
         <v>45317</v>
       </c>
-      <c r="F38" s="50">
+      <c r="F38" s="48">
         <v>0.50972222222222219</v>
       </c>
-      <c r="G38" s="43">
+      <c r="G38" s="41">
         <f t="shared" si="1"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H38" s="48"/>
-      <c r="I38" s="48"/>
-      <c r="J38" s="49">
+      <c r="H38" s="46"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="47">
         <v>45320</v>
       </c>
-      <c r="K38" s="50">
+      <c r="K38" s="48">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L38" s="58">
+      <c r="L38" s="56">
         <f t="shared" si="2"/>
         <v>45320.90625</v>
       </c>
-      <c r="M38" s="48"/>
-      <c r="N38" s="48"/>
-      <c r="O38" s="48">
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46">
         <v>3</v>
       </c>
-      <c r="P38" s="48" t="s">
+      <c r="P38" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q38" s="51"/>
-      <c r="R38" s="51" t="s">
+      <c r="Q38" s="49"/>
+      <c r="R38" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="S38" s="52">
+      <c r="S38" s="50">
         <v>45319.910034722219</v>
       </c>
-      <c r="T38" s="63">
+      <c r="T38" s="73">
         <v>33.123451000000003</v>
       </c>
-      <c r="U38" s="63">
+      <c r="U38" s="73">
         <v>-117.600043</v>
       </c>
-      <c r="V38" s="52">
+      <c r="V38" s="50">
         <v>45320.89980324074</v>
       </c>
-      <c r="W38" s="63">
+      <c r="W38" s="73">
         <v>33.200189999999999</v>
       </c>
-      <c r="X38" s="63">
+      <c r="X38" s="73">
         <v>-117.597759</v>
       </c>
-      <c r="Y38" s="53">
+      <c r="Y38" s="51">
         <f t="shared" ref="Y38" si="3">(V38-S38)*1440/60</f>
         <v>23.754444444493856</v>
       </c>
-      <c r="Z38" s="54">
+      <c r="Z38" s="52">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA38" s="54">
+      <c r="AA38" s="52">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB38" s="48"/>
-      <c r="AC38" s="48">
+      <c r="AB38" s="46"/>
+      <c r="AC38" s="46">
         <v>8</v>
       </c>
-      <c r="AD38" s="48" t="s">
+      <c r="AD38" s="46" t="s">
         <v>97</v>
       </c>
     </row>
@@ -5050,19 +5109,19 @@
       <c r="S39" s="28">
         <v>45317.993379629632</v>
       </c>
-      <c r="T39" s="35">
+      <c r="T39" s="74">
         <v>32.907333000000001</v>
       </c>
-      <c r="U39" s="35">
+      <c r="U39" s="74">
         <v>-117.67442</v>
       </c>
       <c r="V39" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="W39" s="35">
+      <c r="W39" s="74">
         <v>33.012383</v>
       </c>
-      <c r="X39" s="35">
+      <c r="X39" s="74">
         <v>-117.66186500000001</v>
       </c>
       <c r="Y39" s="25">
@@ -5133,19 +5192,19 @@
       <c r="S40" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="T40" s="35">
+      <c r="T40" s="74">
         <v>33.012383</v>
       </c>
-      <c r="U40" s="35">
+      <c r="U40" s="74">
         <v>-117.66186500000001</v>
       </c>
       <c r="V40" s="28">
         <v>45320.848263888889</v>
       </c>
-      <c r="W40" s="35">
+      <c r="W40" s="74">
         <v>33.115271</v>
       </c>
-      <c r="X40" s="35">
+      <c r="X40" s="74">
         <v>-117.89773700000001</v>
       </c>
       <c r="Y40" s="25">
@@ -5166,317 +5225,459 @@
         <v>98</v>
       </c>
     </row>
-    <row r="41" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="20">
+    <row r="41" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="46">
         <v>25</v>
       </c>
-      <c r="B41" s="48" t="s">
+      <c r="B41" s="46" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="20">
+      <c r="C41" s="46">
         <v>5</v>
       </c>
-      <c r="D41" s="20">
+      <c r="D41" s="46">
         <v>1</v>
       </c>
-      <c r="E41" s="21">
+      <c r="E41" s="47">
+        <v>45425</v>
+      </c>
+      <c r="F41" s="48"/>
+      <c r="G41" s="41" t="s">
+        <v>125</v>
+      </c>
+      <c r="H41" s="46"/>
+      <c r="I41" s="46"/>
+      <c r="J41" s="47"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="56" t="s">
+        <v>126</v>
+      </c>
+      <c r="M41" s="46"/>
+      <c r="N41" s="46"/>
+      <c r="O41" s="46">
+        <v>3</v>
+      </c>
+      <c r="P41" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q41" s="49">
+        <v>300434066482170</v>
+      </c>
+      <c r="R41" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="S41" s="54"/>
+      <c r="T41" s="73"/>
+      <c r="U41" s="73"/>
+      <c r="V41" s="54"/>
+      <c r="W41" s="73"/>
+      <c r="X41" s="73"/>
+      <c r="Y41" s="51"/>
+      <c r="Z41" s="52"/>
+      <c r="AA41" s="52"/>
+      <c r="AB41" s="46"/>
+      <c r="AC41" s="46"/>
+      <c r="AD41" s="46"/>
+    </row>
+    <row r="42" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="70">
+        <v>26</v>
+      </c>
+      <c r="B42" s="70" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="70">
+        <v>5</v>
+      </c>
+      <c r="D42" s="70">
+        <v>1</v>
+      </c>
+      <c r="E42" s="80">
         <v>45429</v>
       </c>
-      <c r="F41" s="22">
+      <c r="F42" s="81">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G41" s="22" t="s">
+      <c r="G42" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="H41" s="20"/>
-      <c r="I41" s="20"/>
-      <c r="J41" s="21">
+      <c r="H42" s="70"/>
+      <c r="I42" s="70"/>
+      <c r="J42" s="80">
         <v>45432</v>
       </c>
-      <c r="K41" s="22">
+      <c r="K42" s="81">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L41" s="22" t="s">
+      <c r="L42" s="81" t="s">
         <v>117</v>
       </c>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20"/>
-      <c r="O41" s="20">
+      <c r="M42" s="70"/>
+      <c r="N42" s="70"/>
+      <c r="O42" s="70">
         <v>3</v>
       </c>
-      <c r="P41" s="20" t="s">
+      <c r="P42" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="Q41" s="23"/>
-      <c r="R41" s="23" t="s">
+      <c r="Q42" s="69">
+        <v>300434066482170</v>
+      </c>
+      <c r="R42" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="S41" s="68" t="s">
+      <c r="S42" s="88" t="s">
         <v>119</v>
       </c>
-      <c r="T41" s="69">
+      <c r="T42" s="89">
         <v>32.917650000000002</v>
       </c>
-      <c r="U41" s="69">
+      <c r="U42" s="89">
         <v>-117.794504</v>
       </c>
-      <c r="V41" s="28" t="s">
+      <c r="V42" s="83" t="s">
         <v>118</v>
       </c>
-      <c r="W41" s="69" t="s">
+      <c r="W42" s="89" t="s">
         <v>120</v>
       </c>
-      <c r="X41" s="69" t="s">
+      <c r="X42" s="89" t="s">
         <v>121</v>
       </c>
-      <c r="Y41" s="25"/>
-      <c r="Z41" s="26">
+      <c r="Y42" s="85"/>
+      <c r="Z42" s="86">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA41" s="26">
+      <c r="AA42" s="86">
         <v>0.1125</v>
       </c>
-      <c r="AB41" s="20"/>
-      <c r="AC41" s="20">
+      <c r="AB42" s="70"/>
+      <c r="AC42" s="70">
         <v>7</v>
       </c>
-      <c r="AD41" s="20"/>
-    </row>
-    <row r="42" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="20">
-        <v>25</v>
-      </c>
-      <c r="B42" s="48" t="s">
+      <c r="AD42" s="70"/>
+    </row>
+    <row r="43" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="70">
+        <v>26</v>
+      </c>
+      <c r="B43" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="20">
+      <c r="C43" s="70">
         <v>5</v>
       </c>
-      <c r="D42" s="20">
+      <c r="D43" s="70">
         <v>2</v>
       </c>
-      <c r="E42" s="21">
+      <c r="E43" s="80">
         <v>45429</v>
       </c>
-      <c r="F42" s="22">
+      <c r="F43" s="81">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G42" s="22" t="s">
+      <c r="G43" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="21">
+      <c r="H43" s="70"/>
+      <c r="I43" s="70"/>
+      <c r="J43" s="80">
         <v>45432</v>
       </c>
-      <c r="K42" s="22">
+      <c r="K43" s="81">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L42" s="22" t="s">
+      <c r="L43" s="81" t="s">
         <v>117</v>
       </c>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="20">
+      <c r="M43" s="70"/>
+      <c r="N43" s="70"/>
+      <c r="O43" s="70">
         <v>3</v>
       </c>
-      <c r="P42" s="20" t="s">
+      <c r="P43" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="Q42" s="23"/>
-      <c r="R42" s="23" t="s">
+      <c r="Q43" s="69">
+        <v>300434066482170</v>
+      </c>
+      <c r="R43" s="69" t="s">
         <v>115</v>
       </c>
-      <c r="S42" s="24" t="s">
+      <c r="S43" s="84" t="s">
         <v>122</v>
       </c>
-      <c r="T42" s="69">
+      <c r="T43" s="89">
         <v>32.998700999999997</v>
       </c>
-      <c r="U42" s="69">
+      <c r="U43" s="89">
         <v>-117.874388</v>
       </c>
-      <c r="V42" s="24" t="s">
+      <c r="V43" s="84" t="s">
         <v>123</v>
       </c>
-      <c r="W42" s="69">
+      <c r="W43" s="89">
         <v>33.012540000000001</v>
       </c>
-      <c r="X42" s="20">
+      <c r="X43" s="70">
         <v>-117.890097</v>
       </c>
-      <c r="Y42" s="25"/>
-      <c r="Z42" s="26">
+      <c r="Y43" s="85"/>
+      <c r="Z43" s="86">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA42" s="26">
+      <c r="AA43" s="86">
         <v>0.1125</v>
       </c>
-      <c r="AB42" s="20"/>
-      <c r="AC42" s="20">
+      <c r="AB43" s="70"/>
+      <c r="AC43" s="70">
         <v>7</v>
       </c>
-      <c r="AD42" s="20"/>
-    </row>
-    <row r="43" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="20"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="21"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="20"/>
-      <c r="J43" s="21"/>
-      <c r="K43" s="22"/>
-      <c r="L43" s="22"/>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
-      <c r="O43" s="20"/>
-      <c r="P43" s="20"/>
-      <c r="Q43" s="23"/>
-      <c r="R43" s="23"/>
-      <c r="S43" s="24"/>
-      <c r="T43" s="20"/>
-      <c r="U43" s="20"/>
-      <c r="V43" s="24"/>
-      <c r="W43" s="20"/>
-      <c r="X43" s="20"/>
-      <c r="Y43" s="25"/>
-      <c r="Z43" s="26"/>
-      <c r="AA43" s="26"/>
-      <c r="AB43" s="20"/>
-      <c r="AC43" s="20"/>
-      <c r="AD43" s="20"/>
-    </row>
-    <row r="44" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="20"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="21"/>
-      <c r="K44" s="22"/>
-      <c r="L44" s="22"/>
-      <c r="M44" s="20"/>
-      <c r="N44" s="20"/>
-      <c r="O44" s="20"/>
-      <c r="P44" s="20"/>
-      <c r="Q44" s="23"/>
-      <c r="R44" s="23"/>
-      <c r="S44" s="24"/>
-      <c r="T44" s="20"/>
-      <c r="U44" s="20"/>
-      <c r="V44" s="24"/>
-      <c r="W44" s="20"/>
-      <c r="X44" s="20"/>
-      <c r="Y44" s="25"/>
-      <c r="Z44" s="26"/>
-      <c r="AA44" s="26"/>
-      <c r="AB44" s="20"/>
-      <c r="AC44" s="20"/>
-      <c r="AD44" s="20"/>
-    </row>
-    <row r="45" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="20"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="20"/>
-      <c r="I45" s="20"/>
-      <c r="J45" s="21"/>
-      <c r="K45" s="22"/>
-      <c r="L45" s="22"/>
-      <c r="M45" s="20"/>
-      <c r="N45" s="20"/>
-      <c r="O45" s="20"/>
-      <c r="P45" s="20"/>
-      <c r="Q45" s="23"/>
-      <c r="R45" s="23"/>
-      <c r="S45" s="24"/>
-      <c r="T45" s="20"/>
-      <c r="U45" s="20"/>
-      <c r="V45" s="24"/>
-      <c r="W45" s="20"/>
-      <c r="X45" s="20"/>
-      <c r="Y45" s="25"/>
-      <c r="Z45" s="26"/>
-      <c r="AA45" s="26"/>
-      <c r="AB45" s="20"/>
-      <c r="AC45" s="20"/>
-      <c r="AD45" s="20"/>
-    </row>
-    <row r="46" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="20"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="20"/>
-      <c r="I46" s="20"/>
-      <c r="J46" s="21"/>
-      <c r="K46" s="22"/>
-      <c r="L46" s="22"/>
-      <c r="M46" s="20"/>
-      <c r="N46" s="20"/>
-      <c r="O46" s="20"/>
-      <c r="P46" s="20"/>
-      <c r="Q46" s="23"/>
-      <c r="R46" s="23"/>
-      <c r="S46" s="24"/>
-      <c r="T46" s="20"/>
-      <c r="U46" s="20"/>
-      <c r="V46" s="24"/>
-      <c r="W46" s="20"/>
-      <c r="X46" s="20"/>
-      <c r="Y46" s="25"/>
-      <c r="Z46" s="26"/>
-      <c r="AA46" s="26"/>
-      <c r="AB46" s="20"/>
-      <c r="AC46" s="20"/>
-      <c r="AD46" s="20"/>
-    </row>
-    <row r="47" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="68"/>
-      <c r="F47" s="69"/>
-      <c r="G47" s="69"/>
-      <c r="H47" s="28"/>
-      <c r="I47" s="69"/>
-      <c r="J47" s="69"/>
-      <c r="K47" s="22"/>
-      <c r="L47" s="22"/>
-      <c r="M47" s="20"/>
-      <c r="N47" s="20"/>
-      <c r="O47" s="20"/>
-      <c r="P47" s="20"/>
-      <c r="Q47" s="23"/>
-      <c r="R47" s="23"/>
-      <c r="S47" s="24"/>
-      <c r="T47" s="20"/>
-      <c r="U47" s="20"/>
-      <c r="V47" s="24"/>
-      <c r="W47" s="20"/>
-      <c r="X47" s="20"/>
-      <c r="Y47" s="25"/>
-      <c r="Z47" s="26"/>
-      <c r="AA47" s="26"/>
-      <c r="AB47" s="20"/>
-      <c r="AC47" s="20"/>
-      <c r="AD47" s="20"/>
+      <c r="AD43" s="70"/>
+    </row>
+    <row r="44" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="46">
+        <v>27</v>
+      </c>
+      <c r="B44" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="C44" s="46">
+        <v>5</v>
+      </c>
+      <c r="D44" s="46">
+        <v>1</v>
+      </c>
+      <c r="E44" s="75">
+        <v>45462</v>
+      </c>
+      <c r="F44" s="76">
+        <v>0.625</v>
+      </c>
+      <c r="G44" s="41">
+        <f>$E44+$F44+TIME(AC44,0,0)</f>
+        <v>45462.791666666664</v>
+      </c>
+      <c r="H44" s="46"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="47"/>
+      <c r="K44" s="48"/>
+      <c r="M44" s="73"/>
+      <c r="N44" s="73"/>
+      <c r="O44" s="46">
+        <v>3</v>
+      </c>
+      <c r="P44" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q44" s="49">
+        <v>300434066482170</v>
+      </c>
+      <c r="R44" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="S44" s="54">
+        <v>45462.860289351855</v>
+      </c>
+      <c r="T44" s="73">
+        <v>38.313133999999998</v>
+      </c>
+      <c r="U44" s="73">
+        <v>-63.006925000000003</v>
+      </c>
+      <c r="V44" s="50"/>
+      <c r="W44" s="46"/>
+      <c r="X44" s="46"/>
+      <c r="Y44" s="51"/>
+      <c r="Z44" s="52"/>
+      <c r="AA44" s="52"/>
+      <c r="AB44" s="46"/>
+      <c r="AC44" s="46">
+        <v>4</v>
+      </c>
+      <c r="AD44" s="46"/>
+    </row>
+    <row r="45" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="70">
+        <v>28</v>
+      </c>
+      <c r="B45" s="70" t="s">
+        <v>124</v>
+      </c>
+      <c r="C45" s="70">
+        <v>6</v>
+      </c>
+      <c r="D45" s="70">
+        <v>1</v>
+      </c>
+      <c r="E45" s="78">
+        <v>45462</v>
+      </c>
+      <c r="F45" s="79">
+        <v>0.625</v>
+      </c>
+      <c r="G45" s="67">
+        <f t="shared" ref="G45:G46" si="6">$E45+$F45+TIME(AC45,0,0)</f>
+        <v>45462.791666666664</v>
+      </c>
+      <c r="H45" s="70"/>
+      <c r="I45" s="70"/>
+      <c r="J45" s="80"/>
+      <c r="K45" s="81"/>
+      <c r="L45" s="68"/>
+      <c r="M45" s="82"/>
+      <c r="N45" s="82"/>
+      <c r="O45" s="70">
+        <v>4</v>
+      </c>
+      <c r="P45" s="70" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q45" s="69">
+        <v>300434066480130</v>
+      </c>
+      <c r="R45" s="69" t="s">
+        <v>44</v>
+      </c>
+      <c r="S45" s="83">
+        <v>45462.855231481481</v>
+      </c>
+      <c r="T45" s="82">
+        <v>38.307771000000002</v>
+      </c>
+      <c r="U45" s="82">
+        <v>-62.998032000000002</v>
+      </c>
+      <c r="V45" s="84"/>
+      <c r="W45" s="70"/>
+      <c r="X45" s="70"/>
+      <c r="Y45" s="85"/>
+      <c r="Z45" s="86"/>
+      <c r="AA45" s="86"/>
+      <c r="AB45" s="70"/>
+      <c r="AC45" s="70">
+        <v>4</v>
+      </c>
+      <c r="AD45" s="70"/>
+    </row>
+    <row r="46" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="46">
+        <v>29</v>
+      </c>
+      <c r="B46" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="C46" s="46">
+        <v>4</v>
+      </c>
+      <c r="D46" s="46">
+        <v>1</v>
+      </c>
+      <c r="E46" s="75">
+        <v>45462</v>
+      </c>
+      <c r="F46" s="76">
+        <v>0.625</v>
+      </c>
+      <c r="G46" s="41">
+        <f>$E46+$F46+TIME(AC46,0,0)</f>
+        <v>45462.791666666664</v>
+      </c>
+      <c r="H46" s="46">
+        <v>38.316051999999999</v>
+      </c>
+      <c r="I46" s="46">
+        <v>-63.012607000000003</v>
+      </c>
+      <c r="J46" s="47">
+        <v>45464</v>
+      </c>
+      <c r="K46" s="48">
+        <v>0.125</v>
+      </c>
+      <c r="L46" s="56">
+        <f t="shared" ref="L46" si="7">$J46+$K46 +TIME($AC46,0,0)</f>
+        <v>45464.291666666664</v>
+      </c>
+      <c r="M46" s="73">
+        <v>38.309516000000002</v>
+      </c>
+      <c r="N46" s="73">
+        <v>-62.619463000000003</v>
+      </c>
+      <c r="O46" s="46">
+        <v>1</v>
+      </c>
+      <c r="P46" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q46" s="77">
+        <v>300434066489180</v>
+      </c>
+      <c r="R46" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="S46" s="54">
+        <v>45462.84778935185</v>
+      </c>
+      <c r="T46" s="73">
+        <v>38.315800000000003</v>
+      </c>
+      <c r="U46" s="73">
+        <v>-63.012493999999997</v>
+      </c>
+      <c r="V46" s="54">
+        <v>45463.528101851851</v>
+      </c>
+      <c r="W46" s="73">
+        <v>38.311391</v>
+      </c>
+      <c r="X46" s="73">
+        <v>-62.918548000000001</v>
+      </c>
+      <c r="Y46" s="51">
+        <f t="shared" ref="Y46" si="8">(V46-S46)*1440/60</f>
+        <v>16.32750000001397</v>
+      </c>
+      <c r="Z46" s="52"/>
+      <c r="AA46" s="52"/>
+      <c r="AB46" s="46"/>
+      <c r="AC46" s="46">
+        <v>4</v>
+      </c>
+      <c r="AD46" s="46"/>
+    </row>
+    <row r="47" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="70"/>
+      <c r="B47" s="70"/>
+      <c r="C47" s="70"/>
+      <c r="D47" s="70"/>
+      <c r="E47" s="88"/>
+      <c r="F47" s="89"/>
+      <c r="G47" s="89"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="89"/>
+      <c r="J47" s="90"/>
+      <c r="K47" s="81"/>
+      <c r="L47" s="81"/>
+      <c r="M47" s="70"/>
+      <c r="N47" s="70"/>
+      <c r="O47" s="70"/>
+      <c r="P47" s="70"/>
+      <c r="Q47" s="69"/>
+      <c r="R47" s="69"/>
+      <c r="S47" s="84"/>
+      <c r="T47" s="70"/>
+      <c r="U47" s="70"/>
+      <c r="V47" s="84"/>
+      <c r="W47" s="70"/>
+      <c r="X47" s="70"/>
+      <c r="Y47" s="85"/>
+      <c r="Z47" s="86"/>
+      <c r="AA47" s="86"/>
+      <c r="AB47" s="70"/>
+      <c r="AC47" s="70"/>
+      <c r="AD47" s="70"/>
     </row>
     <row r="48" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="20"/>
@@ -5484,10 +5685,10 @@
       <c r="C48" s="20"/>
       <c r="D48" s="20"/>
       <c r="E48" s="24"/>
-      <c r="F48" s="69"/>
-      <c r="G48" s="69"/>
+      <c r="F48" s="71"/>
+      <c r="G48" s="71"/>
       <c r="H48" s="24"/>
-      <c r="I48" s="69"/>
+      <c r="I48" s="64"/>
       <c r="J48" s="20"/>
       <c r="K48" s="22"/>
       <c r="L48" s="22"/>
@@ -36151,7 +36352,7 @@
     <col min="3" max="3" width="11.33203125" style="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5" style="27" customWidth="1"/>
     <col min="5" max="5" width="20" style="27" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.83203125" style="37" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.83203125" style="35" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" style="27" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="134" style="27" customWidth="1"/>
     <col min="9" max="16384" width="14.5" style="27"/>
@@ -36209,101 +36410,101 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="48">
+    <row r="3" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="46">
         <v>2</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="48">
+      <c r="C3" s="46">
         <v>4</v>
       </c>
-      <c r="D3" s="48">
+      <c r="D3" s="46">
         <v>1</v>
       </c>
-      <c r="E3" s="49">
+      <c r="E3" s="47">
         <v>44983</v>
       </c>
-      <c r="F3" s="53">
+      <c r="F3" s="51">
         <v>12.250277777784504</v>
       </c>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="48"/>
-    </row>
-    <row r="4" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="48">
+      <c r="H3" s="46"/>
+    </row>
+    <row r="4" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="46">
         <v>2</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="48">
+      <c r="C4" s="46">
         <v>4</v>
       </c>
-      <c r="D4" s="48">
+      <c r="D4" s="46">
         <v>2</v>
       </c>
-      <c r="E4" s="49">
+      <c r="E4" s="47">
         <v>44983</v>
       </c>
-      <c r="F4" s="53">
+      <c r="F4" s="51">
         <v>11.499999999941792</v>
       </c>
-      <c r="G4" s="48" t="s">
+      <c r="G4" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="48"/>
-    </row>
-    <row r="5" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="48">
+      <c r="H4" s="46"/>
+    </row>
+    <row r="5" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="46">
         <v>2</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="48">
+      <c r="C5" s="46">
         <v>4</v>
       </c>
-      <c r="D5" s="48">
+      <c r="D5" s="46">
         <v>3</v>
       </c>
-      <c r="E5" s="49">
+      <c r="E5" s="47">
         <v>44983</v>
       </c>
-      <c r="F5" s="53">
+      <c r="F5" s="51">
         <v>12.083333333430346</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="48"/>
-    </row>
-    <row r="6" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="48">
+      <c r="H5" s="46"/>
+    </row>
+    <row r="6" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="46">
         <v>2</v>
       </c>
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="46">
         <v>4</v>
       </c>
-      <c r="D6" s="48">
+      <c r="D6" s="46">
         <v>4</v>
       </c>
-      <c r="E6" s="49">
+      <c r="E6" s="47">
         <v>44983</v>
       </c>
-      <c r="F6" s="53">
+      <c r="F6" s="51">
         <v>11.583055555529427</v>
       </c>
-      <c r="G6" s="48" t="s">
+      <c r="G6" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="48"/>
+      <c r="H6" s="46"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="20">
@@ -36353,29 +36554,29 @@
       </c>
       <c r="H8" s="20"/>
     </row>
-    <row r="9" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="48">
+    <row r="9" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="46">
         <v>4</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="48">
+      <c r="C9" s="46">
         <v>6</v>
       </c>
-      <c r="D9" s="48">
+      <c r="D9" s="46">
         <v>1</v>
       </c>
-      <c r="E9" s="49">
+      <c r="E9" s="47">
         <v>44985</v>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="51">
         <v>1.7480555555666797</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="46" t="s">
         <v>31</v>
       </c>
     </row>
@@ -36405,53 +36606,53 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="48">
+    <row r="11" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="46">
         <v>6</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="46">
         <v>4</v>
       </c>
-      <c r="D11" s="48">
+      <c r="D11" s="46">
         <v>1</v>
       </c>
-      <c r="E11" s="49">
+      <c r="E11" s="47">
         <v>45084</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="51">
         <v>12.746666666760575</v>
       </c>
-      <c r="G11" s="48" t="s">
+      <c r="G11" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="48"/>
-    </row>
-    <row r="12" spans="1:8" s="55" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="48">
+      <c r="H11" s="46"/>
+    </row>
+    <row r="12" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="46">
         <v>7</v>
       </c>
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="C12" s="48">
+      <c r="C12" s="46">
         <v>4</v>
       </c>
-      <c r="D12" s="48">
+      <c r="D12" s="46">
         <v>2</v>
       </c>
-      <c r="E12" s="49">
+      <c r="E12" s="47">
         <v>45084</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="51">
         <v>11.666944444470573</v>
       </c>
-      <c r="G12" s="48" t="s">
+      <c r="G12" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="48"/>
+      <c r="H12" s="46"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="20">
@@ -36501,29 +36702,29 @@
       </c>
       <c r="H14" s="20"/>
     </row>
-    <row r="15" spans="1:8" s="59" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="48">
+    <row r="15" spans="1:8" s="57" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="46">
         <v>10</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="48">
+      <c r="C15" s="46">
         <v>6</v>
       </c>
-      <c r="D15" s="48">
+      <c r="D15" s="46">
         <v>1</v>
       </c>
-      <c r="E15" s="49">
+      <c r="E15" s="47">
         <v>45176</v>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="51">
         <v>88.993611111072823</v>
       </c>
-      <c r="G15" s="48" t="s">
+      <c r="G15" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="48"/>
+      <c r="H15" s="46"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="20">
@@ -36603,55 +36804,55 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="64">
+    <row r="19" spans="1:8" s="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="60">
         <v>12</v>
       </c>
-      <c r="B19" s="64" t="s">
+      <c r="B19" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="64">
+      <c r="C19" s="60">
         <v>6</v>
       </c>
-      <c r="D19" s="64">
+      <c r="D19" s="60">
         <v>1</v>
       </c>
-      <c r="E19" s="65">
+      <c r="E19" s="61">
         <v>45317</v>
       </c>
-      <c r="F19" s="66">
+      <c r="F19" s="62">
         <v>21.333611111040227</v>
       </c>
-      <c r="G19" s="64" t="s">
+      <c r="G19" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="H19" s="64" t="s">
+      <c r="H19" s="60" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="64">
+    <row r="20" spans="1:8" s="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="60">
         <v>12</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="B20" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="64">
+      <c r="C20" s="60">
         <v>6</v>
       </c>
-      <c r="D20" s="64">
+      <c r="D20" s="60">
         <v>1</v>
       </c>
-      <c r="E20" s="65">
+      <c r="E20" s="61">
         <v>45317</v>
       </c>
-      <c r="F20" s="66">
+      <c r="F20" s="62">
         <v>47.183611111133359</v>
       </c>
-      <c r="G20" s="64" t="s">
+      <c r="G20" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="64" t="s">
+      <c r="H20" s="60" t="s">
         <v>98</v>
       </c>
     </row>
@@ -36680,7 +36881,7 @@
       <c r="B23" s="20"/>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
-      <c r="E23" s="36"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="25"/>
       <c r="G23" s="20"/>
       <c r="H23" s="20"/>
@@ -46343,11 +46544,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
update iridium scraper to automatically pick correct folder based on date, add new drifter 6 dives to the deployment log
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49037BF2-BDF3-DC4B-8838-214863E3BF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438AC3A6-A7DD-2E4E-90E3-0292286EAAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="960" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="136">
   <si>
     <t>Deployment</t>
   </si>
@@ -424,6 +424,33 @@
   <si>
     <t>20240513T211836</t>
   </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>20220918T030844</t>
+  </si>
+  <si>
+    <t>20220918T123442</t>
+  </si>
+  <si>
+    <t>20220918T194307</t>
+  </si>
+  <si>
+    <t>20220919T141500</t>
+  </si>
+  <si>
+    <t>20220919T193132</t>
+  </si>
+  <si>
+    <t>20220920T132834</t>
+  </si>
+  <si>
+    <t>Was supposed to dive a third time, but stayed at surface</t>
+  </si>
+  <si>
+    <t>Dove in wrong direction after waking up from hibernation, dove to 950m and dropped weight</t>
+  </si>
 </sst>
 </file>
 
@@ -437,11 +464,18 @@
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
     <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -591,97 +625,97 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="9" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="10" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -690,148 +724,158 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="168" fontId="2" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="22" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="168" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1780,7 +1824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD1005"/>
+  <dimension ref="A1:AD1006"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="27" customWidth="1"/>
@@ -1793,10 +1837,10 @@
     <col min="9" max="9" width="10.83203125" style="27" customWidth="1"/>
     <col min="10" max="10" width="17.5" style="27" customWidth="1"/>
     <col min="11" max="11" width="17.83203125" style="27" customWidth="1"/>
-    <col min="12" max="12" width="20" style="27" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20" style="27" customWidth="1"/>
     <col min="13" max="13" width="12.1640625" style="27" customWidth="1"/>
     <col min="14" max="16" width="13.5" style="27" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.83203125" style="27" customWidth="1"/>
     <col min="18" max="18" width="48" style="27" customWidth="1"/>
     <col min="19" max="19" width="18.83203125" style="27" customWidth="1"/>
     <col min="20" max="21" width="10.83203125" style="27" customWidth="1"/>
@@ -1921,7 +1965,10 @@
       <c r="F2" s="40">
         <v>0.55138888888888882</v>
       </c>
-      <c r="G2" s="41"/>
+      <c r="G2" s="41">
+        <f t="shared" ref="G2:G3" si="0">$E2+$F2+TIME(AC2,0,0)</f>
+        <v>44818.551388888889</v>
+      </c>
       <c r="H2" s="37">
         <v>39.865239000000003</v>
       </c>
@@ -1934,7 +1981,10 @@
       <c r="K2" s="40">
         <v>0.66666666666666663</v>
       </c>
-      <c r="L2" s="40"/>
+      <c r="L2" s="41">
+        <f t="shared" ref="L2:L3" si="1">$J2+$K2 +TIME($AC2,0,0)</f>
+        <v>44818.666666666664</v>
+      </c>
       <c r="M2" s="37">
         <v>39.869919000000003</v>
       </c>
@@ -1973,8 +2023,8 @@
       <c r="B3" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="20">
-        <v>4</v>
+      <c r="C3" s="20" t="s">
+        <v>127</v>
       </c>
       <c r="D3" s="20">
         <v>1</v>
@@ -1985,7 +2035,10 @@
       <c r="F3" s="22">
         <v>0.42638888888888887</v>
       </c>
-      <c r="G3" s="10"/>
+      <c r="G3" s="65">
+        <f t="shared" si="0"/>
+        <v>44819.426388888889</v>
+      </c>
       <c r="H3" s="20">
         <v>39.813581999999997</v>
       </c>
@@ -1998,7 +2051,10 @@
       <c r="K3" s="22">
         <v>0.47638888888888892</v>
       </c>
-      <c r="L3" s="22"/>
+      <c r="L3" s="65">
+        <f t="shared" si="1"/>
+        <v>44819.476388888892</v>
+      </c>
       <c r="M3" s="20">
         <v>39.811808999999997</v>
       </c>
@@ -2068,16 +2124,22 @@
         <v>44822</v>
       </c>
       <c r="F4" s="40"/>
-      <c r="G4" s="41"/>
+      <c r="G4" s="91" t="s">
+        <v>128</v>
+      </c>
       <c r="H4" s="37">
         <v>38.944544999999998</v>
       </c>
       <c r="I4" s="37">
         <v>-63.757482000000003</v>
       </c>
-      <c r="J4" s="39"/>
+      <c r="J4" s="39">
+        <v>44822</v>
+      </c>
       <c r="K4" s="40"/>
-      <c r="L4" s="40"/>
+      <c r="L4" s="92" t="s">
+        <v>129</v>
+      </c>
       <c r="M4" s="37">
         <v>38.974831000000002</v>
       </c>
@@ -2115,7 +2177,7 @@
         <v>-63.696891999999998</v>
       </c>
       <c r="Y4" s="51">
-        <f t="shared" ref="Y4:Y39" si="0">(V4-S4)*1440/60</f>
+        <f t="shared" ref="Y4:Y39" si="2">(V4-S4)*1440/60</f>
         <v>9.1666666666860692</v>
       </c>
       <c r="Z4" s="45">
@@ -2148,16 +2210,22 @@
         <v>44822</v>
       </c>
       <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
+      <c r="G5" s="93" t="s">
+        <v>130</v>
+      </c>
       <c r="H5" s="20">
         <v>38.917915000000001</v>
       </c>
       <c r="I5" s="20">
         <v>-63.991678</v>
       </c>
-      <c r="J5" s="21"/>
+      <c r="J5" s="21">
+        <v>44823</v>
+      </c>
       <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="L5" s="22" t="s">
+        <v>131</v>
+      </c>
       <c r="M5" s="20">
         <v>38.868670000000002</v>
       </c>
@@ -2195,7 +2263,7 @@
         <v>-63.74729</v>
       </c>
       <c r="Y5" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.983333333395422</v>
       </c>
       <c r="Z5" s="26">
@@ -2227,16 +2295,22 @@
         <v>44823</v>
       </c>
       <c r="F6" s="48"/>
-      <c r="G6" s="41"/>
+      <c r="G6" s="91" t="s">
+        <v>132</v>
+      </c>
       <c r="H6" s="46">
         <v>38.885973999999997</v>
       </c>
       <c r="I6" s="46">
         <v>-64.015152</v>
       </c>
-      <c r="J6" s="47"/>
+      <c r="J6" s="47">
+        <v>44824</v>
+      </c>
       <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
+      <c r="L6" s="48" t="s">
+        <v>133</v>
+      </c>
       <c r="M6" s="46">
         <v>38.879128999999999</v>
       </c>
@@ -2274,7 +2348,7 @@
         <v>-63.966763999999998</v>
       </c>
       <c r="Y6" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.166666666686069</v>
       </c>
       <c r="Z6" s="52">
@@ -2361,7 +2435,7 @@
         <v>-117.741158</v>
       </c>
       <c r="Y7" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.4972222220967524</v>
       </c>
       <c r="Z7" s="26">
@@ -2438,7 +2512,7 @@
         <v>-117.73635299999999</v>
       </c>
       <c r="Y8" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.250277777784504</v>
       </c>
       <c r="Z8" s="52">
@@ -2513,7 +2587,7 @@
         <v>-117.753174</v>
       </c>
       <c r="Y9" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.499999999941792</v>
       </c>
       <c r="Z9" s="52">
@@ -2588,7 +2662,7 @@
         <v>-117.769451</v>
       </c>
       <c r="Y10" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.083333333430346</v>
       </c>
       <c r="Z10" s="52">
@@ -2663,7 +2737,7 @@
         <v>-117.768916</v>
       </c>
       <c r="Y11" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.583055555529427</v>
       </c>
       <c r="Z11" s="52">
@@ -2748,7 +2822,7 @@
         <v>-117.742642</v>
       </c>
       <c r="Y12" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.827222222171258</v>
       </c>
       <c r="Z12" s="26">
@@ -2823,7 +2897,7 @@
         <v>-117.75370700000001</v>
       </c>
       <c r="Y13" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.333333333255723</v>
       </c>
       <c r="Z13" s="26">
@@ -2902,7 +2976,7 @@
         <v>-117.69389</v>
       </c>
       <c r="Y14" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.7480555555666797</v>
       </c>
       <c r="Z14" s="52">
@@ -2993,7 +3067,7 @@
         <v>-117.75609900000001</v>
       </c>
       <c r="Y15" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1.0922222222434357</v>
       </c>
       <c r="Z15" s="26">
@@ -3070,7 +3144,7 @@
         <v>-117.83437499999999</v>
       </c>
       <c r="Y16" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.746666666760575</v>
       </c>
       <c r="Z16" s="52">
@@ -3145,7 +3219,7 @@
         <v>-117.875584</v>
       </c>
       <c r="Y17" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.666944444470573</v>
       </c>
       <c r="Z17" s="52">
@@ -3220,7 +3294,7 @@
         <v>-117.835121</v>
       </c>
       <c r="Y18" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.996666666585952</v>
       </c>
       <c r="Z18" s="26">
@@ -3295,7 +3369,7 @@
         <v>-117.87147899999999</v>
       </c>
       <c r="Y19" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10.817222222336568</v>
       </c>
       <c r="Z19" s="26">
@@ -3382,7 +3456,7 @@
         <v>-117.434878</v>
       </c>
       <c r="Y20" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>88.993611111072823</v>
       </c>
       <c r="Z20" s="52">
@@ -3419,7 +3493,7 @@
         <v>0.29722222222222222</v>
       </c>
       <c r="G21" s="10">
-        <f t="shared" ref="G21:G39" si="1">$E21+$F21+TIME(AC21,0,0)</f>
+        <f t="shared" ref="G21:G39" si="3">$E21+$F21+TIME(AC21,0,0)</f>
         <v>45203.463888888888</v>
       </c>
       <c r="H21" s="20">
@@ -3435,7 +3509,7 @@
         <v>0.61805555555555558</v>
       </c>
       <c r="L21" s="30">
-        <f t="shared" ref="L21:L40" si="2">$J21+$K21 +TIME($AC21,0,0)</f>
+        <f t="shared" ref="L21:L40" si="4">$J21+$K21 +TIME($AC21,0,0)</f>
         <v>45204.784722222219</v>
       </c>
       <c r="M21" s="20">
@@ -3475,7 +3549,7 @@
         <v>-64.055627999999999</v>
       </c>
       <c r="Y21" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>30.815277777670417</v>
       </c>
       <c r="Z21" s="26">
@@ -3514,7 +3588,7 @@
         <v>0.29444444444444445</v>
       </c>
       <c r="G22" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45203.461111111108</v>
       </c>
       <c r="H22" s="46">
@@ -3530,7 +3604,7 @@
         <v>0.37847222222222227</v>
       </c>
       <c r="L22" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45205.545138888883</v>
       </c>
       <c r="M22" s="46">
@@ -3570,7 +3644,7 @@
         <v>-64.043930000000003</v>
       </c>
       <c r="Y22" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>28.411111111112405</v>
       </c>
       <c r="Z22" s="52">
@@ -3609,7 +3683,7 @@
         <v>0.29444444444444445</v>
       </c>
       <c r="G23" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45203.461111111108</v>
       </c>
       <c r="H23" s="46">
@@ -3625,7 +3699,7 @@
         <v>0.37847222222222227</v>
       </c>
       <c r="L23" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45205.545138888883</v>
       </c>
       <c r="M23" s="46">
@@ -3665,7 +3739,7 @@
         <v>-64.167721999999998</v>
       </c>
       <c r="Y23" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>13.830833333311602</v>
       </c>
       <c r="Z23" s="52">
@@ -3704,7 +3778,7 @@
         <v>0.3034722222222222</v>
       </c>
       <c r="G24" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45203.470138888886</v>
       </c>
       <c r="H24" s="20">
@@ -3720,7 +3794,7 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="L24" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45205.520833333328</v>
       </c>
       <c r="M24" s="20">
@@ -3760,7 +3834,7 @@
         <v>-64.033095000000003</v>
       </c>
       <c r="Y24" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>28.410833333444316</v>
       </c>
       <c r="Z24" s="26">
@@ -3797,7 +3871,7 @@
         <v>0.3034722222222222</v>
       </c>
       <c r="G25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45203.470138888886</v>
       </c>
       <c r="H25" s="20">
@@ -3813,7 +3887,7 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="L25" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45205.520833333328</v>
       </c>
       <c r="M25" s="20">
@@ -3853,7 +3927,7 @@
         <v>-64.137314000000003</v>
       </c>
       <c r="Y25" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>14.916388888901565</v>
       </c>
       <c r="Z25" s="26">
@@ -3890,7 +3964,7 @@
         <v>0.92152777777777783</v>
       </c>
       <c r="G26" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
       <c r="H26" s="46">
@@ -3906,7 +3980,7 @@
         <v>0.40625</v>
       </c>
       <c r="L26" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
       <c r="M26" s="57">
@@ -3946,7 +4020,7 @@
         <v>-63.796340000000001</v>
       </c>
       <c r="Y26" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12.160833333211485</v>
       </c>
       <c r="Z26" s="52">
@@ -3983,7 +4057,7 @@
         <v>0.92152777777777783</v>
       </c>
       <c r="G27" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
       <c r="H27" s="46">
@@ -3999,7 +4073,7 @@
         <v>0.40625</v>
       </c>
       <c r="L27" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
       <c r="M27" s="57">
@@ -4039,7 +4113,7 @@
         <v>-63.812421999999998</v>
       </c>
       <c r="Y27" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>21.233888888906222</v>
       </c>
       <c r="Z27" s="52">
@@ -4076,7 +4150,7 @@
         <v>0.92152777777777783</v>
       </c>
       <c r="G28" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
       <c r="H28" s="46">
@@ -4092,7 +4166,7 @@
         <v>0.40625</v>
       </c>
       <c r="L28" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
       <c r="M28" s="57">
@@ -4132,7 +4206,7 @@
         <v>-63.867663</v>
       </c>
       <c r="Y28" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>18.994444444484543</v>
       </c>
       <c r="Z28" s="52">
@@ -4169,7 +4243,7 @@
         <v>0.9243055555555556</v>
       </c>
       <c r="G29" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.09097222222</v>
       </c>
       <c r="H29" s="20">
@@ -4185,7 +4259,7 @@
         <v>0.31180555555555556</v>
       </c>
       <c r="L29" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45210.478472222218</v>
       </c>
       <c r="M29" s="20">
@@ -4225,7 +4299,7 @@
         <v>-63.765051999999997</v>
       </c>
       <c r="Y29" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>13.330555555585306</v>
       </c>
       <c r="Z29" s="26">
@@ -4264,7 +4338,7 @@
         <v>0.9243055555555556</v>
       </c>
       <c r="G30" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.09097222222</v>
       </c>
       <c r="H30" s="20">
@@ -4280,7 +4354,7 @@
         <v>0.31180555555555556</v>
       </c>
       <c r="L30" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45210.478472222218</v>
       </c>
       <c r="M30" s="20">
@@ -4320,7 +4394,7 @@
         <v>-63.821711999999998</v>
       </c>
       <c r="Y30" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>20.991944444307592</v>
       </c>
       <c r="Z30" s="26">
@@ -4357,7 +4431,7 @@
         <v>0.59722222222222221</v>
       </c>
       <c r="G31" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45208.763888888883</v>
       </c>
       <c r="H31" s="46">
@@ -4373,7 +4447,7 @@
         <v>0.36805555555555558</v>
       </c>
       <c r="L31" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45209.534722222219</v>
       </c>
       <c r="M31" s="46">
@@ -4413,7 +4487,7 @@
         <v>-63.894246000000003</v>
       </c>
       <c r="Y31" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11.827777777682059</v>
       </c>
       <c r="Z31" s="52">
@@ -4452,7 +4526,7 @@
         <v>0.48333333333333334</v>
       </c>
       <c r="G32" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45210.649999999994</v>
       </c>
       <c r="H32" s="20">
@@ -4468,7 +4542,7 @@
         <v>0.60138888888888886</v>
       </c>
       <c r="L32" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45212.768055555556</v>
       </c>
       <c r="M32" s="20">
@@ -4508,7 +4582,7 @@
         <v>-63.895589000000001</v>
       </c>
       <c r="Y32" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>20.577222222229466</v>
       </c>
       <c r="Z32" s="26">
@@ -4547,7 +4621,7 @@
         <v>0.48333333333333334</v>
       </c>
       <c r="G33" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45210.649999999994</v>
       </c>
       <c r="H33" s="20">
@@ -4563,7 +4637,7 @@
         <v>0.60138888888888886</v>
       </c>
       <c r="L33" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45212.768055555556</v>
       </c>
       <c r="M33" s="20">
@@ -4603,7 +4677,7 @@
         <v>-63.928724000000003</v>
       </c>
       <c r="Y33" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>22.649999999965075</v>
       </c>
       <c r="Z33" s="26">
@@ -4640,7 +4714,7 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="G34" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45211.770833333328</v>
       </c>
       <c r="H34" s="46">
@@ -4656,7 +4730,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="L34" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45212.708333333328</v>
       </c>
       <c r="M34" s="46">
@@ -4696,7 +4770,7 @@
         <v>-63.740850999999999</v>
       </c>
       <c r="Y34" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>16.983888888848014</v>
       </c>
       <c r="Z34" s="52">
@@ -4735,7 +4809,7 @@
         <v>0.60763888888888895</v>
       </c>
       <c r="G35" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45211.774305555555</v>
       </c>
       <c r="H35" s="20">
@@ -4751,7 +4825,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="L35" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45212.708333333328</v>
       </c>
       <c r="M35" s="20">
@@ -4791,7 +4865,7 @@
         <v>-63.744534000000002</v>
       </c>
       <c r="Y35" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>17.161111111112405</v>
       </c>
       <c r="Z35" s="26">
@@ -4830,7 +4904,7 @@
         <v>0.50972222222222219</v>
       </c>
       <c r="G36" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
       <c r="H36" s="46"/>
@@ -4842,7 +4916,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="L36" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
       <c r="M36" s="46"/>
@@ -4853,17 +4927,19 @@
       <c r="P36" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q36" s="49"/>
+      <c r="Q36" s="49">
+        <v>300434066482170</v>
+      </c>
       <c r="R36" s="49" t="s">
         <v>37</v>
       </c>
       <c r="S36" s="50">
         <v>45317.875324074077</v>
       </c>
-      <c r="T36" s="72">
+      <c r="T36" s="70">
         <v>32.909129</v>
       </c>
-      <c r="U36" s="72">
+      <c r="U36" s="70">
         <v>-117.680663</v>
       </c>
       <c r="V36" s="50">
@@ -4876,7 +4952,7 @@
         <v>-117.66408699999999</v>
       </c>
       <c r="Y36" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>24.083333333255723</v>
       </c>
       <c r="Z36" s="52">
@@ -4913,7 +4989,7 @@
         <v>0.50972222222222219</v>
       </c>
       <c r="G37" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
       <c r="H37" s="46"/>
@@ -4925,7 +5001,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="L37" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
       <c r="M37" s="46"/>
@@ -4936,17 +5012,19 @@
       <c r="P37" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q37" s="49"/>
+      <c r="Q37" s="49">
+        <v>300434066482170</v>
+      </c>
       <c r="R37" s="49" t="s">
         <v>37</v>
       </c>
       <c r="S37" s="50">
         <v>45318.931122685186</v>
       </c>
-      <c r="T37" s="72">
+      <c r="T37" s="70">
         <v>33.001423000000003</v>
       </c>
-      <c r="U37" s="72">
+      <c r="U37" s="70">
         <v>-117.65347800000001</v>
       </c>
       <c r="V37" s="50">
@@ -4959,7 +5037,7 @@
         <v>-117.6035</v>
       </c>
       <c r="Y37" s="51">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>22.744166666641831</v>
       </c>
       <c r="Z37" s="52">
@@ -4996,7 +5074,7 @@
         <v>0.50972222222222219</v>
       </c>
       <c r="G38" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
       <c r="H38" s="46"/>
@@ -5008,7 +5086,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="L38" s="56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
       <c r="M38" s="46"/>
@@ -5019,30 +5097,32 @@
       <c r="P38" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="Q38" s="49"/>
+      <c r="Q38" s="49">
+        <v>300434066482170</v>
+      </c>
       <c r="R38" s="49" t="s">
         <v>37</v>
       </c>
       <c r="S38" s="50">
         <v>45319.910034722219</v>
       </c>
-      <c r="T38" s="73">
+      <c r="T38" s="71">
         <v>33.123451000000003</v>
       </c>
-      <c r="U38" s="73">
+      <c r="U38" s="71">
         <v>-117.600043</v>
       </c>
       <c r="V38" s="50">
         <v>45320.89980324074</v>
       </c>
-      <c r="W38" s="73">
+      <c r="W38" s="71">
         <v>33.200189999999999</v>
       </c>
-      <c r="X38" s="73">
+      <c r="X38" s="71">
         <v>-117.597759</v>
       </c>
       <c r="Y38" s="51">
-        <f t="shared" ref="Y38" si="3">(V38-S38)*1440/60</f>
+        <f t="shared" ref="Y38" si="5">(V38-S38)*1440/60</f>
         <v>23.754444444493856</v>
       </c>
       <c r="Z38" s="52">
@@ -5079,7 +5159,7 @@
         <v>0.63472222222222219</v>
       </c>
       <c r="G39" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>45317.968055555561</v>
       </c>
       <c r="H39" s="20"/>
@@ -5091,7 +5171,7 @@
         <v>0.51388888888888895</v>
       </c>
       <c r="L39" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45320.847222222226</v>
       </c>
       <c r="M39" s="20"/>
@@ -5102,30 +5182,32 @@
       <c r="P39" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="Q39" s="23"/>
+      <c r="Q39" s="23">
+        <v>300434066480130</v>
+      </c>
       <c r="R39" s="23" t="s">
         <v>44</v>
       </c>
       <c r="S39" s="28">
         <v>45317.993379629632</v>
       </c>
-      <c r="T39" s="74">
+      <c r="T39" s="72">
         <v>32.907333000000001</v>
       </c>
-      <c r="U39" s="74">
+      <c r="U39" s="72">
         <v>-117.67442</v>
       </c>
       <c r="V39" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="W39" s="74">
+      <c r="W39" s="72">
         <v>33.012383</v>
       </c>
-      <c r="X39" s="74">
+      <c r="X39" s="72">
         <v>-117.66186500000001</v>
       </c>
       <c r="Y39" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>21.333611111040227</v>
       </c>
       <c r="Z39" s="26">
@@ -5162,7 +5244,7 @@
         <v>0.63472222222222219</v>
       </c>
       <c r="G40" s="10">
-        <f t="shared" ref="G40" si="4">$E40+$F40+TIME(AC40,0,0)</f>
+        <f t="shared" ref="G40" si="6">$E40+$F40+TIME(AC40,0,0)</f>
         <v>45317.968055555561</v>
       </c>
       <c r="H40" s="20"/>
@@ -5174,7 +5256,7 @@
         <v>0.51388888888888895</v>
       </c>
       <c r="L40" s="30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>45320.847222222226</v>
       </c>
       <c r="M40" s="20"/>
@@ -5185,30 +5267,32 @@
       <c r="P40" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="Q40" s="23"/>
+      <c r="Q40" s="23">
+        <v>300434066480130</v>
+      </c>
       <c r="R40" s="23" t="s">
         <v>44</v>
       </c>
       <c r="S40" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="T40" s="74">
+      <c r="T40" s="72">
         <v>33.012383</v>
       </c>
-      <c r="U40" s="74">
+      <c r="U40" s="72">
         <v>-117.66186500000001</v>
       </c>
       <c r="V40" s="28">
         <v>45320.848263888889</v>
       </c>
-      <c r="W40" s="74">
+      <c r="W40" s="72">
         <v>33.115271</v>
       </c>
-      <c r="X40" s="74">
+      <c r="X40" s="72">
         <v>-117.89773700000001</v>
       </c>
       <c r="Y40" s="25">
-        <f t="shared" ref="Y40" si="5">(V40-S40)*1440/60</f>
+        <f t="shared" ref="Y40" si="7">(V40-S40)*1440/60</f>
         <v>47.183611111133359</v>
       </c>
       <c r="Z40" s="26">
@@ -5267,11 +5351,11 @@
         <v>37</v>
       </c>
       <c r="S41" s="54"/>
-      <c r="T41" s="73"/>
-      <c r="U41" s="73"/>
+      <c r="T41" s="71"/>
+      <c r="U41" s="71"/>
       <c r="V41" s="54"/>
-      <c r="W41" s="73"/>
-      <c r="X41" s="73"/>
+      <c r="W41" s="71"/>
+      <c r="X41" s="71"/>
       <c r="Y41" s="51"/>
       <c r="Z41" s="52"/>
       <c r="AA41" s="52"/>
@@ -5279,161 +5363,161 @@
       <c r="AC41" s="46"/>
       <c r="AD41" s="46"/>
     </row>
-    <row r="42" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="70">
+    <row r="42" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="68">
         <v>26</v>
       </c>
-      <c r="B42" s="70" t="s">
+      <c r="B42" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="70">
+      <c r="C42" s="68">
         <v>5</v>
       </c>
-      <c r="D42" s="70">
+      <c r="D42" s="68">
         <v>1</v>
       </c>
-      <c r="E42" s="80">
+      <c r="E42" s="78">
         <v>45429</v>
       </c>
-      <c r="F42" s="81">
+      <c r="F42" s="79">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G42" s="81" t="s">
+      <c r="G42" s="79" t="s">
         <v>116</v>
       </c>
-      <c r="H42" s="70"/>
-      <c r="I42" s="70"/>
-      <c r="J42" s="80">
+      <c r="H42" s="68"/>
+      <c r="I42" s="68"/>
+      <c r="J42" s="78">
         <v>45432</v>
       </c>
-      <c r="K42" s="81">
+      <c r="K42" s="79">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L42" s="81" t="s">
+      <c r="L42" s="79" t="s">
         <v>117</v>
       </c>
-      <c r="M42" s="70"/>
-      <c r="N42" s="70"/>
-      <c r="O42" s="70">
+      <c r="M42" s="68"/>
+      <c r="N42" s="68"/>
+      <c r="O42" s="68">
         <v>3</v>
       </c>
-      <c r="P42" s="70" t="s">
+      <c r="P42" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="Q42" s="69">
+      <c r="Q42" s="67">
         <v>300434066482170</v>
       </c>
-      <c r="R42" s="69" t="s">
+      <c r="R42" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="S42" s="88" t="s">
+      <c r="S42" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="T42" s="89">
+      <c r="T42" s="72">
         <v>32.917650000000002</v>
       </c>
-      <c r="U42" s="89">
+      <c r="U42" s="72">
         <v>-117.794504</v>
       </c>
-      <c r="V42" s="83" t="s">
+      <c r="V42" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="W42" s="89" t="s">
+      <c r="W42" s="72" t="s">
         <v>120</v>
       </c>
-      <c r="X42" s="89" t="s">
+      <c r="X42" s="72" t="s">
         <v>121</v>
       </c>
-      <c r="Y42" s="85"/>
-      <c r="Z42" s="86">
+      <c r="Y42" s="83"/>
+      <c r="Z42" s="84">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA42" s="86">
+      <c r="AA42" s="84">
         <v>0.1125</v>
       </c>
-      <c r="AB42" s="70"/>
-      <c r="AC42" s="70">
+      <c r="AB42" s="68"/>
+      <c r="AC42" s="68">
         <v>7</v>
       </c>
-      <c r="AD42" s="70"/>
-    </row>
-    <row r="43" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="70">
+      <c r="AD42" s="68"/>
+    </row>
+    <row r="43" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="68">
         <v>26</v>
       </c>
-      <c r="B43" s="70" t="s">
+      <c r="B43" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="70">
+      <c r="C43" s="68">
         <v>5</v>
       </c>
-      <c r="D43" s="70">
+      <c r="D43" s="68">
         <v>2</v>
       </c>
-      <c r="E43" s="80">
+      <c r="E43" s="78">
         <v>45429</v>
       </c>
-      <c r="F43" s="81">
+      <c r="F43" s="79">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G43" s="81" t="s">
+      <c r="G43" s="79" t="s">
         <v>116</v>
       </c>
-      <c r="H43" s="70"/>
-      <c r="I43" s="70"/>
-      <c r="J43" s="80">
+      <c r="H43" s="68"/>
+      <c r="I43" s="68"/>
+      <c r="J43" s="78">
         <v>45432</v>
       </c>
-      <c r="K43" s="81">
+      <c r="K43" s="79">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L43" s="81" t="s">
+      <c r="L43" s="79" t="s">
         <v>117</v>
       </c>
-      <c r="M43" s="70"/>
-      <c r="N43" s="70"/>
-      <c r="O43" s="70">
+      <c r="M43" s="68"/>
+      <c r="N43" s="68"/>
+      <c r="O43" s="68">
         <v>3</v>
       </c>
-      <c r="P43" s="70" t="s">
+      <c r="P43" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="Q43" s="69">
+      <c r="Q43" s="67">
         <v>300434066482170</v>
       </c>
-      <c r="R43" s="69" t="s">
+      <c r="R43" s="67" t="s">
         <v>115</v>
       </c>
-      <c r="S43" s="84" t="s">
+      <c r="S43" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="T43" s="89">
+      <c r="T43" s="72">
         <v>32.998700999999997</v>
       </c>
-      <c r="U43" s="89">
+      <c r="U43" s="72">
         <v>-117.874388</v>
       </c>
-      <c r="V43" s="84" t="s">
+      <c r="V43" s="28" t="s">
         <v>123</v>
       </c>
-      <c r="W43" s="89">
+      <c r="W43" s="72">
         <v>33.012540000000001</v>
       </c>
-      <c r="X43" s="70">
+      <c r="X43" s="72">
         <v>-117.890097</v>
       </c>
-      <c r="Y43" s="85"/>
-      <c r="Z43" s="86">
+      <c r="Y43" s="83"/>
+      <c r="Z43" s="84">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA43" s="86">
+      <c r="AA43" s="84">
         <v>0.1125</v>
       </c>
-      <c r="AB43" s="70"/>
-      <c r="AC43" s="70">
+      <c r="AB43" s="68"/>
+      <c r="AC43" s="68">
         <v>7</v>
       </c>
-      <c r="AD43" s="70"/>
+      <c r="AD43" s="68"/>
     </row>
     <row r="44" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="46">
@@ -5448,10 +5532,10 @@
       <c r="D44" s="46">
         <v>1</v>
       </c>
-      <c r="E44" s="75">
+      <c r="E44" s="73">
         <v>45462</v>
       </c>
-      <c r="F44" s="76">
+      <c r="F44" s="74">
         <v>0.625</v>
       </c>
       <c r="G44" s="41">
@@ -5462,8 +5546,8 @@
       <c r="I44" s="46"/>
       <c r="J44" s="47"/>
       <c r="K44" s="48"/>
-      <c r="M44" s="73"/>
-      <c r="N44" s="73"/>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
       <c r="O44" s="46">
         <v>3</v>
       </c>
@@ -5479,10 +5563,10 @@
       <c r="S44" s="54">
         <v>45462.860289351855</v>
       </c>
-      <c r="T44" s="73">
+      <c r="T44" s="71">
         <v>38.313133999999998</v>
       </c>
-      <c r="U44" s="73">
+      <c r="U44" s="71">
         <v>-63.006925000000003</v>
       </c>
       <c r="V44" s="50"/>
@@ -5497,231 +5581,276 @@
       </c>
       <c r="AD44" s="46"/>
     </row>
-    <row r="45" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="70">
+    <row r="45" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="68">
         <v>28</v>
       </c>
-      <c r="B45" s="70" t="s">
+      <c r="B45" s="68" t="s">
         <v>124</v>
       </c>
-      <c r="C45" s="70">
+      <c r="C45" s="68">
         <v>6</v>
       </c>
-      <c r="D45" s="70">
+      <c r="D45" s="68">
         <v>1</v>
       </c>
-      <c r="E45" s="78">
+      <c r="E45" s="76">
         <v>45462</v>
       </c>
-      <c r="F45" s="79">
+      <c r="F45" s="77">
         <v>0.625</v>
       </c>
-      <c r="G45" s="67">
-        <f t="shared" ref="G45:G46" si="6">$E45+$F45+TIME(AC45,0,0)</f>
+      <c r="G45" s="65">
+        <f t="shared" ref="G45" si="8">$E45+$F45+TIME(AC45,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H45" s="70"/>
-      <c r="I45" s="70"/>
-      <c r="J45" s="80"/>
-      <c r="K45" s="81"/>
-      <c r="L45" s="68"/>
-      <c r="M45" s="82"/>
-      <c r="N45" s="82"/>
-      <c r="O45" s="70">
+      <c r="H45" s="68"/>
+      <c r="I45" s="68"/>
+      <c r="J45" s="78"/>
+      <c r="K45" s="79"/>
+      <c r="L45" s="66"/>
+      <c r="M45" s="80"/>
+      <c r="N45" s="80"/>
+      <c r="O45" s="68">
         <v>4</v>
       </c>
-      <c r="P45" s="70" t="s">
+      <c r="P45" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="Q45" s="69">
+      <c r="Q45" s="67">
         <v>300434066480130</v>
       </c>
-      <c r="R45" s="69" t="s">
+      <c r="R45" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="S45" s="83">
-        <v>45462.855231481481</v>
-      </c>
-      <c r="T45" s="82">
-        <v>38.307771000000002</v>
-      </c>
-      <c r="U45" s="82">
-        <v>-62.998032000000002</v>
-      </c>
-      <c r="V45" s="84"/>
-      <c r="W45" s="70"/>
-      <c r="X45" s="70"/>
-      <c r="Y45" s="85"/>
-      <c r="Z45" s="86"/>
-      <c r="AA45" s="86"/>
-      <c r="AB45" s="70"/>
-      <c r="AC45" s="70">
+      <c r="S45" s="28">
+        <v>45462.830416666664</v>
+      </c>
+      <c r="T45" s="94">
+        <v>38.311219000000001</v>
+      </c>
+      <c r="U45" s="94">
+        <v>-63.003127999999997</v>
+      </c>
+      <c r="V45" s="28">
+        <v>45462.83388888889</v>
+      </c>
+      <c r="W45" s="94">
+        <v>38.310768000000003</v>
+      </c>
+      <c r="X45" s="94">
+        <v>-63.002412999999997</v>
+      </c>
+      <c r="Y45" s="83"/>
+      <c r="Z45" s="84"/>
+      <c r="AA45" s="84"/>
+      <c r="AB45" s="68"/>
+      <c r="AC45" s="68">
         <v>4</v>
       </c>
-      <c r="AD45" s="70"/>
-    </row>
-    <row r="46" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="46">
+      <c r="AD45" s="68"/>
+    </row>
+    <row r="46" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="68">
+        <v>28</v>
+      </c>
+      <c r="B46" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="C46" s="68">
+        <v>6</v>
+      </c>
+      <c r="D46" s="68">
+        <v>2</v>
+      </c>
+      <c r="E46" s="76">
+        <v>45462</v>
+      </c>
+      <c r="F46" s="77">
+        <v>0.625</v>
+      </c>
+      <c r="G46" s="65">
+        <f t="shared" ref="G46" si="9">$E46+$F46+TIME(AC46,0,0)</f>
+        <v>45462.625</v>
+      </c>
+      <c r="H46" s="68"/>
+      <c r="I46" s="68"/>
+      <c r="J46" s="78"/>
+      <c r="K46" s="79"/>
+      <c r="L46" s="66"/>
+      <c r="M46" s="80"/>
+      <c r="N46" s="80"/>
+      <c r="O46" s="68">
+        <v>4</v>
+      </c>
+      <c r="P46" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="B46" s="46" t="s">
+      <c r="Q46" s="67">
+        <v>300434066480130</v>
+      </c>
+      <c r="R46" s="67" t="s">
+        <v>44</v>
+      </c>
+      <c r="S46" s="81">
+        <v>45465.271736111114</v>
+      </c>
+      <c r="T46" s="94">
+        <v>38.415380999999996</v>
+      </c>
+      <c r="U46" s="94">
+        <v>-62.463433000000002</v>
+      </c>
+      <c r="V46" s="28">
+        <v>45466.125555555554</v>
+      </c>
+      <c r="W46" s="94">
+        <v>38.532255999999997</v>
+      </c>
+      <c r="X46" s="94">
+        <v>-62.362059000000002</v>
+      </c>
+      <c r="Y46" s="83"/>
+      <c r="Z46" s="84"/>
+      <c r="AA46" s="84"/>
+      <c r="AB46" s="68"/>
+      <c r="AC46" s="68"/>
+      <c r="AD46" s="68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="47" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="46">
+        <v>29</v>
+      </c>
+      <c r="B47" s="46" t="s">
         <v>124</v>
       </c>
-      <c r="C46" s="46">
+      <c r="C47" s="46">
         <v>4</v>
       </c>
-      <c r="D46" s="46">
+      <c r="D47" s="46">
         <v>1</v>
       </c>
-      <c r="E46" s="75">
+      <c r="E47" s="73">
         <v>45462</v>
       </c>
-      <c r="F46" s="76">
+      <c r="F47" s="74">
         <v>0.625</v>
       </c>
-      <c r="G46" s="41">
-        <f>$E46+$F46+TIME(AC46,0,0)</f>
+      <c r="G47" s="41">
+        <f>$E47+$F47+TIME(AC47,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H46" s="46">
+      <c r="H47" s="46">
         <v>38.316051999999999</v>
       </c>
-      <c r="I46" s="46">
+      <c r="I47" s="46">
         <v>-63.012607000000003</v>
       </c>
-      <c r="J46" s="47">
+      <c r="J47" s="47">
         <v>45464</v>
       </c>
-      <c r="K46" s="48">
+      <c r="K47" s="48">
         <v>0.125</v>
       </c>
-      <c r="L46" s="56">
-        <f t="shared" ref="L46" si="7">$J46+$K46 +TIME($AC46,0,0)</f>
+      <c r="L47" s="56">
+        <f t="shared" ref="L47" si="10">$J47+$K47 +TIME($AC47,0,0)</f>
         <v>45464.291666666664</v>
       </c>
-      <c r="M46" s="73">
+      <c r="M47" s="71">
         <v>38.309516000000002</v>
       </c>
-      <c r="N46" s="73">
+      <c r="N47" s="71">
         <v>-62.619463000000003</v>
       </c>
-      <c r="O46" s="46">
+      <c r="O47" s="46">
         <v>1</v>
       </c>
-      <c r="P46" s="46" t="s">
+      <c r="P47" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="Q46" s="77">
+      <c r="Q47" s="75">
         <v>300434066489180</v>
       </c>
-      <c r="R46" s="49" t="s">
+      <c r="R47" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="S46" s="54">
+      <c r="S47" s="54">
         <v>45462.84778935185</v>
       </c>
-      <c r="T46" s="73">
+      <c r="T47" s="71">
         <v>38.315800000000003</v>
       </c>
-      <c r="U46" s="73">
+      <c r="U47" s="71">
         <v>-63.012493999999997</v>
       </c>
-      <c r="V46" s="54">
+      <c r="V47" s="54">
         <v>45463.528101851851</v>
       </c>
-      <c r="W46" s="73">
+      <c r="W47" s="71">
         <v>38.311391</v>
       </c>
-      <c r="X46" s="73">
+      <c r="X47" s="71">
         <v>-62.918548000000001</v>
       </c>
-      <c r="Y46" s="51">
-        <f t="shared" ref="Y46" si="8">(V46-S46)*1440/60</f>
+      <c r="Y47" s="51">
+        <f t="shared" ref="Y47" si="11">(V47-S47)*1440/60</f>
         <v>16.32750000001397</v>
       </c>
-      <c r="Z46" s="52"/>
-      <c r="AA46" s="52"/>
-      <c r="AB46" s="46"/>
-      <c r="AC46" s="46">
+      <c r="Z47" s="52"/>
+      <c r="AA47" s="52"/>
+      <c r="AB47" s="46"/>
+      <c r="AC47" s="46">
         <v>4</v>
       </c>
-      <c r="AD46" s="46"/>
-    </row>
-    <row r="47" spans="1:30" s="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="70"/>
-      <c r="B47" s="70"/>
-      <c r="C47" s="70"/>
-      <c r="D47" s="70"/>
-      <c r="E47" s="88"/>
-      <c r="F47" s="89"/>
-      <c r="G47" s="89"/>
-      <c r="H47" s="83"/>
-      <c r="I47" s="89"/>
-      <c r="J47" s="90"/>
-      <c r="K47" s="81"/>
-      <c r="L47" s="81"/>
-      <c r="M47" s="70"/>
-      <c r="N47" s="70"/>
-      <c r="O47" s="70"/>
-      <c r="P47" s="70"/>
-      <c r="Q47" s="69"/>
-      <c r="R47" s="69"/>
-      <c r="S47" s="84"/>
-      <c r="T47" s="70"/>
-      <c r="U47" s="70"/>
-      <c r="V47" s="84"/>
-      <c r="W47" s="70"/>
-      <c r="X47" s="70"/>
-      <c r="Y47" s="85"/>
-      <c r="Z47" s="86"/>
-      <c r="AA47" s="86"/>
-      <c r="AB47" s="70"/>
-      <c r="AC47" s="70"/>
-      <c r="AD47" s="70"/>
-    </row>
-    <row r="48" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="71"/>
-      <c r="G48" s="71"/>
-      <c r="H48" s="24"/>
-      <c r="I48" s="64"/>
-      <c r="J48" s="20"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="20"/>
-      <c r="N48" s="20"/>
-      <c r="O48" s="20"/>
-      <c r="P48" s="20"/>
-      <c r="Q48" s="23"/>
-      <c r="R48" s="23"/>
-      <c r="S48" s="24"/>
-      <c r="T48" s="20"/>
-      <c r="U48" s="20"/>
-      <c r="V48" s="24"/>
-      <c r="W48" s="20"/>
-      <c r="X48" s="20"/>
-      <c r="Y48" s="25"/>
-      <c r="Z48" s="26"/>
-      <c r="AA48" s="26"/>
-      <c r="AB48" s="20"/>
-      <c r="AC48" s="20"/>
-      <c r="AD48" s="20"/>
+      <c r="AD47" s="46" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="48" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="68"/>
+      <c r="B48" s="68"/>
+      <c r="C48" s="68"/>
+      <c r="D48" s="68"/>
+      <c r="E48" s="86"/>
+      <c r="F48" s="87"/>
+      <c r="G48" s="87"/>
+      <c r="H48" s="81"/>
+      <c r="I48" s="87"/>
+      <c r="J48" s="88"/>
+      <c r="K48" s="79"/>
+      <c r="L48" s="79"/>
+      <c r="M48" s="68"/>
+      <c r="N48" s="68"/>
+      <c r="O48" s="68"/>
+      <c r="P48" s="68"/>
+      <c r="Q48" s="67"/>
+      <c r="R48" s="67"/>
+      <c r="S48" s="82"/>
+      <c r="T48" s="68"/>
+      <c r="U48" s="68"/>
+      <c r="V48" s="82"/>
+      <c r="W48" s="68"/>
+      <c r="X48" s="68"/>
+      <c r="Y48" s="83"/>
+      <c r="Z48" s="84"/>
+      <c r="AA48" s="84"/>
+      <c r="AB48" s="68"/>
+      <c r="AC48" s="68"/>
+      <c r="AD48" s="68"/>
     </row>
     <row r="49" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="20"/>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
       <c r="D49" s="20"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="20"/>
-      <c r="J49" s="21"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="69"/>
+      <c r="G49" s="69"/>
+      <c r="H49" s="24"/>
+      <c r="I49" s="64"/>
+      <c r="J49" s="20"/>
       <c r="K49" s="22"/>
       <c r="L49" s="22"/>
       <c r="M49" s="20"/>
@@ -36335,6 +36464,38 @@
       <c r="AC1005" s="20"/>
       <c r="AD1005" s="20"/>
     </row>
+    <row r="1006" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1006" s="20"/>
+      <c r="B1006" s="20"/>
+      <c r="C1006" s="20"/>
+      <c r="D1006" s="20"/>
+      <c r="E1006" s="21"/>
+      <c r="F1006" s="22"/>
+      <c r="G1006" s="22"/>
+      <c r="H1006" s="20"/>
+      <c r="I1006" s="20"/>
+      <c r="J1006" s="21"/>
+      <c r="K1006" s="22"/>
+      <c r="L1006" s="22"/>
+      <c r="M1006" s="20"/>
+      <c r="N1006" s="20"/>
+      <c r="O1006" s="20"/>
+      <c r="P1006" s="20"/>
+      <c r="Q1006" s="23"/>
+      <c r="R1006" s="23"/>
+      <c r="S1006" s="24"/>
+      <c r="T1006" s="20"/>
+      <c r="U1006" s="20"/>
+      <c r="V1006" s="24"/>
+      <c r="W1006" s="20"/>
+      <c r="X1006" s="20"/>
+      <c r="Y1006" s="25"/>
+      <c r="Z1006" s="26"/>
+      <c r="AA1006" s="26"/>
+      <c r="AB1006" s="20"/>
+      <c r="AC1006" s="20"/>
+      <c r="AD1006" s="20"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AD35" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -46544,11 +46705,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="89" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
correcting folder names for 2022 data
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438AC3A6-A7DD-2E4E-90E3-0292286EAAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9132FCAC-2B56-8345-83BA-723C5DE4829E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="135">
   <si>
     <t>Deployment</t>
   </si>
@@ -425,9 +425,6 @@
     <t>20240513T211836</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
     <t>20220918T030844</t>
   </si>
   <si>
@@ -745,9 +742,6 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -862,10 +856,6 @@
     <xf numFmtId="22" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="168" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -876,6 +866,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -2004,12 +1999,19 @@
         <v>36</v>
       </c>
       <c r="S2" s="43"/>
+      <c r="T2" s="94"/>
+      <c r="U2" s="94"/>
       <c r="V2" s="43"/>
-      <c r="Y2" s="44"/>
-      <c r="Z2" s="45">
+      <c r="W2" s="94"/>
+      <c r="X2" s="94"/>
+      <c r="Y2" s="50">
+        <f t="shared" ref="Y2:Y39" si="2">(V2-S2)*1440/60</f>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="44">
         <v>0.43124999999999997</v>
       </c>
-      <c r="AA2" s="45">
+      <c r="AA2" s="44">
         <v>0.45208333333333334</v>
       </c>
       <c r="AD2" s="37" t="s">
@@ -2023,8 +2025,8 @@
       <c r="B3" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="20" t="s">
-        <v>127</v>
+      <c r="C3" s="20">
+        <v>4</v>
       </c>
       <c r="D3" s="20">
         <v>1</v>
@@ -2035,7 +2037,7 @@
       <c r="F3" s="22">
         <v>0.42638888888888887</v>
       </c>
-      <c r="G3" s="65">
+      <c r="G3" s="64">
         <f t="shared" si="0"/>
         <v>44819.426388888889</v>
       </c>
@@ -2051,7 +2053,7 @@
       <c r="K3" s="22">
         <v>0.47638888888888892</v>
       </c>
-      <c r="L3" s="65">
+      <c r="L3" s="64">
         <f t="shared" si="1"/>
         <v>44819.476388888892</v>
       </c>
@@ -2124,8 +2126,8 @@
         <v>44822</v>
       </c>
       <c r="F4" s="40"/>
-      <c r="G4" s="91" t="s">
-        <v>128</v>
+      <c r="G4" s="88" t="s">
+        <v>127</v>
       </c>
       <c r="H4" s="37">
         <v>38.944544999999998</v>
@@ -2137,8 +2139,8 @@
         <v>44822</v>
       </c>
       <c r="K4" s="40"/>
-      <c r="L4" s="92" t="s">
-        <v>129</v>
+      <c r="L4" s="89" t="s">
+        <v>128</v>
       </c>
       <c r="M4" s="37">
         <v>38.974831000000002</v>
@@ -2176,14 +2178,14 @@
       <c r="X4" s="37">
         <v>-63.696891999999998</v>
       </c>
-      <c r="Y4" s="51">
-        <f t="shared" ref="Y4:Y39" si="2">(V4-S4)*1440/60</f>
+      <c r="Y4" s="50">
+        <f t="shared" si="2"/>
         <v>9.1666666666860692</v>
       </c>
-      <c r="Z4" s="45">
+      <c r="Z4" s="44">
         <v>0.41597222222222219</v>
       </c>
-      <c r="AA4" s="45">
+      <c r="AA4" s="44">
         <v>0.92986111111111114</v>
       </c>
       <c r="AB4" s="37">
@@ -2210,8 +2212,8 @@
         <v>44822</v>
       </c>
       <c r="F5" s="22"/>
-      <c r="G5" s="93" t="s">
-        <v>130</v>
+      <c r="G5" s="90" t="s">
+        <v>129</v>
       </c>
       <c r="H5" s="20">
         <v>38.917915000000001</v>
@@ -2224,7 +2226,7 @@
       </c>
       <c r="K5" s="22"/>
       <c r="L5" s="22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M5" s="20">
         <v>38.868670000000002</v>
@@ -2278,90 +2280,90 @@
       <c r="AC5" s="20"/>
       <c r="AD5" s="20"/>
     </row>
-    <row r="6" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="46">
+    <row r="6" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="45">
         <v>5</v>
       </c>
       <c r="B6" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="45">
         <v>4</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="45">
         <v>1</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="46">
         <v>44823</v>
       </c>
-      <c r="F6" s="48"/>
-      <c r="G6" s="91" t="s">
+      <c r="F6" s="47"/>
+      <c r="G6" s="88" t="s">
+        <v>131</v>
+      </c>
+      <c r="H6" s="45">
+        <v>38.885973999999997</v>
+      </c>
+      <c r="I6" s="45">
+        <v>-64.015152</v>
+      </c>
+      <c r="J6" s="46">
+        <v>44824</v>
+      </c>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47" t="s">
         <v>132</v>
       </c>
-      <c r="H6" s="46">
-        <v>38.885973999999997</v>
-      </c>
-      <c r="I6" s="46">
-        <v>-64.015152</v>
-      </c>
-      <c r="J6" s="47">
-        <v>44824</v>
-      </c>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="M6" s="46">
+      <c r="M6" s="45">
         <v>38.879128999999999</v>
       </c>
-      <c r="N6" s="46">
+      <c r="N6" s="45">
         <v>-63.895172000000002</v>
       </c>
-      <c r="O6" s="46">
+      <c r="O6" s="45">
         <v>1</v>
       </c>
-      <c r="P6" s="46" t="s">
+      <c r="P6" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q6" s="49">
+      <c r="Q6" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R6" s="49" t="s">
+      <c r="R6" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="S6" s="50">
+      <c r="S6" s="49">
         <v>44823.822916666664</v>
       </c>
-      <c r="T6" s="46">
+      <c r="T6" s="45">
         <v>38.886195999999998</v>
       </c>
-      <c r="U6" s="46">
+      <c r="U6" s="45">
         <v>-64.012355999999997</v>
       </c>
-      <c r="V6" s="50">
+      <c r="V6" s="49">
         <v>44824.329861111109</v>
       </c>
-      <c r="W6" s="46">
+      <c r="W6" s="45">
         <v>38.854120000000002</v>
       </c>
-      <c r="X6" s="46">
+      <c r="X6" s="45">
         <v>-63.966763999999998</v>
       </c>
-      <c r="Y6" s="51">
+      <c r="Y6" s="50">
         <f t="shared" si="2"/>
         <v>12.166666666686069</v>
       </c>
-      <c r="Z6" s="52">
+      <c r="Z6" s="51">
         <v>0.41666666666666669</v>
       </c>
-      <c r="AA6" s="52">
+      <c r="AA6" s="51">
         <v>0.92847222222222225</v>
       </c>
-      <c r="AB6" s="46">
+      <c r="AB6" s="45">
         <v>400</v>
       </c>
-      <c r="AC6" s="46"/>
-      <c r="AD6" s="46" t="s">
+      <c r="AC6" s="45"/>
+      <c r="AD6" s="45" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2452,305 +2454,305 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="46">
+    <row r="8" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="45">
         <v>7</v>
       </c>
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="45">
         <v>4</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="45">
         <v>1</v>
       </c>
-      <c r="E8" s="47">
+      <c r="E8" s="46">
         <v>44983</v>
       </c>
-      <c r="F8" s="48"/>
+      <c r="F8" s="47"/>
       <c r="G8" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="46"/>
-      <c r="I8" s="46"/>
-      <c r="J8" s="47"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48" t="s">
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="M8" s="46"/>
-      <c r="N8" s="46"/>
-      <c r="O8" s="46">
+      <c r="M8" s="45"/>
+      <c r="N8" s="45"/>
+      <c r="O8" s="45">
         <v>1</v>
       </c>
-      <c r="P8" s="46" t="s">
+      <c r="P8" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q8" s="49">
+      <c r="Q8" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R8" s="49" t="s">
+      <c r="R8" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S8" s="50">
+      <c r="S8" s="49">
         <v>44983.875324074077</v>
       </c>
-      <c r="T8" s="46">
+      <c r="T8" s="45">
         <v>32.910995</v>
       </c>
-      <c r="U8" s="46">
+      <c r="U8" s="45">
         <v>-117.74101400000001</v>
       </c>
-      <c r="V8" s="50">
+      <c r="V8" s="49">
         <v>44984.385752314818</v>
       </c>
-      <c r="W8" s="46">
+      <c r="W8" s="45">
         <v>32.911644000000003</v>
       </c>
-      <c r="X8" s="46">
+      <c r="X8" s="45">
         <v>-117.73635299999999</v>
       </c>
-      <c r="Y8" s="51">
+      <c r="Y8" s="50">
         <f t="shared" si="2"/>
         <v>12.250277777784504</v>
       </c>
-      <c r="Z8" s="52">
+      <c r="Z8" s="51">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA8" s="52">
+      <c r="AA8" s="51">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB8" s="46">
+      <c r="AB8" s="45">
         <v>250</v>
       </c>
-      <c r="AC8" s="46"/>
-      <c r="AD8" s="46"/>
-    </row>
-    <row r="9" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="46">
+      <c r="AC8" s="45"/>
+      <c r="AD8" s="45"/>
+    </row>
+    <row r="9" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="45">
         <v>7</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="45">
         <v>4</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="45">
         <v>2</v>
       </c>
-      <c r="E9" s="47">
+      <c r="E9" s="46">
         <v>44983</v>
       </c>
-      <c r="F9" s="48"/>
+      <c r="F9" s="47"/>
       <c r="G9" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
-      <c r="J9" s="47"/>
-      <c r="K9" s="48"/>
-      <c r="L9" s="48" t="s">
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="M9" s="46"/>
-      <c r="N9" s="46"/>
-      <c r="O9" s="46">
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45">
         <v>1</v>
       </c>
-      <c r="P9" s="46" t="s">
+      <c r="P9" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q9" s="49">
+      <c r="Q9" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R9" s="49" t="s">
+      <c r="R9" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S9" s="50">
+      <c r="S9" s="49">
         <v>44984.416990740741</v>
       </c>
-      <c r="T9" s="46">
+      <c r="T9" s="45">
         <v>32.908870999999998</v>
       </c>
-      <c r="U9" s="46">
+      <c r="U9" s="45">
         <v>-117.73746199999999</v>
       </c>
-      <c r="V9" s="50">
+      <c r="V9" s="49">
         <v>44984.896157407406</v>
       </c>
-      <c r="W9" s="46">
+      <c r="W9" s="45">
         <v>32.92512</v>
       </c>
-      <c r="X9" s="46">
+      <c r="X9" s="45">
         <v>-117.753174</v>
       </c>
-      <c r="Y9" s="51">
+      <c r="Y9" s="50">
         <f t="shared" si="2"/>
         <v>11.499999999941792</v>
       </c>
-      <c r="Z9" s="52">
+      <c r="Z9" s="51">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA9" s="52">
+      <c r="AA9" s="51">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB9" s="46">
+      <c r="AB9" s="45">
         <v>250</v>
       </c>
-      <c r="AC9" s="46"/>
-      <c r="AD9" s="46"/>
-    </row>
-    <row r="10" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="46">
+      <c r="AC9" s="45"/>
+      <c r="AD9" s="45"/>
+    </row>
+    <row r="10" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="45">
         <v>7</v>
       </c>
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="45">
         <v>4</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="45">
         <v>3</v>
       </c>
-      <c r="E10" s="47">
+      <c r="E10" s="46">
         <v>44983</v>
       </c>
-      <c r="F10" s="48"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="48" t="s">
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="M10" s="46"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46">
+      <c r="M10" s="45"/>
+      <c r="N10" s="45"/>
+      <c r="O10" s="45">
         <v>1</v>
       </c>
-      <c r="P10" s="46" t="s">
+      <c r="P10" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q10" s="49">
+      <c r="Q10" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R10" s="49" t="s">
+      <c r="R10" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S10" s="50">
+      <c r="S10" s="49">
         <v>44984.896157407406</v>
       </c>
-      <c r="T10" s="46">
+      <c r="T10" s="45">
         <v>32.92512</v>
       </c>
-      <c r="U10" s="46">
+      <c r="U10" s="45">
         <v>-117.753174</v>
       </c>
-      <c r="V10" s="50">
+      <c r="V10" s="49">
         <v>44985.399629629632</v>
       </c>
-      <c r="W10" s="46">
+      <c r="W10" s="45">
         <v>32.922975999999998</v>
       </c>
-      <c r="X10" s="46">
+      <c r="X10" s="45">
         <v>-117.769451</v>
       </c>
-      <c r="Y10" s="51">
+      <c r="Y10" s="50">
         <f t="shared" si="2"/>
         <v>12.083333333430346</v>
       </c>
-      <c r="Z10" s="52">
+      <c r="Z10" s="51">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA10" s="52">
+      <c r="AA10" s="51">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB10" s="46">
+      <c r="AB10" s="45">
         <v>250</v>
       </c>
-      <c r="AC10" s="46"/>
-      <c r="AD10" s="46"/>
-    </row>
-    <row r="11" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="46">
+      <c r="AC10" s="45"/>
+      <c r="AD10" s="45"/>
+    </row>
+    <row r="11" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="45">
         <v>7</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="45">
         <v>4</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="45">
         <v>4</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="46">
         <v>44983</v>
       </c>
-      <c r="F11" s="48"/>
+      <c r="F11" s="47"/>
       <c r="G11" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="48"/>
-      <c r="L11" s="48" t="s">
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="47"/>
+      <c r="L11" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="M11" s="46"/>
-      <c r="N11" s="46"/>
-      <c r="O11" s="46">
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45">
         <v>1</v>
       </c>
-      <c r="P11" s="46" t="s">
+      <c r="P11" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q11" s="49">
+      <c r="Q11" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R11" s="49" t="s">
+      <c r="R11" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S11" s="50">
+      <c r="S11" s="49">
         <v>44985.403113425928</v>
       </c>
-      <c r="T11" s="46">
+      <c r="T11" s="45">
         <v>32.922437000000002</v>
       </c>
-      <c r="U11" s="46">
+      <c r="U11" s="45">
         <v>-117.76988799999999</v>
       </c>
-      <c r="V11" s="50">
+      <c r="V11" s="49">
         <v>44985.885740740741</v>
       </c>
-      <c r="W11" s="46">
+      <c r="W11" s="45">
         <v>32.938851</v>
       </c>
-      <c r="X11" s="46">
+      <c r="X11" s="45">
         <v>-117.768916</v>
       </c>
-      <c r="Y11" s="51">
+      <c r="Y11" s="50">
         <f t="shared" si="2"/>
         <v>11.583055555529427</v>
       </c>
-      <c r="Z11" s="52">
+      <c r="Z11" s="51">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA11" s="52">
+      <c r="AA11" s="51">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB11" s="46">
+      <c r="AB11" s="45">
         <v>250</v>
       </c>
-      <c r="AC11" s="46"/>
-      <c r="AD11" s="46"/>
+      <c r="AC11" s="45"/>
+      <c r="AD11" s="45"/>
     </row>
     <row r="12" spans="1:30" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="20">
@@ -2912,84 +2914,84 @@
       <c r="AC13" s="20"/>
       <c r="AD13" s="20"/>
     </row>
-    <row r="14" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="46">
+    <row r="14" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="45">
         <v>9</v>
       </c>
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="45">
         <v>6</v>
       </c>
-      <c r="D14" s="46">
+      <c r="D14" s="45">
         <v>1</v>
       </c>
-      <c r="E14" s="47">
+      <c r="E14" s="46">
         <v>44985</v>
       </c>
-      <c r="F14" s="48"/>
+      <c r="F14" s="47"/>
       <c r="G14" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="46">
+      <c r="H14" s="45">
         <v>32.912492</v>
       </c>
-      <c r="I14" s="46">
+      <c r="I14" s="45">
         <v>-117.69094200000001</v>
       </c>
-      <c r="J14" s="47"/>
-      <c r="K14" s="48"/>
-      <c r="L14" s="48" t="s">
+      <c r="J14" s="46"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="M14" s="46"/>
-      <c r="N14" s="46"/>
-      <c r="O14" s="46">
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+      <c r="O14" s="45">
         <v>4</v>
       </c>
-      <c r="P14" s="46" t="s">
+      <c r="P14" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="49">
+      <c r="Q14" s="48">
         <v>300434066489180</v>
       </c>
-      <c r="R14" s="49" t="s">
+      <c r="R14" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="S14" s="50">
+      <c r="S14" s="49">
         <v>44985.715925925928</v>
       </c>
-      <c r="T14" s="46">
+      <c r="T14" s="45">
         <v>32.911934000000002</v>
       </c>
-      <c r="U14" s="46">
+      <c r="U14" s="45">
         <v>-117.691322</v>
       </c>
-      <c r="V14" s="50">
+      <c r="V14" s="49">
         <v>44985.788761574076</v>
       </c>
-      <c r="W14" s="46">
+      <c r="W14" s="45">
         <v>32.910586000000002</v>
       </c>
-      <c r="X14" s="46">
+      <c r="X14" s="45">
         <v>-117.69389</v>
       </c>
-      <c r="Y14" s="51">
+      <c r="Y14" s="50">
         <f t="shared" si="2"/>
         <v>1.7480555555666797</v>
       </c>
-      <c r="Z14" s="52">
+      <c r="Z14" s="51">
         <v>0.59861111111111109</v>
       </c>
-      <c r="AA14" s="52">
+      <c r="AA14" s="51">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="AB14" s="46">
+      <c r="AB14" s="45">
         <v>250</v>
       </c>
-      <c r="AC14" s="46"/>
-      <c r="AD14" s="46" t="s">
+      <c r="AC14" s="45"/>
+      <c r="AD14" s="45" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3084,155 +3086,155 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="46">
+    <row r="16" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="45">
         <v>11</v>
       </c>
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="45">
         <v>4</v>
       </c>
-      <c r="D16" s="46">
+      <c r="D16" s="45">
         <v>1</v>
       </c>
-      <c r="E16" s="47">
+      <c r="E16" s="46">
         <v>45084</v>
       </c>
-      <c r="F16" s="48"/>
+      <c r="F16" s="47"/>
       <c r="G16" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="47"/>
-      <c r="K16" s="48"/>
-      <c r="L16" s="48" t="s">
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="46"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="M16" s="46"/>
-      <c r="N16" s="46"/>
-      <c r="O16" s="46">
+      <c r="M16" s="45"/>
+      <c r="N16" s="45"/>
+      <c r="O16" s="45">
         <v>1</v>
       </c>
-      <c r="P16" s="46" t="s">
+      <c r="P16" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q16" s="49">
+      <c r="Q16" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R16" s="49" t="s">
+      <c r="R16" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S16" s="50">
+      <c r="S16" s="49">
         <v>45084.72278935185</v>
       </c>
-      <c r="T16" s="46">
+      <c r="T16" s="45">
         <v>32.907145</v>
       </c>
-      <c r="U16" s="46">
+      <c r="U16" s="45">
         <v>-117.747221</v>
       </c>
-      <c r="V16" s="50">
+      <c r="V16" s="49">
         <v>45085.253900462965</v>
       </c>
-      <c r="W16" s="46">
+      <c r="W16" s="45">
         <v>32.939883999999999</v>
       </c>
-      <c r="X16" s="46">
+      <c r="X16" s="45">
         <v>-117.83437499999999</v>
       </c>
-      <c r="Y16" s="51">
+      <c r="Y16" s="50">
         <f t="shared" si="2"/>
         <v>12.746666666760575</v>
       </c>
-      <c r="Z16" s="52">
+      <c r="Z16" s="51">
         <v>0.52916666666666667</v>
       </c>
-      <c r="AA16" s="52">
+      <c r="AA16" s="51">
         <v>0.12291666666666667</v>
       </c>
-      <c r="AB16" s="46">
+      <c r="AB16" s="45">
         <v>250</v>
       </c>
-      <c r="AC16" s="46"/>
-      <c r="AD16" s="46"/>
-    </row>
-    <row r="17" spans="1:30" s="53" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="46">
+      <c r="AC16" s="45"/>
+      <c r="AD16" s="45"/>
+    </row>
+    <row r="17" spans="1:30" s="52" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="45">
         <v>11</v>
       </c>
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="45">
         <v>4</v>
       </c>
-      <c r="D17" s="46">
+      <c r="D17" s="45">
         <v>2</v>
       </c>
-      <c r="E17" s="47">
+      <c r="E17" s="46">
         <v>45084</v>
       </c>
-      <c r="F17" s="48"/>
+      <c r="F17" s="47"/>
       <c r="G17" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="47"/>
-      <c r="K17" s="48"/>
-      <c r="L17" s="48" t="s">
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="46"/>
+      <c r="K17" s="47"/>
+      <c r="L17" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="M17" s="46"/>
-      <c r="N17" s="46"/>
-      <c r="O17" s="46">
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
+      <c r="O17" s="45">
         <v>1</v>
       </c>
-      <c r="P17" s="46" t="s">
+      <c r="P17" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q17" s="49">
+      <c r="Q17" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R17" s="49" t="s">
+      <c r="R17" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="S17" s="54">
+      <c r="S17" s="53">
         <v>45085.26767361111</v>
       </c>
-      <c r="T17" s="55">
+      <c r="T17" s="54">
         <v>32.939607000000002</v>
       </c>
-      <c r="U17" s="55">
+      <c r="U17" s="54">
         <v>-117.834576</v>
       </c>
-      <c r="V17" s="54">
+      <c r="V17" s="53">
         <v>45085.753796296296</v>
       </c>
-      <c r="W17" s="55">
+      <c r="W17" s="54">
         <v>32.963126000000003</v>
       </c>
-      <c r="X17" s="55">
+      <c r="X17" s="54">
         <v>-117.875584</v>
       </c>
-      <c r="Y17" s="51">
+      <c r="Y17" s="50">
         <f t="shared" si="2"/>
         <v>11.666944444470573</v>
       </c>
-      <c r="Z17" s="52">
+      <c r="Z17" s="51">
         <v>0.52916666666666667</v>
       </c>
-      <c r="AA17" s="52">
+      <c r="AA17" s="51">
         <v>0.12291666666666667</v>
       </c>
-      <c r="AB17" s="46">
+      <c r="AB17" s="45">
         <v>250</v>
       </c>
-      <c r="AC17" s="46"/>
-      <c r="AD17" s="46"/>
+      <c r="AC17" s="45"/>
+      <c r="AD17" s="45"/>
     </row>
     <row r="18" spans="1:30" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="20">
@@ -3384,94 +3386,94 @@
       <c r="AC19" s="20"/>
       <c r="AD19" s="20"/>
     </row>
-    <row r="20" spans="1:30" s="57" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="46">
+    <row r="20" spans="1:30" s="56" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="45">
         <v>13</v>
       </c>
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="46">
+      <c r="C20" s="45">
         <v>6</v>
       </c>
-      <c r="D20" s="46">
+      <c r="D20" s="45">
         <v>1</v>
       </c>
-      <c r="E20" s="47">
+      <c r="E20" s="46">
         <v>45176</v>
       </c>
-      <c r="F20" s="48">
+      <c r="F20" s="47">
         <v>0.37708333333333338</v>
       </c>
       <c r="G20" s="41">
         <f>$E20+$F20+TIME(AC20,0,0)</f>
         <v>45176.668749999997</v>
       </c>
-      <c r="H20" s="46">
+      <c r="H20" s="45">
         <v>32.910367999999998</v>
       </c>
-      <c r="I20" s="46">
+      <c r="I20" s="45">
         <v>-117.737223</v>
       </c>
-      <c r="J20" s="47">
+      <c r="J20" s="46">
         <v>45180</v>
       </c>
-      <c r="K20" s="48">
+      <c r="K20" s="47">
         <v>0.25</v>
       </c>
-      <c r="L20" s="56">
+      <c r="L20" s="55">
         <f>$J20+$K20 +TIME($AC20,0,0)</f>
         <v>45180.541666666664</v>
       </c>
-      <c r="M20" s="46"/>
-      <c r="N20" s="46"/>
-      <c r="O20" s="46">
+      <c r="M20" s="45"/>
+      <c r="N20" s="45"/>
+      <c r="O20" s="45">
         <v>4</v>
       </c>
-      <c r="P20" s="46" t="s">
+      <c r="P20" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="49">
+      <c r="Q20" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R20" s="49" t="s">
+      <c r="R20" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="S20" s="54">
+      <c r="S20" s="53">
         <v>45176.681122685186</v>
       </c>
-      <c r="T20" s="55">
+      <c r="T20" s="54">
         <v>32.911997999999997</v>
       </c>
-      <c r="U20" s="55">
+      <c r="U20" s="54">
         <v>-117.736034</v>
       </c>
-      <c r="V20" s="54">
+      <c r="V20" s="53">
         <v>45180.389189814814</v>
       </c>
-      <c r="W20" s="55">
+      <c r="W20" s="54">
         <v>32.880761</v>
       </c>
-      <c r="X20" s="55">
+      <c r="X20" s="54">
         <v>-117.434878</v>
       </c>
-      <c r="Y20" s="51">
+      <c r="Y20" s="50">
         <f t="shared" si="2"/>
         <v>88.993611111072823</v>
       </c>
-      <c r="Z20" s="52">
+      <c r="Z20" s="51">
         <v>0.57361111111111118</v>
       </c>
-      <c r="AA20" s="52">
+      <c r="AA20" s="51">
         <v>6.2847222222222221E-2</v>
       </c>
-      <c r="AB20" s="46">
+      <c r="AB20" s="45">
         <v>250</v>
       </c>
-      <c r="AC20" s="46">
+      <c r="AC20" s="45">
         <v>7</v>
       </c>
-      <c r="AD20" s="46"/>
+      <c r="AD20" s="45"/>
     </row>
     <row r="21" spans="1:30" s="31" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="20">
@@ -3568,193 +3570,193 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="46">
+    <row r="22" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="45">
         <v>15</v>
       </c>
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="46">
+      <c r="C22" s="45">
         <v>5</v>
       </c>
-      <c r="D22" s="46">
+      <c r="D22" s="45">
         <v>1</v>
       </c>
-      <c r="E22" s="47">
+      <c r="E22" s="46">
         <v>45203</v>
       </c>
-      <c r="F22" s="48">
+      <c r="F22" s="47">
         <v>0.29444444444444445</v>
       </c>
       <c r="G22" s="41">
         <f t="shared" si="3"/>
         <v>45203.461111111108</v>
       </c>
-      <c r="H22" s="46">
+      <c r="H22" s="45">
         <v>38.708799999999997</v>
       </c>
-      <c r="I22" s="46">
+      <c r="I22" s="45">
         <v>-64.031542999999999</v>
       </c>
-      <c r="J22" s="47">
+      <c r="J22" s="46">
         <v>45205</v>
       </c>
-      <c r="K22" s="48">
+      <c r="K22" s="47">
         <v>0.37847222222222227</v>
       </c>
-      <c r="L22" s="56">
+      <c r="L22" s="55">
         <f t="shared" si="4"/>
         <v>45205.545138888883</v>
       </c>
-      <c r="M22" s="46">
+      <c r="M22" s="45">
         <v>38.943779999999997</v>
       </c>
-      <c r="N22" s="46">
+      <c r="N22" s="45">
         <v>-64.196479999999994</v>
       </c>
-      <c r="O22" s="46">
+      <c r="O22" s="45">
         <v>3</v>
       </c>
-      <c r="P22" s="46" t="s">
+      <c r="P22" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q22" s="49">
+      <c r="Q22" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R22" s="49" t="s">
+      <c r="R22" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S22" s="50">
+      <c r="S22" s="49">
         <v>45203.535277777781</v>
       </c>
-      <c r="T22" s="55">
+      <c r="T22" s="54">
         <v>38.722087999999999</v>
       </c>
-      <c r="U22" s="55">
+      <c r="U22" s="54">
         <v>-64.021294999999995</v>
       </c>
-      <c r="V22" s="50">
+      <c r="V22" s="49">
         <v>45204.719074074077</v>
       </c>
-      <c r="W22" s="55">
+      <c r="W22" s="54">
         <v>38.866824999999999</v>
       </c>
-      <c r="X22" s="55">
+      <c r="X22" s="54">
         <v>-64.043930000000003</v>
       </c>
-      <c r="Y22" s="51">
+      <c r="Y22" s="50">
         <f t="shared" si="2"/>
         <v>28.411111111112405</v>
       </c>
-      <c r="Z22" s="52">
+      <c r="Z22" s="51">
         <v>0.42708333333333331</v>
       </c>
-      <c r="AA22" s="52">
+      <c r="AA22" s="51">
         <v>0.91180555555555554</v>
       </c>
-      <c r="AB22" s="46">
+      <c r="AB22" s="45">
         <v>300</v>
       </c>
-      <c r="AC22" s="46">
+      <c r="AC22" s="45">
         <v>4</v>
       </c>
-      <c r="AD22" s="46" t="s">
+      <c r="AD22" s="45" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="46">
+    <row r="23" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="45">
         <v>15</v>
       </c>
-      <c r="B23" s="46" t="s">
+      <c r="B23" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="46">
+      <c r="C23" s="45">
         <v>5</v>
       </c>
-      <c r="D23" s="46">
+      <c r="D23" s="45">
         <v>2</v>
       </c>
-      <c r="E23" s="47">
+      <c r="E23" s="46">
         <v>45203</v>
       </c>
-      <c r="F23" s="48">
+      <c r="F23" s="47">
         <v>0.29444444444444445</v>
       </c>
       <c r="G23" s="41">
         <f t="shared" si="3"/>
         <v>45203.461111111108</v>
       </c>
-      <c r="H23" s="46">
+      <c r="H23" s="45">
         <v>38.708799999999997</v>
       </c>
-      <c r="I23" s="46">
+      <c r="I23" s="45">
         <v>-64.031542999999999</v>
       </c>
-      <c r="J23" s="47">
+      <c r="J23" s="46">
         <v>45205</v>
       </c>
-      <c r="K23" s="48">
+      <c r="K23" s="47">
         <v>0.37847222222222227</v>
       </c>
-      <c r="L23" s="56">
+      <c r="L23" s="55">
         <f t="shared" si="4"/>
         <v>45205.545138888883</v>
       </c>
-      <c r="M23" s="46">
+      <c r="M23" s="45">
         <v>38.943779999999997</v>
       </c>
-      <c r="N23" s="46">
+      <c r="N23" s="45">
         <v>-64.196479999999994</v>
       </c>
-      <c r="O23" s="46">
+      <c r="O23" s="45">
         <v>3</v>
       </c>
-      <c r="P23" s="46" t="s">
+      <c r="P23" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q23" s="49">
+      <c r="Q23" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R23" s="49" t="s">
+      <c r="R23" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S23" s="54">
+      <c r="S23" s="53">
         <v>45204.812939814816</v>
       </c>
-      <c r="T23" s="55">
+      <c r="T23" s="54">
         <v>38.887227000000003</v>
       </c>
-      <c r="U23" s="55">
+      <c r="U23" s="54">
         <v>-64.073801000000003</v>
       </c>
-      <c r="V23" s="54">
+      <c r="V23" s="53">
         <v>45205.389224537037</v>
       </c>
-      <c r="W23" s="55">
+      <c r="W23" s="54">
         <v>38.930204000000003</v>
       </c>
-      <c r="X23" s="55">
+      <c r="X23" s="54">
         <v>-64.167721999999998</v>
       </c>
-      <c r="Y23" s="51">
+      <c r="Y23" s="50">
         <f t="shared" si="2"/>
         <v>13.830833333311602</v>
       </c>
-      <c r="Z23" s="52">
+      <c r="Z23" s="51">
         <v>0.42708333333333331</v>
       </c>
-      <c r="AA23" s="52">
+      <c r="AA23" s="51">
         <v>0.91180555555555554</v>
       </c>
-      <c r="AB23" s="46">
+      <c r="AB23" s="45">
         <v>300</v>
       </c>
-      <c r="AC23" s="46">
+      <c r="AC23" s="45">
         <v>4</v>
       </c>
-      <c r="AD23" s="46" t="s">
+      <c r="AD23" s="45" t="s">
         <v>49</v>
       </c>
     </row>
@@ -3944,284 +3946,284 @@
       </c>
       <c r="AD25" s="20"/>
     </row>
-    <row r="26" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="46">
+    <row r="26" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="45">
         <v>17</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="46">
+      <c r="C26" s="45">
         <v>6</v>
       </c>
-      <c r="D26" s="46">
+      <c r="D26" s="45">
         <v>1</v>
       </c>
-      <c r="E26" s="47">
+      <c r="E26" s="46">
         <v>45207</v>
       </c>
-      <c r="F26" s="48">
+      <c r="F26" s="47">
         <v>0.92152777777777783</v>
       </c>
       <c r="G26" s="41">
         <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H26" s="46">
+      <c r="H26" s="45">
         <v>38.767780000000002</v>
       </c>
-      <c r="I26" s="46">
+      <c r="I26" s="45">
         <v>-63.738374</v>
       </c>
-      <c r="J26" s="47">
+      <c r="J26" s="46">
         <v>45210</v>
       </c>
-      <c r="K26" s="48">
+      <c r="K26" s="47">
         <v>0.40625</v>
       </c>
-      <c r="L26" s="56">
+      <c r="L26" s="55">
         <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M26" s="57">
+      <c r="M26" s="56">
         <v>38.954067000000002</v>
       </c>
-      <c r="N26" s="46">
+      <c r="N26" s="45">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O26" s="46">
+      <c r="O26" s="45">
         <v>4</v>
       </c>
-      <c r="P26" s="46" t="s">
+      <c r="P26" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q26" s="49">
+      <c r="Q26" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R26" s="49" t="s">
+      <c r="R26" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="S26" s="54">
+      <c r="S26" s="53">
         <v>45208.132511574076</v>
       </c>
-      <c r="T26" s="58">
+      <c r="T26" s="57">
         <v>38.769841999999997</v>
       </c>
-      <c r="U26" s="58">
+      <c r="U26" s="57">
         <v>-63.7483</v>
       </c>
-      <c r="V26" s="54">
+      <c r="V26" s="53">
         <v>45208.63921296296</v>
       </c>
-      <c r="W26" s="58">
+      <c r="W26" s="57">
         <v>38.832385000000002</v>
       </c>
-      <c r="X26" s="58">
+      <c r="X26" s="57">
         <v>-63.796340000000001</v>
       </c>
-      <c r="Y26" s="51">
+      <c r="Y26" s="50">
         <f t="shared" si="2"/>
         <v>12.160833333211485</v>
       </c>
-      <c r="Z26" s="52">
+      <c r="Z26" s="51">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA26" s="52">
+      <c r="AA26" s="51">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB26" s="46">
+      <c r="AB26" s="45">
         <v>200</v>
       </c>
-      <c r="AC26" s="46">
+      <c r="AC26" s="45">
         <v>4</v>
       </c>
-      <c r="AD26" s="46"/>
-    </row>
-    <row r="27" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="46">
+      <c r="AD26" s="45"/>
+    </row>
+    <row r="27" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="45">
         <v>17</v>
       </c>
-      <c r="B27" s="46" t="s">
+      <c r="B27" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="46">
+      <c r="C27" s="45">
         <v>6</v>
       </c>
-      <c r="D27" s="46">
+      <c r="D27" s="45">
         <v>2</v>
       </c>
-      <c r="E27" s="47">
+      <c r="E27" s="46">
         <v>45207</v>
       </c>
-      <c r="F27" s="48">
+      <c r="F27" s="47">
         <v>0.92152777777777783</v>
       </c>
       <c r="G27" s="41">
         <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H27" s="46">
+      <c r="H27" s="45">
         <v>38.767780000000002</v>
       </c>
-      <c r="I27" s="46">
+      <c r="I27" s="45">
         <v>-63.738374</v>
       </c>
-      <c r="J27" s="47">
+      <c r="J27" s="46">
         <v>45210</v>
       </c>
-      <c r="K27" s="48">
+      <c r="K27" s="47">
         <v>0.40625</v>
       </c>
-      <c r="L27" s="56">
+      <c r="L27" s="55">
         <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M27" s="57">
+      <c r="M27" s="56">
         <v>38.954067000000002</v>
       </c>
-      <c r="N27" s="46">
+      <c r="N27" s="45">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O27" s="46">
+      <c r="O27" s="45">
         <v>4</v>
       </c>
-      <c r="P27" s="46" t="s">
+      <c r="P27" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q27" s="49">
+      <c r="Q27" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R27" s="49" t="s">
+      <c r="R27" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="S27" s="54">
+      <c r="S27" s="53">
         <v>45208.771828703706</v>
       </c>
-      <c r="T27" s="58">
+      <c r="T27" s="57">
         <v>38.857106999999999</v>
       </c>
-      <c r="U27" s="58">
+      <c r="U27" s="57">
         <v>-63.781923999999997</v>
       </c>
-      <c r="V27" s="54">
+      <c r="V27" s="53">
         <v>45209.656574074077</v>
       </c>
-      <c r="W27" s="58">
+      <c r="W27" s="57">
         <v>38.923247000000003</v>
       </c>
-      <c r="X27" s="58">
+      <c r="X27" s="57">
         <v>-63.812421999999998</v>
       </c>
-      <c r="Y27" s="51">
+      <c r="Y27" s="50">
         <f t="shared" si="2"/>
         <v>21.233888888906222</v>
       </c>
-      <c r="Z27" s="52">
+      <c r="Z27" s="51">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA27" s="52">
+      <c r="AA27" s="51">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB27" s="46">
+      <c r="AB27" s="45">
         <v>300</v>
       </c>
-      <c r="AC27" s="46">
+      <c r="AC27" s="45">
         <v>4</v>
       </c>
-      <c r="AD27" s="46"/>
-    </row>
-    <row r="28" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="46">
+      <c r="AD27" s="45"/>
+    </row>
+    <row r="28" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="45">
         <v>17</v>
       </c>
-      <c r="B28" s="46" t="s">
+      <c r="B28" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="46">
+      <c r="C28" s="45">
         <v>6</v>
       </c>
-      <c r="D28" s="46">
+      <c r="D28" s="45">
         <v>3</v>
       </c>
-      <c r="E28" s="47">
+      <c r="E28" s="46">
         <v>45207</v>
       </c>
-      <c r="F28" s="48">
+      <c r="F28" s="47">
         <v>0.92152777777777783</v>
       </c>
       <c r="G28" s="41">
         <f t="shared" si="3"/>
         <v>45208.088194444441</v>
       </c>
-      <c r="H28" s="46">
+      <c r="H28" s="45">
         <v>38.767780000000002</v>
       </c>
-      <c r="I28" s="46">
+      <c r="I28" s="45">
         <v>-63.738374</v>
       </c>
-      <c r="J28" s="47">
+      <c r="J28" s="46">
         <v>45210</v>
       </c>
-      <c r="K28" s="48">
+      <c r="K28" s="47">
         <v>0.40625</v>
       </c>
-      <c r="L28" s="56">
+      <c r="L28" s="55">
         <f t="shared" si="4"/>
         <v>45210.572916666664</v>
       </c>
-      <c r="M28" s="57">
+      <c r="M28" s="56">
         <v>38.954067000000002</v>
       </c>
-      <c r="N28" s="46">
+      <c r="N28" s="45">
         <v>-63.862921999999998</v>
       </c>
-      <c r="O28" s="46">
+      <c r="O28" s="45">
         <v>4</v>
       </c>
-      <c r="P28" s="46" t="s">
+      <c r="P28" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q28" s="49">
+      <c r="Q28" s="48">
         <v>300434066480130</v>
       </c>
-      <c r="R28" s="49" t="s">
+      <c r="R28" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="S28" s="54">
+      <c r="S28" s="53">
         <v>45209.750567129631</v>
       </c>
-      <c r="T28" s="58">
+      <c r="T28" s="57">
         <v>38.923658000000003</v>
       </c>
-      <c r="U28" s="58">
+      <c r="U28" s="57">
         <v>-63.819659000000001</v>
       </c>
-      <c r="V28" s="54">
+      <c r="V28" s="53">
         <v>45210.542002314818</v>
       </c>
-      <c r="W28" s="58">
+      <c r="W28" s="57">
         <v>38.940576999999998</v>
       </c>
-      <c r="X28" s="58">
+      <c r="X28" s="57">
         <v>-63.867663</v>
       </c>
-      <c r="Y28" s="51">
+      <c r="Y28" s="50">
         <f t="shared" si="2"/>
         <v>18.994444444484543</v>
       </c>
-      <c r="Z28" s="52">
+      <c r="Z28" s="51">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA28" s="52">
+      <c r="AA28" s="51">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB28" s="46">
+      <c r="AB28" s="45">
         <v>200</v>
       </c>
-      <c r="AC28" s="46">
+      <c r="AC28" s="45">
         <v>4</v>
       </c>
-      <c r="AD28" s="46"/>
+      <c r="AD28" s="45"/>
     </row>
     <row r="29" spans="1:30" s="31" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20">
@@ -4411,98 +4413,98 @@
       </c>
       <c r="AD30" s="20"/>
     </row>
-    <row r="31" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="46">
+    <row r="31" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="45">
         <v>19</v>
       </c>
-      <c r="B31" s="46" t="s">
+      <c r="B31" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="46">
+      <c r="C31" s="45">
         <v>5</v>
       </c>
-      <c r="D31" s="46">
+      <c r="D31" s="45">
         <v>1</v>
       </c>
-      <c r="E31" s="47">
+      <c r="E31" s="46">
         <v>45208</v>
       </c>
-      <c r="F31" s="48">
+      <c r="F31" s="47">
         <v>0.59722222222222221</v>
       </c>
       <c r="G31" s="41">
         <f t="shared" si="3"/>
         <v>45208.763888888883</v>
       </c>
-      <c r="H31" s="46">
+      <c r="H31" s="45">
         <v>38.826842999999997</v>
       </c>
-      <c r="I31" s="46">
+      <c r="I31" s="45">
         <v>-63.845635000000001</v>
       </c>
-      <c r="J31" s="47">
+      <c r="J31" s="46">
         <v>45209</v>
       </c>
-      <c r="K31" s="48">
+      <c r="K31" s="47">
         <v>0.36805555555555558</v>
       </c>
-      <c r="L31" s="56">
+      <c r="L31" s="55">
         <f t="shared" si="4"/>
         <v>45209.534722222219</v>
       </c>
-      <c r="M31" s="46">
+      <c r="M31" s="45">
         <v>38.862192</v>
       </c>
-      <c r="N31" s="46">
+      <c r="N31" s="45">
         <v>-63.908256999999999</v>
       </c>
-      <c r="O31" s="46">
+      <c r="O31" s="45">
         <v>3</v>
       </c>
-      <c r="P31" s="46" t="s">
+      <c r="P31" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q31" s="49">
+      <c r="Q31" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R31" s="49" t="s">
+      <c r="R31" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S31" s="54">
+      <c r="S31" s="53">
         <v>45208.77138888889</v>
       </c>
-      <c r="T31" s="58">
+      <c r="T31" s="57">
         <v>38.827702000000002</v>
       </c>
-      <c r="U31" s="58">
+      <c r="U31" s="57">
         <v>-63.844456999999998</v>
       </c>
-      <c r="V31" s="50">
+      <c r="V31" s="49">
         <v>45209.26421296296</v>
       </c>
-      <c r="W31" s="58">
+      <c r="W31" s="57">
         <v>38.862524999999998</v>
       </c>
-      <c r="X31" s="58">
+      <c r="X31" s="57">
         <v>-63.894246000000003</v>
       </c>
-      <c r="Y31" s="51">
+      <c r="Y31" s="50">
         <f t="shared" si="2"/>
         <v>11.827777777682059</v>
       </c>
-      <c r="Z31" s="52">
+      <c r="Z31" s="51">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA31" s="52">
+      <c r="AA31" s="51">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB31" s="46">
+      <c r="AB31" s="45">
         <v>100</v>
       </c>
-      <c r="AC31" s="46">
+      <c r="AC31" s="45">
         <v>4</v>
       </c>
-      <c r="AD31" s="46" t="s">
+      <c r="AD31" s="45" t="s">
         <v>47</v>
       </c>
     </row>
@@ -4694,98 +4696,98 @@
       </c>
       <c r="AD33" s="20"/>
     </row>
-    <row r="34" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="46">
+    <row r="34" spans="1:30" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="45">
         <v>21</v>
       </c>
-      <c r="B34" s="46" t="s">
+      <c r="B34" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="46">
+      <c r="C34" s="45">
         <v>4</v>
       </c>
-      <c r="D34" s="46">
+      <c r="D34" s="45">
         <v>1</v>
       </c>
-      <c r="E34" s="47">
+      <c r="E34" s="46">
         <v>45211</v>
       </c>
-      <c r="F34" s="48">
+      <c r="F34" s="47">
         <v>0.60416666666666663</v>
       </c>
       <c r="G34" s="41">
         <f t="shared" si="3"/>
         <v>45211.770833333328</v>
       </c>
-      <c r="H34" s="46">
+      <c r="H34" s="45">
         <v>38.834505</v>
       </c>
-      <c r="I34" s="46">
+      <c r="I34" s="45">
         <v>-63.75074</v>
       </c>
-      <c r="J34" s="47">
+      <c r="J34" s="46">
         <v>45212</v>
       </c>
-      <c r="K34" s="48">
+      <c r="K34" s="47">
         <v>0.54166666666666663</v>
       </c>
-      <c r="L34" s="56">
+      <c r="L34" s="55">
         <f t="shared" si="4"/>
         <v>45212.708333333328</v>
       </c>
-      <c r="M34" s="46">
+      <c r="M34" s="45">
         <v>38.856884999999998</v>
       </c>
-      <c r="N34" s="46">
+      <c r="N34" s="45">
         <v>-63.746738999999998</v>
       </c>
-      <c r="O34" s="46">
+      <c r="O34" s="45">
         <v>1</v>
       </c>
-      <c r="P34" s="46" t="s">
+      <c r="P34" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q34" s="49">
+      <c r="Q34" s="48">
         <v>300434066489180</v>
       </c>
-      <c r="R34" s="49" t="s">
+      <c r="R34" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="S34" s="54">
+      <c r="S34" s="53">
         <v>45211.834328703706</v>
       </c>
-      <c r="T34" s="58">
+      <c r="T34" s="57">
         <v>38.831561999999998</v>
       </c>
-      <c r="U34" s="58">
+      <c r="U34" s="57">
         <v>-63.740231999999999</v>
       </c>
-      <c r="V34" s="59">
+      <c r="V34" s="58">
         <v>45212.541990740741</v>
       </c>
-      <c r="W34" s="58">
+      <c r="W34" s="57">
         <v>38.884850999999998</v>
       </c>
-      <c r="X34" s="58">
+      <c r="X34" s="57">
         <v>-63.740850999999999</v>
       </c>
-      <c r="Y34" s="51">
+      <c r="Y34" s="50">
         <f t="shared" si="2"/>
         <v>16.983888888848014</v>
       </c>
-      <c r="Z34" s="52">
+      <c r="Z34" s="51">
         <v>0.42708333333333298</v>
       </c>
-      <c r="AA34" s="52">
+      <c r="AA34" s="51">
         <v>0.91180555555555598</v>
       </c>
-      <c r="AB34" s="46">
+      <c r="AB34" s="45">
         <v>125</v>
       </c>
-      <c r="AC34" s="46">
+      <c r="AC34" s="45">
         <v>4</v>
       </c>
-      <c r="AD34" s="46" t="s">
+      <c r="AD34" s="45" t="s">
         <v>52</v>
       </c>
     </row>
@@ -4884,258 +4886,258 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="46">
+    <row r="36" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="45">
         <v>23</v>
       </c>
-      <c r="B36" s="46" t="s">
+      <c r="B36" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="46">
+      <c r="C36" s="45">
         <v>5</v>
       </c>
-      <c r="D36" s="46">
+      <c r="D36" s="45">
         <v>1</v>
       </c>
-      <c r="E36" s="47">
+      <c r="E36" s="46">
         <v>45317</v>
       </c>
-      <c r="F36" s="48">
+      <c r="F36" s="47">
         <v>0.50972222222222219</v>
       </c>
       <c r="G36" s="41">
         <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H36" s="46"/>
-      <c r="I36" s="46"/>
-      <c r="J36" s="47">
+      <c r="H36" s="45"/>
+      <c r="I36" s="45"/>
+      <c r="J36" s="46">
         <v>45320</v>
       </c>
-      <c r="K36" s="48">
+      <c r="K36" s="47">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L36" s="56">
+      <c r="L36" s="55">
         <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
-      <c r="M36" s="46"/>
-      <c r="N36" s="46"/>
-      <c r="O36" s="46">
+      <c r="M36" s="45"/>
+      <c r="N36" s="45"/>
+      <c r="O36" s="45">
         <v>3</v>
       </c>
-      <c r="P36" s="46" t="s">
+      <c r="P36" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q36" s="49">
+      <c r="Q36" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R36" s="49" t="s">
+      <c r="R36" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S36" s="50">
+      <c r="S36" s="49">
         <v>45317.875324074077</v>
       </c>
-      <c r="T36" s="70">
+      <c r="T36" s="69">
         <v>32.909129</v>
       </c>
-      <c r="U36" s="70">
+      <c r="U36" s="69">
         <v>-117.680663</v>
       </c>
-      <c r="V36" s="50">
+      <c r="V36" s="49">
         <v>45318.878796296296</v>
       </c>
-      <c r="W36" s="46">
+      <c r="W36" s="45">
         <v>32.999972</v>
       </c>
-      <c r="X36" s="46">
+      <c r="X36" s="45">
         <v>-117.66408699999999</v>
       </c>
-      <c r="Y36" s="51">
+      <c r="Y36" s="50">
         <f t="shared" si="2"/>
         <v>24.083333333255723</v>
       </c>
-      <c r="Z36" s="52">
+      <c r="Z36" s="51">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA36" s="52">
+      <c r="AA36" s="51">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB36" s="46"/>
-      <c r="AC36" s="46">
+      <c r="AB36" s="45"/>
+      <c r="AC36" s="45">
         <v>8</v>
       </c>
-      <c r="AD36" s="46" t="s">
+      <c r="AD36" s="45" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="46">
+    <row r="37" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="45">
         <v>23</v>
       </c>
-      <c r="B37" s="46" t="s">
+      <c r="B37" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="46">
+      <c r="C37" s="45">
         <v>5</v>
       </c>
-      <c r="D37" s="46">
+      <c r="D37" s="45">
         <v>2</v>
       </c>
-      <c r="E37" s="47">
+      <c r="E37" s="46">
         <v>45317</v>
       </c>
-      <c r="F37" s="48">
+      <c r="F37" s="47">
         <v>0.50972222222222219</v>
       </c>
       <c r="G37" s="41">
         <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H37" s="46"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="47">
+      <c r="H37" s="45"/>
+      <c r="I37" s="45"/>
+      <c r="J37" s="46">
         <v>45320</v>
       </c>
-      <c r="K37" s="48">
+      <c r="K37" s="47">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L37" s="56">
+      <c r="L37" s="55">
         <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
-      <c r="M37" s="46"/>
-      <c r="N37" s="46"/>
-      <c r="O37" s="46">
+      <c r="M37" s="45"/>
+      <c r="N37" s="45"/>
+      <c r="O37" s="45">
         <v>3</v>
       </c>
-      <c r="P37" s="46" t="s">
+      <c r="P37" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q37" s="49">
+      <c r="Q37" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R37" s="49" t="s">
+      <c r="R37" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S37" s="50">
+      <c r="S37" s="49">
         <v>45318.931122685186</v>
       </c>
-      <c r="T37" s="70">
+      <c r="T37" s="69">
         <v>33.001423000000003</v>
       </c>
-      <c r="U37" s="70">
+      <c r="U37" s="69">
         <v>-117.65347800000001</v>
       </c>
-      <c r="V37" s="50">
+      <c r="V37" s="49">
         <v>45319.878796296296</v>
       </c>
-      <c r="W37" s="46">
+      <c r="W37" s="45">
         <v>33.117448000000003</v>
       </c>
-      <c r="X37" s="46">
+      <c r="X37" s="45">
         <v>-117.6035</v>
       </c>
-      <c r="Y37" s="51">
+      <c r="Y37" s="50">
         <f t="shared" si="2"/>
         <v>22.744166666641831</v>
       </c>
-      <c r="Z37" s="52">
+      <c r="Z37" s="51">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA37" s="52">
+      <c r="AA37" s="51">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB37" s="46"/>
-      <c r="AC37" s="46">
+      <c r="AB37" s="45"/>
+      <c r="AC37" s="45">
         <v>8</v>
       </c>
-      <c r="AD37" s="46" t="s">
+      <c r="AD37" s="45" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="46">
+    <row r="38" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="45">
         <v>23</v>
       </c>
-      <c r="B38" s="46" t="s">
+      <c r="B38" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="C38" s="46">
+      <c r="C38" s="45">
         <v>5</v>
       </c>
-      <c r="D38" s="46">
+      <c r="D38" s="45">
         <v>3</v>
       </c>
-      <c r="E38" s="47">
+      <c r="E38" s="46">
         <v>45317</v>
       </c>
-      <c r="F38" s="48">
+      <c r="F38" s="47">
         <v>0.50972222222222219</v>
       </c>
       <c r="G38" s="41">
         <f t="shared" si="3"/>
         <v>45317.843055555561</v>
       </c>
-      <c r="H38" s="46"/>
-      <c r="I38" s="46"/>
-      <c r="J38" s="47">
+      <c r="H38" s="45"/>
+      <c r="I38" s="45"/>
+      <c r="J38" s="46">
         <v>45320</v>
       </c>
-      <c r="K38" s="48">
+      <c r="K38" s="47">
         <v>0.57291666666666663</v>
       </c>
-      <c r="L38" s="56">
+      <c r="L38" s="55">
         <f t="shared" si="4"/>
         <v>45320.90625</v>
       </c>
-      <c r="M38" s="46"/>
-      <c r="N38" s="46"/>
-      <c r="O38" s="46">
+      <c r="M38" s="45"/>
+      <c r="N38" s="45"/>
+      <c r="O38" s="45">
         <v>3</v>
       </c>
-      <c r="P38" s="46" t="s">
+      <c r="P38" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q38" s="49">
+      <c r="Q38" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R38" s="49" t="s">
+      <c r="R38" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S38" s="50">
+      <c r="S38" s="49">
         <v>45319.910034722219</v>
       </c>
-      <c r="T38" s="71">
+      <c r="T38" s="70">
         <v>33.123451000000003</v>
       </c>
-      <c r="U38" s="71">
+      <c r="U38" s="70">
         <v>-117.600043</v>
       </c>
-      <c r="V38" s="50">
+      <c r="V38" s="49">
         <v>45320.89980324074</v>
       </c>
-      <c r="W38" s="71">
+      <c r="W38" s="70">
         <v>33.200189999999999</v>
       </c>
-      <c r="X38" s="71">
+      <c r="X38" s="70">
         <v>-117.597759</v>
       </c>
-      <c r="Y38" s="51">
+      <c r="Y38" s="50">
         <f t="shared" ref="Y38" si="5">(V38-S38)*1440/60</f>
         <v>23.754444444493856</v>
       </c>
-      <c r="Z38" s="52">
+      <c r="Z38" s="51">
         <v>0.6166666666666667</v>
       </c>
-      <c r="AA38" s="52">
+      <c r="AA38" s="51">
         <v>5.2777777777777778E-2</v>
       </c>
-      <c r="AB38" s="46"/>
-      <c r="AC38" s="46">
+      <c r="AB38" s="45"/>
+      <c r="AC38" s="45">
         <v>8</v>
       </c>
-      <c r="AD38" s="46" t="s">
+      <c r="AD38" s="45" t="s">
         <v>97</v>
       </c>
     </row>
@@ -5191,19 +5193,19 @@
       <c r="S39" s="28">
         <v>45317.993379629632</v>
       </c>
-      <c r="T39" s="72">
+      <c r="T39" s="71">
         <v>32.907333000000001</v>
       </c>
-      <c r="U39" s="72">
+      <c r="U39" s="71">
         <v>-117.67442</v>
       </c>
       <c r="V39" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="W39" s="72">
+      <c r="W39" s="71">
         <v>33.012383</v>
       </c>
-      <c r="X39" s="72">
+      <c r="X39" s="71">
         <v>-117.66186500000001</v>
       </c>
       <c r="Y39" s="25">
@@ -5276,19 +5278,19 @@
       <c r="S40" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="T40" s="72">
+      <c r="T40" s="71">
         <v>33.012383</v>
       </c>
-      <c r="U40" s="72">
+      <c r="U40" s="71">
         <v>-117.66186500000001</v>
       </c>
       <c r="V40" s="28">
         <v>45320.848263888889</v>
       </c>
-      <c r="W40" s="72">
+      <c r="W40" s="71">
         <v>33.115271</v>
       </c>
-      <c r="X40" s="72">
+      <c r="X40" s="71">
         <v>-117.89773700000001</v>
       </c>
       <c r="Y40" s="25">
@@ -5309,536 +5311,536 @@
         <v>98</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="46">
+    <row r="41" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="45">
         <v>25</v>
       </c>
-      <c r="B41" s="46" t="s">
+      <c r="B41" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="46">
+      <c r="C41" s="45">
         <v>5</v>
       </c>
-      <c r="D41" s="46">
+      <c r="D41" s="45">
         <v>1</v>
       </c>
-      <c r="E41" s="47">
+      <c r="E41" s="46">
         <v>45425</v>
       </c>
-      <c r="F41" s="48"/>
+      <c r="F41" s="47"/>
       <c r="G41" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="H41" s="46"/>
-      <c r="I41" s="46"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="48"/>
-      <c r="L41" s="56" t="s">
+      <c r="H41" s="45"/>
+      <c r="I41" s="45"/>
+      <c r="J41" s="46"/>
+      <c r="K41" s="47"/>
+      <c r="L41" s="55" t="s">
         <v>126</v>
       </c>
-      <c r="M41" s="46"/>
-      <c r="N41" s="46"/>
-      <c r="O41" s="46">
+      <c r="M41" s="45"/>
+      <c r="N41" s="45"/>
+      <c r="O41" s="45">
         <v>3</v>
       </c>
-      <c r="P41" s="46" t="s">
+      <c r="P41" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q41" s="49">
+      <c r="Q41" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R41" s="49" t="s">
+      <c r="R41" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S41" s="54"/>
-      <c r="T41" s="71"/>
-      <c r="U41" s="71"/>
-      <c r="V41" s="54"/>
-      <c r="W41" s="71"/>
-      <c r="X41" s="71"/>
-      <c r="Y41" s="51"/>
-      <c r="Z41" s="52"/>
-      <c r="AA41" s="52"/>
-      <c r="AB41" s="46"/>
-      <c r="AC41" s="46"/>
-      <c r="AD41" s="46"/>
-    </row>
-    <row r="42" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="68">
+      <c r="S41" s="53"/>
+      <c r="T41" s="70"/>
+      <c r="U41" s="70"/>
+      <c r="V41" s="53"/>
+      <c r="W41" s="70"/>
+      <c r="X41" s="70"/>
+      <c r="Y41" s="50"/>
+      <c r="Z41" s="51"/>
+      <c r="AA41" s="51"/>
+      <c r="AB41" s="45"/>
+      <c r="AC41" s="45"/>
+      <c r="AD41" s="45"/>
+    </row>
+    <row r="42" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="67">
         <v>26</v>
       </c>
-      <c r="B42" s="68" t="s">
+      <c r="B42" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="68">
+      <c r="C42" s="67">
         <v>5</v>
       </c>
-      <c r="D42" s="68">
+      <c r="D42" s="67">
         <v>1</v>
       </c>
-      <c r="E42" s="78">
+      <c r="E42" s="77">
         <v>45429</v>
       </c>
-      <c r="F42" s="79">
+      <c r="F42" s="78">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G42" s="79" t="s">
+      <c r="G42" s="78" t="s">
         <v>116</v>
       </c>
-      <c r="H42" s="68"/>
-      <c r="I42" s="68"/>
-      <c r="J42" s="78">
+      <c r="H42" s="67"/>
+      <c r="I42" s="67"/>
+      <c r="J42" s="77">
         <v>45432</v>
       </c>
-      <c r="K42" s="79">
+      <c r="K42" s="78">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L42" s="79" t="s">
+      <c r="L42" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="M42" s="68"/>
-      <c r="N42" s="68"/>
-      <c r="O42" s="68">
+      <c r="M42" s="67"/>
+      <c r="N42" s="67"/>
+      <c r="O42" s="67">
         <v>3</v>
       </c>
-      <c r="P42" s="68" t="s">
+      <c r="P42" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="Q42" s="67">
+      <c r="Q42" s="66">
         <v>300434066482170</v>
       </c>
-      <c r="R42" s="67" t="s">
+      <c r="R42" s="66" t="s">
         <v>115</v>
       </c>
       <c r="S42" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="T42" s="72">
+      <c r="T42" s="71">
         <v>32.917650000000002</v>
       </c>
-      <c r="U42" s="72">
+      <c r="U42" s="71">
         <v>-117.794504</v>
       </c>
       <c r="V42" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="W42" s="72" t="s">
+      <c r="W42" s="71" t="s">
         <v>120</v>
       </c>
-      <c r="X42" s="72" t="s">
+      <c r="X42" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="Y42" s="83"/>
-      <c r="Z42" s="84">
+      <c r="Y42" s="82"/>
+      <c r="Z42" s="83">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA42" s="84">
+      <c r="AA42" s="83">
         <v>0.1125</v>
       </c>
-      <c r="AB42" s="68"/>
-      <c r="AC42" s="68">
+      <c r="AB42" s="67"/>
+      <c r="AC42" s="67">
         <v>7</v>
       </c>
-      <c r="AD42" s="68"/>
-    </row>
-    <row r="43" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="68">
+      <c r="AD42" s="67"/>
+    </row>
+    <row r="43" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="67">
         <v>26</v>
       </c>
-      <c r="B43" s="68" t="s">
+      <c r="B43" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="68">
+      <c r="C43" s="67">
         <v>5</v>
       </c>
-      <c r="D43" s="68">
+      <c r="D43" s="67">
         <v>2</v>
       </c>
-      <c r="E43" s="78">
+      <c r="E43" s="77">
         <v>45429</v>
       </c>
-      <c r="F43" s="79">
+      <c r="F43" s="78">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G43" s="79" t="s">
+      <c r="G43" s="78" t="s">
         <v>116</v>
       </c>
-      <c r="H43" s="68"/>
-      <c r="I43" s="68"/>
-      <c r="J43" s="78">
+      <c r="H43" s="67"/>
+      <c r="I43" s="67"/>
+      <c r="J43" s="77">
         <v>45432</v>
       </c>
-      <c r="K43" s="79">
+      <c r="K43" s="78">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L43" s="79" t="s">
+      <c r="L43" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="M43" s="68"/>
-      <c r="N43" s="68"/>
-      <c r="O43" s="68">
+      <c r="M43" s="67"/>
+      <c r="N43" s="67"/>
+      <c r="O43" s="67">
         <v>3</v>
       </c>
-      <c r="P43" s="68" t="s">
+      <c r="P43" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="Q43" s="67">
+      <c r="Q43" s="66">
         <v>300434066482170</v>
       </c>
-      <c r="R43" s="67" t="s">
+      <c r="R43" s="66" t="s">
         <v>115</v>
       </c>
       <c r="S43" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="T43" s="72">
+      <c r="T43" s="71">
         <v>32.998700999999997</v>
       </c>
-      <c r="U43" s="72">
+      <c r="U43" s="71">
         <v>-117.874388</v>
       </c>
       <c r="V43" s="28" t="s">
         <v>123</v>
       </c>
-      <c r="W43" s="72">
+      <c r="W43" s="71">
         <v>33.012540000000001</v>
       </c>
-      <c r="X43" s="72">
+      <c r="X43" s="71">
         <v>-117.890097</v>
       </c>
-      <c r="Y43" s="83"/>
-      <c r="Z43" s="84">
+      <c r="Y43" s="82"/>
+      <c r="Z43" s="83">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA43" s="84">
+      <c r="AA43" s="83">
         <v>0.1125</v>
       </c>
-      <c r="AB43" s="68"/>
-      <c r="AC43" s="68">
+      <c r="AB43" s="67"/>
+      <c r="AC43" s="67">
         <v>7</v>
       </c>
-      <c r="AD43" s="68"/>
-    </row>
-    <row r="44" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="46">
+      <c r="AD43" s="67"/>
+    </row>
+    <row r="44" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="45">
         <v>27</v>
       </c>
-      <c r="B44" s="46" t="s">
+      <c r="B44" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="C44" s="46">
+      <c r="C44" s="45">
         <v>5</v>
       </c>
-      <c r="D44" s="46">
+      <c r="D44" s="45">
         <v>1</v>
       </c>
-      <c r="E44" s="73">
+      <c r="E44" s="72">
         <v>45462</v>
       </c>
-      <c r="F44" s="74">
+      <c r="F44" s="73">
         <v>0.625</v>
       </c>
       <c r="G44" s="41">
         <f>$E44+$F44+TIME(AC44,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H44" s="46"/>
-      <c r="I44" s="46"/>
-      <c r="J44" s="47"/>
-      <c r="K44" s="48"/>
-      <c r="M44" s="71"/>
-      <c r="N44" s="71"/>
-      <c r="O44" s="46">
+      <c r="H44" s="45"/>
+      <c r="I44" s="45"/>
+      <c r="J44" s="46"/>
+      <c r="K44" s="47"/>
+      <c r="M44" s="70"/>
+      <c r="N44" s="70"/>
+      <c r="O44" s="45">
         <v>3</v>
       </c>
-      <c r="P44" s="46" t="s">
+      <c r="P44" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="Q44" s="49">
+      <c r="Q44" s="48">
         <v>300434066482170</v>
       </c>
-      <c r="R44" s="49" t="s">
+      <c r="R44" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="S44" s="54">
+      <c r="S44" s="53">
         <v>45462.860289351855</v>
       </c>
-      <c r="T44" s="71">
+      <c r="T44" s="70">
         <v>38.313133999999998</v>
       </c>
-      <c r="U44" s="71">
+      <c r="U44" s="70">
         <v>-63.006925000000003</v>
       </c>
-      <c r="V44" s="50"/>
-      <c r="W44" s="46"/>
-      <c r="X44" s="46"/>
-      <c r="Y44" s="51"/>
-      <c r="Z44" s="52"/>
-      <c r="AA44" s="52"/>
-      <c r="AB44" s="46"/>
-      <c r="AC44" s="46">
+      <c r="V44" s="49"/>
+      <c r="W44" s="45"/>
+      <c r="X44" s="45"/>
+      <c r="Y44" s="50"/>
+      <c r="Z44" s="51"/>
+      <c r="AA44" s="51"/>
+      <c r="AB44" s="45"/>
+      <c r="AC44" s="45">
         <v>4</v>
       </c>
-      <c r="AD44" s="46"/>
-    </row>
-    <row r="45" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="68">
+      <c r="AD44" s="45"/>
+    </row>
+    <row r="45" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="67">
         <v>28</v>
       </c>
-      <c r="B45" s="68" t="s">
+      <c r="B45" s="67" t="s">
         <v>124</v>
       </c>
-      <c r="C45" s="68">
+      <c r="C45" s="67">
         <v>6</v>
       </c>
-      <c r="D45" s="68">
+      <c r="D45" s="67">
         <v>1</v>
       </c>
-      <c r="E45" s="76">
+      <c r="E45" s="75">
         <v>45462</v>
       </c>
-      <c r="F45" s="77">
+      <c r="F45" s="76">
         <v>0.625</v>
       </c>
-      <c r="G45" s="65">
+      <c r="G45" s="64">
         <f t="shared" ref="G45" si="8">$E45+$F45+TIME(AC45,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H45" s="68"/>
-      <c r="I45" s="68"/>
-      <c r="J45" s="78"/>
-      <c r="K45" s="79"/>
-      <c r="L45" s="66"/>
-      <c r="M45" s="80"/>
-      <c r="N45" s="80"/>
-      <c r="O45" s="68">
+      <c r="H45" s="67"/>
+      <c r="I45" s="67"/>
+      <c r="J45" s="77"/>
+      <c r="K45" s="78"/>
+      <c r="L45" s="65"/>
+      <c r="M45" s="79"/>
+      <c r="N45" s="79"/>
+      <c r="O45" s="67">
         <v>4</v>
       </c>
-      <c r="P45" s="68" t="s">
+      <c r="P45" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="Q45" s="67">
+      <c r="Q45" s="66">
         <v>300434066480130</v>
       </c>
-      <c r="R45" s="67" t="s">
+      <c r="R45" s="66" t="s">
         <v>44</v>
       </c>
       <c r="S45" s="28">
         <v>45462.830416666664</v>
       </c>
-      <c r="T45" s="94">
+      <c r="T45" s="91">
         <v>38.311219000000001</v>
       </c>
-      <c r="U45" s="94">
+      <c r="U45" s="91">
         <v>-63.003127999999997</v>
       </c>
       <c r="V45" s="28">
         <v>45462.83388888889</v>
       </c>
-      <c r="W45" s="94">
+      <c r="W45" s="91">
         <v>38.310768000000003</v>
       </c>
-      <c r="X45" s="94">
+      <c r="X45" s="91">
         <v>-63.002412999999997</v>
       </c>
-      <c r="Y45" s="83"/>
-      <c r="Z45" s="84"/>
-      <c r="AA45" s="84"/>
-      <c r="AB45" s="68"/>
-      <c r="AC45" s="68">
+      <c r="Y45" s="82"/>
+      <c r="Z45" s="83"/>
+      <c r="AA45" s="83"/>
+      <c r="AB45" s="67"/>
+      <c r="AC45" s="67">
         <v>4</v>
       </c>
-      <c r="AD45" s="68"/>
-    </row>
-    <row r="46" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="68">
+      <c r="AD45" s="67"/>
+    </row>
+    <row r="46" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="67">
         <v>28</v>
       </c>
-      <c r="B46" s="68" t="s">
+      <c r="B46" s="67" t="s">
         <v>124</v>
       </c>
-      <c r="C46" s="68">
+      <c r="C46" s="67">
         <v>6</v>
       </c>
-      <c r="D46" s="68">
+      <c r="D46" s="67">
         <v>2</v>
       </c>
-      <c r="E46" s="76">
+      <c r="E46" s="75">
         <v>45462</v>
       </c>
-      <c r="F46" s="77">
+      <c r="F46" s="76">
         <v>0.625</v>
       </c>
-      <c r="G46" s="65">
+      <c r="G46" s="64">
         <f t="shared" ref="G46" si="9">$E46+$F46+TIME(AC46,0,0)</f>
         <v>45462.625</v>
       </c>
-      <c r="H46" s="68"/>
-      <c r="I46" s="68"/>
-      <c r="J46" s="78"/>
-      <c r="K46" s="79"/>
-      <c r="L46" s="66"/>
-      <c r="M46" s="80"/>
-      <c r="N46" s="80"/>
-      <c r="O46" s="68">
+      <c r="H46" s="67"/>
+      <c r="I46" s="67"/>
+      <c r="J46" s="77"/>
+      <c r="K46" s="78"/>
+      <c r="L46" s="65"/>
+      <c r="M46" s="79"/>
+      <c r="N46" s="79"/>
+      <c r="O46" s="67">
         <v>4</v>
       </c>
-      <c r="P46" s="68" t="s">
+      <c r="P46" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="Q46" s="67">
+      <c r="Q46" s="66">
         <v>300434066480130</v>
       </c>
-      <c r="R46" s="67" t="s">
+      <c r="R46" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="S46" s="81">
+      <c r="S46" s="80">
         <v>45465.271736111114</v>
       </c>
-      <c r="T46" s="94">
+      <c r="T46" s="91">
         <v>38.415380999999996</v>
       </c>
-      <c r="U46" s="94">
+      <c r="U46" s="91">
         <v>-62.463433000000002</v>
       </c>
       <c r="V46" s="28">
         <v>45466.125555555554</v>
       </c>
-      <c r="W46" s="94">
+      <c r="W46" s="91">
         <v>38.532255999999997</v>
       </c>
-      <c r="X46" s="94">
+      <c r="X46" s="91">
         <v>-62.362059000000002</v>
       </c>
-      <c r="Y46" s="83"/>
-      <c r="Z46" s="84"/>
-      <c r="AA46" s="84"/>
-      <c r="AB46" s="68"/>
-      <c r="AC46" s="68"/>
-      <c r="AD46" s="68" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="47" spans="1:30" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="46">
+      <c r="Y46" s="82"/>
+      <c r="Z46" s="83"/>
+      <c r="AA46" s="83"/>
+      <c r="AB46" s="67"/>
+      <c r="AC46" s="67"/>
+      <c r="AD46" s="67" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="47" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="45">
         <v>29</v>
       </c>
-      <c r="B47" s="46" t="s">
+      <c r="B47" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="C47" s="46">
+      <c r="C47" s="45">
         <v>4</v>
       </c>
-      <c r="D47" s="46">
+      <c r="D47" s="45">
         <v>1</v>
       </c>
-      <c r="E47" s="73">
+      <c r="E47" s="72">
         <v>45462</v>
       </c>
-      <c r="F47" s="74">
+      <c r="F47" s="73">
         <v>0.625</v>
       </c>
       <c r="G47" s="41">
         <f>$E47+$F47+TIME(AC47,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H47" s="46">
+      <c r="H47" s="45">
         <v>38.316051999999999</v>
       </c>
-      <c r="I47" s="46">
+      <c r="I47" s="45">
         <v>-63.012607000000003</v>
       </c>
-      <c r="J47" s="47">
+      <c r="J47" s="46">
         <v>45464</v>
       </c>
-      <c r="K47" s="48">
+      <c r="K47" s="47">
         <v>0.125</v>
       </c>
-      <c r="L47" s="56">
+      <c r="L47" s="55">
         <f t="shared" ref="L47" si="10">$J47+$K47 +TIME($AC47,0,0)</f>
         <v>45464.291666666664</v>
       </c>
-      <c r="M47" s="71">
+      <c r="M47" s="70">
         <v>38.309516000000002</v>
       </c>
-      <c r="N47" s="71">
+      <c r="N47" s="70">
         <v>-62.619463000000003</v>
       </c>
-      <c r="O47" s="46">
+      <c r="O47" s="45">
         <v>1</v>
       </c>
-      <c r="P47" s="46" t="s">
+      <c r="P47" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q47" s="75">
+      <c r="Q47" s="74">
         <v>300434066489180</v>
       </c>
-      <c r="R47" s="49" t="s">
+      <c r="R47" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="S47" s="54">
+      <c r="S47" s="53">
         <v>45462.84778935185</v>
       </c>
-      <c r="T47" s="71">
+      <c r="T47" s="70">
         <v>38.315800000000003</v>
       </c>
-      <c r="U47" s="71">
+      <c r="U47" s="70">
         <v>-63.012493999999997</v>
       </c>
-      <c r="V47" s="54">
+      <c r="V47" s="53">
         <v>45463.528101851851</v>
       </c>
-      <c r="W47" s="71">
+      <c r="W47" s="70">
         <v>38.311391</v>
       </c>
-      <c r="X47" s="71">
+      <c r="X47" s="70">
         <v>-62.918548000000001</v>
       </c>
-      <c r="Y47" s="51">
+      <c r="Y47" s="50">
         <f t="shared" ref="Y47" si="11">(V47-S47)*1440/60</f>
         <v>16.32750000001397</v>
       </c>
-      <c r="Z47" s="52"/>
-      <c r="AA47" s="52"/>
-      <c r="AB47" s="46"/>
-      <c r="AC47" s="46">
+      <c r="Z47" s="51"/>
+      <c r="AA47" s="51"/>
+      <c r="AB47" s="45"/>
+      <c r="AC47" s="45">
         <v>4</v>
       </c>
-      <c r="AD47" s="46" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="48" spans="1:30" s="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="68"/>
-      <c r="B48" s="68"/>
-      <c r="C48" s="68"/>
-      <c r="D48" s="68"/>
-      <c r="E48" s="86"/>
-      <c r="F48" s="87"/>
-      <c r="G48" s="87"/>
-      <c r="H48" s="81"/>
-      <c r="I48" s="87"/>
-      <c r="J48" s="88"/>
-      <c r="K48" s="79"/>
-      <c r="L48" s="79"/>
-      <c r="M48" s="68"/>
-      <c r="N48" s="68"/>
-      <c r="O48" s="68"/>
-      <c r="P48" s="68"/>
-      <c r="Q48" s="67"/>
-      <c r="R48" s="67"/>
-      <c r="S48" s="82"/>
-      <c r="T48" s="68"/>
-      <c r="U48" s="68"/>
-      <c r="V48" s="82"/>
-      <c r="W48" s="68"/>
-      <c r="X48" s="68"/>
-      <c r="Y48" s="83"/>
-      <c r="Z48" s="84"/>
-      <c r="AA48" s="84"/>
-      <c r="AB48" s="68"/>
-      <c r="AC48" s="68"/>
-      <c r="AD48" s="68"/>
+      <c r="AD47" s="45" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="67"/>
+      <c r="B48" s="67"/>
+      <c r="C48" s="67"/>
+      <c r="D48" s="67"/>
+      <c r="E48" s="85"/>
+      <c r="F48" s="86"/>
+      <c r="G48" s="86"/>
+      <c r="H48" s="80"/>
+      <c r="I48" s="86"/>
+      <c r="J48" s="87"/>
+      <c r="K48" s="78"/>
+      <c r="L48" s="78"/>
+      <c r="M48" s="67"/>
+      <c r="N48" s="67"/>
+      <c r="O48" s="67"/>
+      <c r="P48" s="67"/>
+      <c r="Q48" s="66"/>
+      <c r="R48" s="66"/>
+      <c r="S48" s="81"/>
+      <c r="T48" s="67"/>
+      <c r="U48" s="67"/>
+      <c r="V48" s="81"/>
+      <c r="W48" s="67"/>
+      <c r="X48" s="67"/>
+      <c r="Y48" s="82"/>
+      <c r="Z48" s="83"/>
+      <c r="AA48" s="83"/>
+      <c r="AB48" s="67"/>
+      <c r="AC48" s="67"/>
+      <c r="AD48" s="67"/>
     </row>
     <row r="49" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="20"/>
@@ -5846,10 +5848,10 @@
       <c r="C49" s="20"/>
       <c r="D49" s="20"/>
       <c r="E49" s="24"/>
-      <c r="F49" s="69"/>
-      <c r="G49" s="69"/>
+      <c r="F49" s="68"/>
+      <c r="G49" s="68"/>
       <c r="H49" s="24"/>
-      <c r="I49" s="64"/>
+      <c r="I49" s="63"/>
       <c r="J49" s="20"/>
       <c r="K49" s="22"/>
       <c r="L49" s="22"/>
@@ -36571,101 +36573,101 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="46">
+    <row r="3" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="45">
         <v>2</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="46">
+      <c r="C3" s="45">
         <v>4</v>
       </c>
-      <c r="D3" s="46">
+      <c r="D3" s="45">
         <v>1</v>
       </c>
-      <c r="E3" s="47">
+      <c r="E3" s="46">
         <v>44983</v>
       </c>
-      <c r="F3" s="51">
+      <c r="F3" s="50">
         <v>12.250277777784504</v>
       </c>
-      <c r="G3" s="46" t="s">
+      <c r="G3" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="46"/>
-    </row>
-    <row r="4" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="46">
+      <c r="H3" s="45"/>
+    </row>
+    <row r="4" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="45">
         <v>2</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="45">
         <v>4</v>
       </c>
-      <c r="D4" s="46">
+      <c r="D4" s="45">
         <v>2</v>
       </c>
-      <c r="E4" s="47">
+      <c r="E4" s="46">
         <v>44983</v>
       </c>
-      <c r="F4" s="51">
+      <c r="F4" s="50">
         <v>11.499999999941792</v>
       </c>
-      <c r="G4" s="46" t="s">
+      <c r="G4" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="46"/>
-    </row>
-    <row r="5" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="46">
+      <c r="H4" s="45"/>
+    </row>
+    <row r="5" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="45">
         <v>2</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="45">
         <v>4</v>
       </c>
-      <c r="D5" s="46">
+      <c r="D5" s="45">
         <v>3</v>
       </c>
-      <c r="E5" s="47">
+      <c r="E5" s="46">
         <v>44983</v>
       </c>
-      <c r="F5" s="51">
+      <c r="F5" s="50">
         <v>12.083333333430346</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="46"/>
-    </row>
-    <row r="6" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="46">
+      <c r="H5" s="45"/>
+    </row>
+    <row r="6" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="45">
         <v>2</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="45">
         <v>4</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="45">
         <v>4</v>
       </c>
-      <c r="E6" s="47">
+      <c r="E6" s="46">
         <v>44983</v>
       </c>
-      <c r="F6" s="51">
+      <c r="F6" s="50">
         <v>11.583055555529427</v>
       </c>
-      <c r="G6" s="46" t="s">
+      <c r="G6" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="46"/>
+      <c r="H6" s="45"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="20">
@@ -36715,29 +36717,29 @@
       </c>
       <c r="H8" s="20"/>
     </row>
-    <row r="9" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="46">
+    <row r="9" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="45">
         <v>4</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="45">
         <v>6</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="45">
         <v>1</v>
       </c>
-      <c r="E9" s="47">
+      <c r="E9" s="46">
         <v>44985</v>
       </c>
-      <c r="F9" s="51">
+      <c r="F9" s="50">
         <v>1.7480555555666797</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="G9" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="46" t="s">
+      <c r="H9" s="45" t="s">
         <v>31</v>
       </c>
     </row>
@@ -36767,53 +36769,53 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="46">
+    <row r="11" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="45">
         <v>6</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="45">
         <v>4</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="45">
         <v>1</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="46">
         <v>45084</v>
       </c>
-      <c r="F11" s="51">
+      <c r="F11" s="50">
         <v>12.746666666760575</v>
       </c>
-      <c r="G11" s="46" t="s">
+      <c r="G11" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="46"/>
-    </row>
-    <row r="12" spans="1:8" s="53" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="46">
+      <c r="H11" s="45"/>
+    </row>
+    <row r="12" spans="1:8" s="52" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="45">
         <v>7</v>
       </c>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="45">
         <v>4</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="45">
         <v>2</v>
       </c>
-      <c r="E12" s="47">
+      <c r="E12" s="46">
         <v>45084</v>
       </c>
-      <c r="F12" s="51">
+      <c r="F12" s="50">
         <v>11.666944444470573</v>
       </c>
-      <c r="G12" s="46" t="s">
+      <c r="G12" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="46"/>
+      <c r="H12" s="45"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="20">
@@ -36863,29 +36865,29 @@
       </c>
       <c r="H14" s="20"/>
     </row>
-    <row r="15" spans="1:8" s="57" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="46">
+    <row r="15" spans="1:8" s="56" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="45">
         <v>10</v>
       </c>
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="45">
         <v>6</v>
       </c>
-      <c r="D15" s="46">
+      <c r="D15" s="45">
         <v>1</v>
       </c>
-      <c r="E15" s="47">
+      <c r="E15" s="46">
         <v>45176</v>
       </c>
-      <c r="F15" s="51">
+      <c r="F15" s="50">
         <v>88.993611111072823</v>
       </c>
-      <c r="G15" s="46" t="s">
+      <c r="G15" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="46"/>
+      <c r="H15" s="45"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="20">
@@ -36965,55 +36967,55 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="60">
+    <row r="19" spans="1:8" s="62" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="59">
         <v>12</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="60">
+      <c r="C19" s="59">
         <v>6</v>
       </c>
-      <c r="D19" s="60">
+      <c r="D19" s="59">
         <v>1</v>
       </c>
-      <c r="E19" s="61">
+      <c r="E19" s="60">
         <v>45317</v>
       </c>
-      <c r="F19" s="62">
+      <c r="F19" s="61">
         <v>21.333611111040227</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="H19" s="60" t="s">
+      <c r="H19" s="59" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="60">
+    <row r="20" spans="1:8" s="62" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="59">
         <v>12</v>
       </c>
-      <c r="B20" s="60" t="s">
+      <c r="B20" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="60">
+      <c r="C20" s="59">
         <v>6</v>
       </c>
-      <c r="D20" s="60">
+      <c r="D20" s="59">
         <v>1</v>
       </c>
-      <c r="E20" s="61">
+      <c r="E20" s="60">
         <v>45317</v>
       </c>
-      <c r="F20" s="62">
+      <c r="F20" s="61">
         <v>47.183611111133359</v>
       </c>
-      <c r="G20" s="60" t="s">
+      <c r="G20" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="60" t="s">
+      <c r="H20" s="59" t="s">
         <v>98</v>
       </c>
     </row>
@@ -46705,11 +46707,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="92" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
adding time first/last sat for first deployment in 2022
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3566AD84-CB95-BE4D-8594-32FE44B64926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60FB676B-4435-E14B-83B4-D71C86BC1473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2620" yWindow="7220" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -866,11 +866,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1998,15 +1998,27 @@
       <c r="R2" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="S2" s="43"/>
-      <c r="T2" s="92"/>
-      <c r="U2" s="92"/>
-      <c r="V2" s="43"/>
-      <c r="W2" s="92"/>
-      <c r="X2" s="92"/>
+      <c r="S2" s="43">
+        <v>44818.76803240741</v>
+      </c>
+      <c r="T2" s="94">
+        <v>39.866098999999998</v>
+      </c>
+      <c r="U2" s="94">
+        <v>-70.443217000000004</v>
+      </c>
+      <c r="V2" s="43">
+        <v>44818.809594907405</v>
+      </c>
+      <c r="W2" s="94">
+        <v>39.867842000000003</v>
+      </c>
+      <c r="X2" s="94">
+        <v>-70.437183000000005</v>
+      </c>
       <c r="Y2" s="50">
         <f t="shared" ref="Y2:Y39" si="2">(V2-S2)*1440/60</f>
-        <v>0</v>
+        <v>0.99749999988125637</v>
       </c>
       <c r="Z2" s="44">
         <v>0.43124999999999997</v>
@@ -46719,11 +46731,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="92" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
fix for plotting when no control system data exists, update config file names for 2024 in spreadsheet to match others (taking the convention that I only change the name of the config file if something in it changes)
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLab/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60FB676B-4435-E14B-83B4-D71C86BC1473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3612F36B-A290-014A-8094-2BA0BABA3395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6580" yWindow="500" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Drifter Log 2022-2023'!$A$1:$AD$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SanDiegoSummary!$A$1:$H$15</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="134">
   <si>
     <t>Deployment</t>
   </si>
@@ -387,9 +386,6 @@
   </si>
   <si>
     <t>2024_May_CA</t>
-  </si>
-  <si>
-    <t>acoustic_config_Drifter5_VS209_2024.txt</t>
   </si>
   <si>
     <t>20240517T172653</t>
@@ -866,11 +862,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -2001,19 +1997,19 @@
       <c r="S2" s="43">
         <v>44818.76803240741</v>
       </c>
-      <c r="T2" s="94">
+      <c r="T2" s="92">
         <v>39.866098999999998</v>
       </c>
-      <c r="U2" s="94">
+      <c r="U2" s="92">
         <v>-70.443217000000004</v>
       </c>
       <c r="V2" s="43">
         <v>44818.809594907405</v>
       </c>
-      <c r="W2" s="94">
+      <c r="W2" s="92">
         <v>39.867842000000003</v>
       </c>
-      <c r="X2" s="94">
+      <c r="X2" s="92">
         <v>-70.437183000000005</v>
       </c>
       <c r="Y2" s="50">
@@ -2144,7 +2140,7 @@
       </c>
       <c r="F4" s="40"/>
       <c r="G4" s="88" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H4" s="37">
         <v>38.944544999999998</v>
@@ -2157,7 +2153,7 @@
       </c>
       <c r="K4" s="40"/>
       <c r="L4" s="89" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M4" s="37">
         <v>38.974831000000002</v>
@@ -2233,7 +2229,7 @@
       </c>
       <c r="F5" s="22"/>
       <c r="G5" s="90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H5" s="20">
         <v>38.917915000000001</v>
@@ -2246,7 +2242,7 @@
       </c>
       <c r="K5" s="22"/>
       <c r="L5" s="22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M5" s="20">
         <v>38.868670000000002</v>
@@ -2320,7 +2316,7 @@
       </c>
       <c r="F6" s="47"/>
       <c r="G6" s="88" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H6" s="45">
         <v>38.885973999999997</v>
@@ -2333,7 +2329,7 @@
       </c>
       <c r="K6" s="47"/>
       <c r="L6" s="47" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M6" s="45">
         <v>38.879128999999999</v>
@@ -5353,14 +5349,14 @@
       </c>
       <c r="F41" s="47"/>
       <c r="G41" s="41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H41" s="45"/>
       <c r="I41" s="45"/>
       <c r="J41" s="46"/>
       <c r="K41" s="47"/>
       <c r="L41" s="55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M41" s="45"/>
       <c r="N41" s="45"/>
@@ -5409,7 +5405,7 @@
         <v>0.43533564814814812</v>
       </c>
       <c r="G42" s="78" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H42" s="67"/>
       <c r="I42" s="67"/>
@@ -5420,7 +5416,7 @@
         <v>0.52296296296296296</v>
       </c>
       <c r="L42" s="78" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M42" s="67"/>
       <c r="N42" s="67"/>
@@ -5434,10 +5430,10 @@
         <v>300434066482170</v>
       </c>
       <c r="R42" s="66" t="s">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="S42" s="28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="T42" s="71">
         <v>32.917650000000002</v>
@@ -5446,13 +5442,13 @@
         <v>-117.794504</v>
       </c>
       <c r="V42" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W42" s="71" t="s">
+        <v>119</v>
+      </c>
+      <c r="X42" s="71" t="s">
         <v>120</v>
-      </c>
-      <c r="X42" s="71" t="s">
-        <v>121</v>
       </c>
       <c r="Y42" s="82"/>
       <c r="Z42" s="83">
@@ -5487,7 +5483,7 @@
         <v>0.43533564814814812</v>
       </c>
       <c r="G43" s="78" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H43" s="67"/>
       <c r="I43" s="67"/>
@@ -5498,7 +5494,7 @@
         <v>0.52296296296296296</v>
       </c>
       <c r="L43" s="78" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M43" s="67"/>
       <c r="N43" s="67"/>
@@ -5512,10 +5508,10 @@
         <v>300434066482170</v>
       </c>
       <c r="R43" s="66" t="s">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="S43" s="28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="T43" s="71">
         <v>32.998700999999997</v>
@@ -5524,7 +5520,7 @@
         <v>-117.874388</v>
       </c>
       <c r="V43" s="28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="W43" s="71">
         <v>33.012540000000001</v>
@@ -5550,7 +5546,7 @@
         <v>27</v>
       </c>
       <c r="B44" s="45" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C44" s="45">
         <v>5</v>
@@ -5612,7 +5608,7 @@
         <v>28</v>
       </c>
       <c r="B45" s="67" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C45" s="67">
         <v>6</v>
@@ -5681,7 +5677,7 @@
         <v>28</v>
       </c>
       <c r="B46" s="67" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C46" s="67">
         <v>6</v>
@@ -5742,7 +5738,7 @@
       <c r="AB46" s="67"/>
       <c r="AC46" s="67"/>
       <c r="AD46" s="67" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:30" s="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5750,7 +5746,7 @@
         <v>29</v>
       </c>
       <c r="B47" s="45" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C47" s="45">
         <v>4</v>
@@ -5831,7 +5827,7 @@
         <v>4</v>
       </c>
       <c r="AD47" s="45" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" spans="1:30" s="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -46731,11 +46727,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="93" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="93"/>
-      <c r="C1" s="93"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
adding june seamount map plot, updating deployment log entries for June, adding colormaps, minor updates to some other functions
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLabClean/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7A4832-EED6-2C40-9589-82941276B62B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3628C5A1-1AC3-C147-B852-5B8C89A5AA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6580" yWindow="500" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1960" yWindow="560" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -5585,8 +5585,12 @@
         <f>$E44+$F44+TIME(AC44,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H44" s="44"/>
-      <c r="I44" s="44"/>
+      <c r="H44">
+        <v>38.314742000000003</v>
+      </c>
+      <c r="I44">
+        <v>-63.009855000000002</v>
+      </c>
       <c r="J44" s="45">
         <v>45468</v>
       </c>
@@ -5594,8 +5598,12 @@
       <c r="L44" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="M44" s="68"/>
-      <c r="N44" s="68"/>
+      <c r="M44" s="77">
+        <v>38.937788333333302</v>
+      </c>
+      <c r="N44" s="68">
+        <v>-64.252854999999997</v>
+      </c>
       <c r="O44" s="44">
         <v>3</v>
       </c>
@@ -5617,7 +5625,9 @@
       <c r="U44" s="68">
         <v>-63.006925000000003</v>
       </c>
-      <c r="V44" s="48"/>
+      <c r="V44" s="78">
+        <v>45465.117199074077</v>
+      </c>
       <c r="W44" s="44"/>
       <c r="X44" s="44"/>
       <c r="Y44" s="25"/>
@@ -5654,8 +5664,12 @@
         <f t="shared" ref="G45" si="8">$E45+$F45+TIME(AC45,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H45" s="65"/>
-      <c r="I45" s="65"/>
+      <c r="H45">
+        <v>38.315010000000001</v>
+      </c>
+      <c r="I45">
+        <v>-63.010885000000002</v>
+      </c>
       <c r="J45" s="75">
         <v>45466</v>
       </c>
@@ -5666,8 +5680,12 @@
         <f t="shared" ref="L45:L46" si="9">$J45+$K45 +TIME($AC45,0,0)</f>
         <v>45467.041666666664</v>
       </c>
-      <c r="M45" s="77"/>
-      <c r="N45" s="77"/>
+      <c r="M45" s="82">
+        <v>39.013003333333302</v>
+      </c>
+      <c r="N45" s="77">
+        <v>-63.364616666666699</v>
+      </c>
       <c r="O45" s="65">
         <v>4</v>
       </c>
@@ -5733,8 +5751,12 @@
         <f t="shared" ref="G46" si="10">$E46+$F46+TIME(AC46,0,0)</f>
         <v>45462.791666666664</v>
       </c>
-      <c r="H46" s="65"/>
-      <c r="I46" s="65"/>
+      <c r="H46">
+        <v>38.315010000000001</v>
+      </c>
+      <c r="I46">
+        <v>-63.010885000000002</v>
+      </c>
       <c r="J46" s="75">
         <v>45466</v>
       </c>
@@ -5745,8 +5767,12 @@
         <f t="shared" si="9"/>
         <v>45467.041666666664</v>
       </c>
-      <c r="M46" s="77"/>
-      <c r="N46" s="77"/>
+      <c r="M46" s="82">
+        <v>39.013003333333302</v>
+      </c>
+      <c r="N46" s="77">
+        <v>-63.364616666666699</v>
+      </c>
       <c r="O46" s="65">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Added 2025 Hawaii to drifter log
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/ThodeLabClean/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3628C5A1-1AC3-C147-B852-5B8C89A5AA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F92BF0B-768C-3245-818D-542440B2C96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1960" yWindow="560" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1960" yWindow="560" windowWidth="39000" windowHeight="24780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
+    <sheet name="Drifter Log 2022-2025" sheetId="1" r:id="rId1"/>
     <sheet name="SanDiegoSummary" sheetId="4" r:id="rId2"/>
     <sheet name="NOAA Solar Calculator" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Drifter Log 2022-2023'!$A$1:$AD$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Drifter Log 2022-2025'!$A$1:$AD$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SanDiegoSummary!$A$1:$H$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="140">
   <si>
     <t>Deployment</t>
   </si>
@@ -460,18 +460,20 @@
   <si>
     <t>2024_Jun_Seamounts</t>
   </si>
+  <si>
+    <t>2025_Hawaii</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\Thh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
     <numFmt numFmtId="167" formatCode="0.00000000"/>
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
-    <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -637,7 +639,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -825,22 +827,16 @@
     <xf numFmtId="14" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2007,19 +2003,19 @@
       <c r="S2" s="42">
         <v>44818.76803240741</v>
       </c>
-      <c r="T2" s="90">
+      <c r="T2" s="88">
         <v>39.866098999999998</v>
       </c>
-      <c r="U2" s="90">
+      <c r="U2" s="88">
         <v>-70.443217000000004</v>
       </c>
       <c r="V2" s="42">
         <v>44818.809594907405</v>
       </c>
-      <c r="W2" s="90">
+      <c r="W2" s="88">
         <v>39.867842000000003</v>
       </c>
-      <c r="X2" s="90">
+      <c r="X2" s="88">
         <v>-70.437183000000005</v>
       </c>
       <c r="Y2" s="49">
@@ -2149,7 +2145,7 @@
         <v>44822</v>
       </c>
       <c r="F4" s="39"/>
-      <c r="G4" s="86" t="s">
+      <c r="G4" s="84" t="s">
         <v>125</v>
       </c>
       <c r="H4" s="36">
@@ -2162,7 +2158,7 @@
         <v>44822</v>
       </c>
       <c r="K4" s="39"/>
-      <c r="L4" s="87" t="s">
+      <c r="L4" s="85" t="s">
         <v>126</v>
       </c>
       <c r="M4" s="36">
@@ -2238,7 +2234,7 @@
         <v>44822</v>
       </c>
       <c r="F5" s="22"/>
-      <c r="G5" s="88" t="s">
+      <c r="G5" s="86" t="s">
         <v>127</v>
       </c>
       <c r="H5" s="20">
@@ -2325,7 +2321,7 @@
         <v>44823</v>
       </c>
       <c r="F6" s="46"/>
-      <c r="G6" s="86" t="s">
+      <c r="G6" s="84" t="s">
         <v>129</v>
       </c>
       <c r="H6" s="44">
@@ -5402,7 +5398,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="65">
         <v>26</v>
       </c>
@@ -5415,24 +5411,24 @@
       <c r="D42" s="65">
         <v>1</v>
       </c>
-      <c r="E42" s="75">
+      <c r="E42" s="74">
         <v>45429</v>
       </c>
-      <c r="F42" s="76">
+      <c r="F42" s="73">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G42" s="76" t="s">
+      <c r="G42" s="73" t="s">
         <v>115</v>
       </c>
       <c r="H42" s="65"/>
       <c r="I42" s="65"/>
-      <c r="J42" s="75">
+      <c r="J42" s="74">
         <v>45432</v>
       </c>
-      <c r="K42" s="76">
+      <c r="K42" s="73">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L42" s="76" t="s">
+      <c r="L42" s="73" t="s">
         <v>116</v>
       </c>
       <c r="M42" s="65"/>
@@ -5449,7 +5445,7 @@
       <c r="R42" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="S42" s="78" t="s">
+      <c r="S42" s="76" t="s">
         <v>118</v>
       </c>
       <c r="T42" s="69">
@@ -5458,7 +5454,7 @@
       <c r="U42" s="69">
         <v>-117.794504</v>
       </c>
-      <c r="V42" s="78" t="s">
+      <c r="V42" s="76" t="s">
         <v>117</v>
       </c>
       <c r="W42" s="69" t="s">
@@ -5468,10 +5464,10 @@
         <v>120</v>
       </c>
       <c r="Y42" s="25"/>
-      <c r="Z42" s="81">
+      <c r="Z42" s="79">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA42" s="81">
+      <c r="AA42" s="79">
         <v>0.1125</v>
       </c>
       <c r="AB42" s="65"/>
@@ -5482,7 +5478,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="65">
         <v>26</v>
       </c>
@@ -5495,24 +5491,24 @@
       <c r="D43" s="65">
         <v>2</v>
       </c>
-      <c r="E43" s="75">
+      <c r="E43" s="74">
         <v>45429</v>
       </c>
-      <c r="F43" s="76">
+      <c r="F43" s="73">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G43" s="76" t="s">
+      <c r="G43" s="73" t="s">
         <v>115</v>
       </c>
       <c r="H43" s="65"/>
       <c r="I43" s="65"/>
-      <c r="J43" s="75">
+      <c r="J43" s="74">
         <v>45432</v>
       </c>
-      <c r="K43" s="76">
+      <c r="K43" s="73">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L43" s="76" t="s">
+      <c r="L43" s="73" t="s">
         <v>116</v>
       </c>
       <c r="M43" s="65"/>
@@ -5529,7 +5525,7 @@
       <c r="R43" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="S43" s="78" t="s">
+      <c r="S43" s="76" t="s">
         <v>121</v>
       </c>
       <c r="T43" s="69">
@@ -5538,7 +5534,7 @@
       <c r="U43" s="69">
         <v>-117.874388</v>
       </c>
-      <c r="V43" s="78" t="s">
+      <c r="V43" s="76" t="s">
         <v>122</v>
       </c>
       <c r="W43" s="69">
@@ -5548,10 +5544,10 @@
         <v>-117.890097</v>
       </c>
       <c r="Y43" s="25"/>
-      <c r="Z43" s="81">
+      <c r="Z43" s="79">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA43" s="81">
+      <c r="AA43" s="79">
         <v>0.1125</v>
       </c>
       <c r="AB43" s="65"/>
@@ -5578,7 +5574,7 @@
       <c r="E44" s="70">
         <v>45462</v>
       </c>
-      <c r="F44" s="71">
+      <c r="F44" s="46">
         <v>0.625</v>
       </c>
       <c r="G44" s="40">
@@ -5598,7 +5594,7 @@
       <c r="L44" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="M44" s="77">
+      <c r="M44" s="75">
         <v>38.937788333333302</v>
       </c>
       <c r="N44" s="68">
@@ -5625,7 +5621,7 @@
       <c r="U44" s="68">
         <v>-63.006925000000003</v>
       </c>
-      <c r="V44" s="78">
+      <c r="V44" s="76">
         <v>45465.117199074077</v>
       </c>
       <c r="W44" s="44"/>
@@ -5641,7 +5637,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="65">
         <v>28</v>
       </c>
@@ -5654,10 +5650,10 @@
       <c r="D45" s="65">
         <v>1</v>
       </c>
-      <c r="E45" s="73">
+      <c r="E45" s="72">
         <v>45462</v>
       </c>
-      <c r="F45" s="74">
+      <c r="F45" s="73">
         <v>0.625</v>
       </c>
       <c r="G45" s="62">
@@ -5670,20 +5666,20 @@
       <c r="I45">
         <v>-63.010885000000002</v>
       </c>
-      <c r="J45" s="75">
+      <c r="J45" s="74">
         <v>45466</v>
       </c>
-      <c r="K45" s="76">
+      <c r="K45" s="73">
         <v>0.875</v>
       </c>
       <c r="L45" s="63">
         <f t="shared" ref="L45:L46" si="9">$J45+$K45 +TIME($AC45,0,0)</f>
         <v>45467.041666666664</v>
       </c>
-      <c r="M45" s="82">
+      <c r="M45" s="80">
         <v>39.013003333333302</v>
       </c>
-      <c r="N45" s="77">
+      <c r="N45" s="75">
         <v>-63.364616666666699</v>
       </c>
       <c r="O45" s="65">
@@ -5698,37 +5694,37 @@
       <c r="R45" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="S45" s="78">
+      <c r="S45" s="76">
         <v>45462.855231481481</v>
       </c>
-      <c r="T45" s="89">
+      <c r="T45" s="87">
         <v>38.307771000000002</v>
       </c>
-      <c r="U45" s="89">
+      <c r="U45" s="87">
         <v>-62.998032000000002</v>
       </c>
-      <c r="V45" s="78">
+      <c r="V45" s="76">
         <v>45465.11142361111</v>
       </c>
-      <c r="W45" s="89">
+      <c r="W45" s="87">
         <v>38.406742000000001</v>
       </c>
-      <c r="X45" s="89">
+      <c r="X45" s="87">
         <v>-62.544604</v>
       </c>
       <c r="Y45" s="25">
         <f t="shared" si="7"/>
         <v>54.148611111100763</v>
       </c>
-      <c r="Z45" s="81"/>
-      <c r="AA45" s="81"/>
+      <c r="Z45" s="79"/>
+      <c r="AA45" s="79"/>
       <c r="AB45" s="65"/>
       <c r="AC45" s="65">
         <v>4</v>
       </c>
       <c r="AD45" s="65"/>
     </row>
-    <row r="46" spans="1:30" s="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="65">
         <v>28</v>
       </c>
@@ -5741,10 +5737,10 @@
       <c r="D46" s="65">
         <v>2</v>
       </c>
-      <c r="E46" s="73">
+      <c r="E46" s="72">
         <v>45462</v>
       </c>
-      <c r="F46" s="74">
+      <c r="F46" s="73">
         <v>0.625</v>
       </c>
       <c r="G46" s="62">
@@ -5757,20 +5753,20 @@
       <c r="I46">
         <v>-63.010885000000002</v>
       </c>
-      <c r="J46" s="75">
+      <c r="J46" s="74">
         <v>45466</v>
       </c>
-      <c r="K46" s="76">
+      <c r="K46" s="73">
         <v>0.875</v>
       </c>
       <c r="L46" s="63">
         <f t="shared" si="9"/>
         <v>45467.041666666664</v>
       </c>
-      <c r="M46" s="82">
+      <c r="M46" s="80">
         <v>39.013003333333302</v>
       </c>
-      <c r="N46" s="77">
+      <c r="N46" s="75">
         <v>-63.364616666666699</v>
       </c>
       <c r="O46" s="65">
@@ -5785,30 +5781,30 @@
       <c r="R46" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="S46" s="78">
+      <c r="S46" s="76">
         <v>45465.271736111114</v>
       </c>
-      <c r="T46" s="89">
+      <c r="T46" s="87">
         <v>38.415380999999996</v>
       </c>
-      <c r="U46" s="89">
+      <c r="U46" s="87">
         <v>-62.463433000000002</v>
       </c>
       <c r="V46" s="28">
         <v>45466.125555555554</v>
       </c>
-      <c r="W46" s="89">
+      <c r="W46" s="87">
         <v>38.532255999999997</v>
       </c>
-      <c r="X46" s="89">
+      <c r="X46" s="87">
         <v>-62.362059000000002</v>
       </c>
       <c r="Y46" s="25">
         <f t="shared" si="7"/>
         <v>20.491666666581295</v>
       </c>
-      <c r="Z46" s="81"/>
-      <c r="AA46" s="81"/>
+      <c r="Z46" s="79"/>
+      <c r="AA46" s="79"/>
       <c r="AB46" s="65"/>
       <c r="AC46" s="65">
         <v>4</v>
@@ -5833,7 +5829,7 @@
       <c r="E47" s="70">
         <v>45462</v>
       </c>
-      <c r="F47" s="71">
+      <c r="F47" s="46">
         <v>0.625</v>
       </c>
       <c r="G47" s="40">
@@ -5868,7 +5864,7 @@
       <c r="P47" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="Q47" s="72">
+      <c r="Q47" s="71">
         <v>300434066489180</v>
       </c>
       <c r="R47" s="47" t="s">
@@ -5906,42 +5902,58 @@
         <v>132</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="65"/>
-      <c r="B48" s="65"/>
-      <c r="C48" s="65"/>
-      <c r="D48" s="65"/>
-      <c r="E48" s="83"/>
-      <c r="F48" s="84"/>
-      <c r="G48" s="84"/>
-      <c r="H48" s="78"/>
-      <c r="I48" s="84"/>
-      <c r="J48" s="85"/>
-      <c r="K48" s="76"/>
-      <c r="L48" s="76"/>
+    <row r="48" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="65">
+        <v>30</v>
+      </c>
+      <c r="B48" s="65" t="s">
+        <v>139</v>
+      </c>
+      <c r="C48" s="65">
+        <v>5</v>
+      </c>
+      <c r="D48" s="65">
+        <v>1</v>
+      </c>
+      <c r="E48" s="81"/>
+      <c r="F48" s="82"/>
+      <c r="G48" s="82"/>
+      <c r="H48" s="76"/>
+      <c r="I48" s="82"/>
+      <c r="J48" s="83"/>
+      <c r="K48" s="73"/>
+      <c r="L48" s="73"/>
       <c r="M48" s="65"/>
       <c r="N48" s="65"/>
       <c r="O48" s="65"/>
       <c r="P48" s="65"/>
       <c r="Q48" s="64"/>
       <c r="R48" s="64"/>
-      <c r="S48" s="79"/>
+      <c r="S48" s="77"/>
       <c r="T48" s="65"/>
       <c r="U48" s="65"/>
       <c r="W48" s="65"/>
       <c r="X48" s="65"/>
-      <c r="Y48" s="80"/>
-      <c r="Z48" s="81"/>
-      <c r="AA48" s="81"/>
+      <c r="Y48" s="78"/>
+      <c r="Z48" s="79"/>
+      <c r="AA48" s="79"/>
       <c r="AB48" s="65"/>
       <c r="AC48" s="65"/>
       <c r="AD48" s="65"/>
     </row>
     <row r="49" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="20"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
+      <c r="A49" s="20">
+        <v>30</v>
+      </c>
+      <c r="B49" s="65" t="s">
+        <v>139</v>
+      </c>
+      <c r="C49" s="20">
+        <v>5</v>
+      </c>
+      <c r="D49" s="20">
+        <v>2</v>
+      </c>
       <c r="E49" s="24"/>
       <c r="F49" s="66"/>
       <c r="G49" s="66"/>
@@ -5970,10 +5982,18 @@
       <c r="AD49" s="20"/>
     </row>
     <row r="50" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="20"/>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
+      <c r="A50" s="20">
+        <v>31</v>
+      </c>
+      <c r="B50" s="65" t="s">
+        <v>139</v>
+      </c>
+      <c r="C50" s="20">
+        <v>5</v>
+      </c>
+      <c r="D50" s="20">
+        <v>1</v>
+      </c>
       <c r="E50" s="21"/>
       <c r="F50" s="22"/>
       <c r="G50" s="22"/>
@@ -6002,10 +6022,18 @@
       <c r="AD50" s="20"/>
     </row>
     <row r="51" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="20"/>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
+      <c r="A51" s="20">
+        <v>32</v>
+      </c>
+      <c r="B51" s="65" t="s">
+        <v>139</v>
+      </c>
+      <c r="C51" s="20">
+        <v>5</v>
+      </c>
+      <c r="D51" s="20">
+        <v>1</v>
+      </c>
       <c r="E51" s="21"/>
       <c r="F51" s="22"/>
       <c r="G51" s="22"/>
@@ -46802,11 +46830,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="89" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
updating log to be consistent with bulk processing runs on macmussel for Nov and HI
</commit_message>
<xml_diff>
--- a/drifter/TFO_Drifter_deployment_log.xlsx
+++ b/drifter/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thode/Desktop/ThodeLab/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/ThodeLab/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F92BF0B-768C-3245-818D-542440B2C96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D802BC-8FDF-D740-AB78-7F60DCBB4BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1960" yWindow="560" windowWidth="39000" windowHeight="24780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12780" yWindow="500" windowWidth="39000" windowHeight="20860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2025" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="148">
   <si>
     <t>Deployment</t>
   </si>
@@ -461,25 +461,57 @@
     <t>2024_Jun_Seamounts</t>
   </si>
   <si>
-    <t>2025_Hawaii</t>
+    <t>2024_Nov_CA</t>
+  </si>
+  <si>
+    <t>2025_May_HI</t>
+  </si>
+  <si>
+    <t>20250503T220700</t>
+  </si>
+  <si>
+    <t>20250505T220000</t>
+  </si>
+  <si>
+    <t>Deployed with TIDAL, which may have dragged on the ground</t>
+  </si>
+  <si>
+    <t>20250507T203200</t>
+  </si>
+  <si>
+    <t>20250509T011700</t>
+  </si>
+  <si>
+    <t>20250512T032100</t>
+  </si>
+  <si>
+    <t>20250512T230000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\Thh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
     <numFmt numFmtId="167" formatCode="0.00000000"/>
     <numFmt numFmtId="168" formatCode="yyyymmdd\Thhmmss"/>
+    <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -571,6 +603,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -636,94 +674,94 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="10" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="11" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -732,147 +770,153 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="3" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="169" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="168" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="1" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -2003,19 +2047,19 @@
       <c r="S2" s="42">
         <v>44818.76803240741</v>
       </c>
-      <c r="T2" s="88">
+      <c r="T2" s="85">
         <v>39.866098999999998</v>
       </c>
-      <c r="U2" s="88">
+      <c r="U2" s="85">
         <v>-70.443217000000004</v>
       </c>
       <c r="V2" s="42">
         <v>44818.809594907405</v>
       </c>
-      <c r="W2" s="88">
+      <c r="W2" s="85">
         <v>39.867842000000003</v>
       </c>
-      <c r="X2" s="88">
+      <c r="X2" s="85">
         <v>-70.437183000000005</v>
       </c>
       <c r="Y2" s="49">
@@ -2054,7 +2098,7 @@
       <c r="F3" s="22">
         <v>0.42638888888888887</v>
       </c>
-      <c r="G3" s="62">
+      <c r="G3" s="61">
         <f t="shared" si="0"/>
         <v>44819.593055555553</v>
       </c>
@@ -2070,7 +2114,7 @@
       <c r="K3" s="22">
         <v>0.47638888888888892</v>
       </c>
-      <c r="L3" s="62">
+      <c r="L3" s="61">
         <f t="shared" si="1"/>
         <v>44819.643055555556</v>
       </c>
@@ -2145,7 +2189,7 @@
         <v>44822</v>
       </c>
       <c r="F4" s="39"/>
-      <c r="G4" s="84" t="s">
+      <c r="G4" s="81" t="s">
         <v>125</v>
       </c>
       <c r="H4" s="36">
@@ -2158,7 +2202,7 @@
         <v>44822</v>
       </c>
       <c r="K4" s="39"/>
-      <c r="L4" s="85" t="s">
+      <c r="L4" s="82" t="s">
         <v>126</v>
       </c>
       <c r="M4" s="36">
@@ -2234,7 +2278,7 @@
         <v>44822</v>
       </c>
       <c r="F5" s="22"/>
-      <c r="G5" s="86" t="s">
+      <c r="G5" s="83" t="s">
         <v>127</v>
       </c>
       <c r="H5" s="20">
@@ -2321,7 +2365,7 @@
         <v>44823</v>
       </c>
       <c r="F6" s="46"/>
-      <c r="G6" s="84" t="s">
+      <c r="G6" s="81" t="s">
         <v>129</v>
       </c>
       <c r="H6" s="44">
@@ -4966,10 +5010,10 @@
       <c r="S36" s="48">
         <v>45317.875324074077</v>
       </c>
-      <c r="T36" s="67">
+      <c r="T36" s="65">
         <v>32.909129</v>
       </c>
-      <c r="U36" s="67">
+      <c r="U36" s="65">
         <v>-117.680663</v>
       </c>
       <c r="V36" s="48">
@@ -5051,10 +5095,10 @@
       <c r="S37" s="48">
         <v>45318.931122685186</v>
       </c>
-      <c r="T37" s="67">
+      <c r="T37" s="65">
         <v>33.001423000000003</v>
       </c>
-      <c r="U37" s="67">
+      <c r="U37" s="65">
         <v>-117.65347800000001</v>
       </c>
       <c r="V37" s="48">
@@ -5136,19 +5180,19 @@
       <c r="S38" s="48">
         <v>45319.910034722219</v>
       </c>
-      <c r="T38" s="68">
+      <c r="T38" s="66">
         <v>33.123451000000003</v>
       </c>
-      <c r="U38" s="68">
+      <c r="U38" s="66">
         <v>-117.600043</v>
       </c>
       <c r="V38" s="48">
         <v>45320.89980324074</v>
       </c>
-      <c r="W38" s="68">
+      <c r="W38" s="66">
         <v>33.200189999999999</v>
       </c>
-      <c r="X38" s="68">
+      <c r="X38" s="66">
         <v>-117.597759</v>
       </c>
       <c r="Y38" s="49">
@@ -5221,19 +5265,19 @@
       <c r="S39" s="28">
         <v>45317.993379629632</v>
       </c>
-      <c r="T39" s="69">
+      <c r="T39" s="67">
         <v>32.907333000000001</v>
       </c>
-      <c r="U39" s="69">
+      <c r="U39" s="67">
         <v>-117.67442</v>
       </c>
       <c r="V39" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="W39" s="69">
+      <c r="W39" s="67">
         <v>33.012383</v>
       </c>
-      <c r="X39" s="69">
+      <c r="X39" s="67">
         <v>-117.66186500000001</v>
       </c>
       <c r="Y39" s="25">
@@ -5306,19 +5350,19 @@
       <c r="S40" s="28">
         <v>45318.882280092592</v>
       </c>
-      <c r="T40" s="69">
+      <c r="T40" s="67">
         <v>33.012383</v>
       </c>
-      <c r="U40" s="69">
+      <c r="U40" s="67">
         <v>-117.66186500000001</v>
       </c>
       <c r="V40" s="28">
         <v>45320.848263888889</v>
       </c>
-      <c r="W40" s="69">
+      <c r="W40" s="67">
         <v>33.115271</v>
       </c>
-      <c r="X40" s="69">
+      <c r="X40" s="67">
         <v>-117.89773700000001</v>
       </c>
       <c r="Y40" s="25">
@@ -5381,11 +5425,11 @@
         <v>37</v>
       </c>
       <c r="S41" s="52"/>
-      <c r="T41" s="68"/>
-      <c r="U41" s="68"/>
+      <c r="T41" s="66"/>
+      <c r="U41" s="66"/>
       <c r="V41" s="52"/>
-      <c r="W41" s="68"/>
-      <c r="X41" s="68"/>
+      <c r="W41" s="66"/>
+      <c r="X41" s="66"/>
       <c r="Y41" s="25">
         <f t="shared" si="7"/>
         <v>0</v>
@@ -5398,163 +5442,163 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="65">
+    <row r="42" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="64">
         <v>26</v>
       </c>
-      <c r="B42" s="65" t="s">
+      <c r="B42" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="65">
+      <c r="C42" s="64">
         <v>5</v>
       </c>
-      <c r="D42" s="65">
+      <c r="D42" s="64">
         <v>1</v>
       </c>
-      <c r="E42" s="74">
+      <c r="E42" s="72">
         <v>45429</v>
       </c>
-      <c r="F42" s="73">
+      <c r="F42" s="71">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G42" s="73" t="s">
+      <c r="G42" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="H42" s="65"/>
-      <c r="I42" s="65"/>
-      <c r="J42" s="74">
+      <c r="H42" s="64"/>
+      <c r="I42" s="64"/>
+      <c r="J42" s="72">
         <v>45432</v>
       </c>
-      <c r="K42" s="73">
+      <c r="K42" s="71">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L42" s="73" t="s">
+      <c r="L42" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="M42" s="65"/>
-      <c r="N42" s="65"/>
-      <c r="O42" s="65">
+      <c r="M42" s="64"/>
+      <c r="N42" s="64"/>
+      <c r="O42" s="64">
         <v>3</v>
       </c>
-      <c r="P42" s="65" t="s">
+      <c r="P42" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="Q42" s="64">
+      <c r="Q42" s="63">
         <v>300434066482170</v>
       </c>
-      <c r="R42" s="64" t="s">
+      <c r="R42" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="S42" s="76" t="s">
+      <c r="S42" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="T42" s="69">
+      <c r="T42" s="67">
         <v>32.917650000000002</v>
       </c>
-      <c r="U42" s="69">
+      <c r="U42" s="67">
         <v>-117.794504</v>
       </c>
-      <c r="V42" s="76" t="s">
+      <c r="V42" s="74" t="s">
         <v>117</v>
       </c>
-      <c r="W42" s="69" t="s">
+      <c r="W42" s="67" t="s">
         <v>119</v>
       </c>
-      <c r="X42" s="69" t="s">
+      <c r="X42" s="67" t="s">
         <v>120</v>
       </c>
       <c r="Y42" s="25"/>
-      <c r="Z42" s="79">
+      <c r="Z42" s="77">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA42" s="79">
+      <c r="AA42" s="77">
         <v>0.1125</v>
       </c>
-      <c r="AB42" s="65"/>
-      <c r="AC42" s="65">
+      <c r="AB42" s="64"/>
+      <c r="AC42" s="64">
         <v>7</v>
       </c>
-      <c r="AD42" s="65" t="s">
+      <c r="AD42" s="64" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="65">
+    <row r="43" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="64">
         <v>26</v>
       </c>
-      <c r="B43" s="65" t="s">
+      <c r="B43" s="64" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="65">
+      <c r="C43" s="64">
         <v>5</v>
       </c>
-      <c r="D43" s="65">
+      <c r="D43" s="64">
         <v>2</v>
       </c>
-      <c r="E43" s="74">
+      <c r="E43" s="72">
         <v>45429</v>
       </c>
-      <c r="F43" s="73">
+      <c r="F43" s="71">
         <v>0.43533564814814812</v>
       </c>
-      <c r="G43" s="73" t="s">
+      <c r="G43" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="H43" s="65"/>
-      <c r="I43" s="65"/>
-      <c r="J43" s="74">
+      <c r="H43" s="64"/>
+      <c r="I43" s="64"/>
+      <c r="J43" s="72">
         <v>45432</v>
       </c>
-      <c r="K43" s="73">
+      <c r="K43" s="71">
         <v>0.52296296296296296</v>
       </c>
-      <c r="L43" s="73" t="s">
+      <c r="L43" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="M43" s="65"/>
-      <c r="N43" s="65"/>
-      <c r="O43" s="65">
+      <c r="M43" s="64"/>
+      <c r="N43" s="64"/>
+      <c r="O43" s="64">
         <v>3</v>
       </c>
-      <c r="P43" s="65" t="s">
+      <c r="P43" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="Q43" s="64">
+      <c r="Q43" s="63">
         <v>300434066482170</v>
       </c>
-      <c r="R43" s="64" t="s">
+      <c r="R43" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="S43" s="76" t="s">
+      <c r="S43" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="T43" s="69">
+      <c r="T43" s="67">
         <v>32.998700999999997</v>
       </c>
-      <c r="U43" s="69">
+      <c r="U43" s="67">
         <v>-117.874388</v>
       </c>
-      <c r="V43" s="76" t="s">
+      <c r="V43" s="74" t="s">
         <v>122</v>
       </c>
-      <c r="W43" s="69">
+      <c r="W43" s="67">
         <v>33.012540000000001</v>
       </c>
-      <c r="X43" s="69">
+      <c r="X43" s="67">
         <v>-117.890097</v>
       </c>
       <c r="Y43" s="25"/>
-      <c r="Z43" s="79">
+      <c r="Z43" s="77">
         <v>0.53263888888888888</v>
       </c>
-      <c r="AA43" s="79">
+      <c r="AA43" s="77">
         <v>0.1125</v>
       </c>
-      <c r="AB43" s="65"/>
-      <c r="AC43" s="65">
+      <c r="AB43" s="64"/>
+      <c r="AC43" s="64">
         <v>7</v>
       </c>
-      <c r="AD43" s="65" t="s">
+      <c r="AD43" s="64" t="s">
         <v>136</v>
       </c>
     </row>
@@ -5571,7 +5615,7 @@
       <c r="D44" s="44">
         <v>1</v>
       </c>
-      <c r="E44" s="70">
+      <c r="E44" s="68">
         <v>45462</v>
       </c>
       <c r="F44" s="46">
@@ -5594,10 +5638,10 @@
       <c r="L44" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="M44" s="75">
+      <c r="M44" s="73">
         <v>38.937788333333302</v>
       </c>
-      <c r="N44" s="68">
+      <c r="N44" s="66">
         <v>-64.252854999999997</v>
       </c>
       <c r="O44" s="44">
@@ -5615,13 +5659,13 @@
       <c r="S44" s="52">
         <v>45462.860289351855</v>
       </c>
-      <c r="T44" s="68">
+      <c r="T44" s="66">
         <v>38.313133999999998</v>
       </c>
-      <c r="U44" s="68">
+      <c r="U44" s="66">
         <v>-63.006925000000003</v>
       </c>
-      <c r="V44" s="76">
+      <c r="V44" s="74">
         <v>45465.117199074077</v>
       </c>
       <c r="W44" s="44"/>
@@ -5637,26 +5681,26 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="65">
+    <row r="45" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="64">
         <v>28</v>
       </c>
-      <c r="B45" s="65" t="s">
+      <c r="B45" s="64" t="s">
         <v>138</v>
       </c>
-      <c r="C45" s="65">
+      <c r="C45" s="64">
         <v>6</v>
       </c>
-      <c r="D45" s="65">
+      <c r="D45" s="64">
         <v>1</v>
       </c>
-      <c r="E45" s="72">
+      <c r="E45" s="70">
         <v>45462</v>
       </c>
-      <c r="F45" s="73">
+      <c r="F45" s="71">
         <v>0.625</v>
       </c>
-      <c r="G45" s="62">
+      <c r="G45" s="61">
         <f t="shared" ref="G45" si="8">$E45+$F45+TIME(AC45,0,0)</f>
         <v>45462.791666666664</v>
       </c>
@@ -5666,84 +5710,84 @@
       <c r="I45">
         <v>-63.010885000000002</v>
       </c>
-      <c r="J45" s="74">
+      <c r="J45" s="72">
         <v>45466</v>
       </c>
-      <c r="K45" s="73">
+      <c r="K45" s="71">
         <v>0.875</v>
       </c>
-      <c r="L45" s="63">
+      <c r="L45" s="62">
         <f t="shared" ref="L45:L46" si="9">$J45+$K45 +TIME($AC45,0,0)</f>
         <v>45467.041666666664</v>
       </c>
-      <c r="M45" s="80">
+      <c r="M45" s="78">
         <v>39.013003333333302</v>
       </c>
-      <c r="N45" s="75">
+      <c r="N45" s="73">
         <v>-63.364616666666699</v>
       </c>
-      <c r="O45" s="65">
+      <c r="O45" s="64">
         <v>4</v>
       </c>
-      <c r="P45" s="65" t="s">
+      <c r="P45" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="Q45" s="64">
+      <c r="Q45" s="63">
         <v>300434066480130</v>
       </c>
-      <c r="R45" s="64" t="s">
+      <c r="R45" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="S45" s="76">
+      <c r="S45" s="74">
         <v>45462.855231481481</v>
       </c>
-      <c r="T45" s="87">
+      <c r="T45" s="84">
         <v>38.307771000000002</v>
       </c>
-      <c r="U45" s="87">
+      <c r="U45" s="84">
         <v>-62.998032000000002</v>
       </c>
-      <c r="V45" s="76">
+      <c r="V45" s="74">
         <v>45465.11142361111</v>
       </c>
-      <c r="W45" s="87">
+      <c r="W45" s="84">
         <v>38.406742000000001</v>
       </c>
-      <c r="X45" s="87">
+      <c r="X45" s="84">
         <v>-62.544604</v>
       </c>
       <c r="Y45" s="25">
         <f t="shared" si="7"/>
         <v>54.148611111100763</v>
       </c>
-      <c r="Z45" s="79"/>
-      <c r="AA45" s="79"/>
-      <c r="AB45" s="65"/>
-      <c r="AC45" s="65">
+      <c r="Z45" s="77"/>
+      <c r="AA45" s="77"/>
+      <c r="AB45" s="64"/>
+      <c r="AC45" s="64">
         <v>4</v>
       </c>
-      <c r="AD45" s="65"/>
-    </row>
-    <row r="46" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="65">
+      <c r="AD45" s="64"/>
+    </row>
+    <row r="46" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="64">
         <v>28</v>
       </c>
-      <c r="B46" s="65" t="s">
+      <c r="B46" s="64" t="s">
         <v>138</v>
       </c>
-      <c r="C46" s="65">
+      <c r="C46" s="64">
         <v>6</v>
       </c>
-      <c r="D46" s="65">
+      <c r="D46" s="64">
         <v>2</v>
       </c>
-      <c r="E46" s="72">
+      <c r="E46" s="70">
         <v>45462</v>
       </c>
-      <c r="F46" s="73">
+      <c r="F46" s="71">
         <v>0.625</v>
       </c>
-      <c r="G46" s="62">
+      <c r="G46" s="61">
         <f t="shared" ref="G46" si="10">$E46+$F46+TIME(AC46,0,0)</f>
         <v>45462.791666666664</v>
       </c>
@@ -5753,63 +5797,63 @@
       <c r="I46">
         <v>-63.010885000000002</v>
       </c>
-      <c r="J46" s="74">
+      <c r="J46" s="72">
         <v>45466</v>
       </c>
-      <c r="K46" s="73">
+      <c r="K46" s="71">
         <v>0.875</v>
       </c>
-      <c r="L46" s="63">
+      <c r="L46" s="62">
         <f t="shared" si="9"/>
         <v>45467.041666666664</v>
       </c>
-      <c r="M46" s="80">
+      <c r="M46" s="78">
         <v>39.013003333333302</v>
       </c>
-      <c r="N46" s="75">
+      <c r="N46" s="73">
         <v>-63.364616666666699</v>
       </c>
-      <c r="O46" s="65">
+      <c r="O46" s="64">
         <v>4</v>
       </c>
-      <c r="P46" s="65" t="s">
+      <c r="P46" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="Q46" s="64">
+      <c r="Q46" s="63">
         <v>300434066480130</v>
       </c>
-      <c r="R46" s="64" t="s">
+      <c r="R46" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="S46" s="76">
+      <c r="S46" s="74">
         <v>45465.271736111114</v>
       </c>
-      <c r="T46" s="87">
+      <c r="T46" s="84">
         <v>38.415380999999996</v>
       </c>
-      <c r="U46" s="87">
+      <c r="U46" s="84">
         <v>-62.463433000000002</v>
       </c>
       <c r="V46" s="28">
         <v>45466.125555555554</v>
       </c>
-      <c r="W46" s="87">
+      <c r="W46" s="84">
         <v>38.532255999999997</v>
       </c>
-      <c r="X46" s="87">
+      <c r="X46" s="84">
         <v>-62.362059000000002</v>
       </c>
       <c r="Y46" s="25">
         <f t="shared" si="7"/>
         <v>20.491666666581295</v>
       </c>
-      <c r="Z46" s="79"/>
-      <c r="AA46" s="79"/>
-      <c r="AB46" s="65"/>
-      <c r="AC46" s="65">
+      <c r="Z46" s="77"/>
+      <c r="AA46" s="77"/>
+      <c r="AB46" s="64"/>
+      <c r="AC46" s="64">
         <v>4</v>
       </c>
-      <c r="AD46" s="65" t="s">
+      <c r="AD46" s="64" t="s">
         <v>131</v>
       </c>
     </row>
@@ -5826,7 +5870,7 @@
       <c r="D47" s="44">
         <v>1</v>
       </c>
-      <c r="E47" s="70">
+      <c r="E47" s="68">
         <v>45462</v>
       </c>
       <c r="F47" s="46">
@@ -5852,10 +5896,10 @@
         <f t="shared" ref="L47" si="11">$J47+$K47 +TIME($AC47,0,0)</f>
         <v>45464.291666666664</v>
       </c>
-      <c r="M47" s="68">
+      <c r="M47" s="66">
         <v>38.309516000000002</v>
       </c>
-      <c r="N47" s="68">
+      <c r="N47" s="66">
         <v>-62.619463000000003</v>
       </c>
       <c r="O47" s="44">
@@ -5864,7 +5908,7 @@
       <c r="P47" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="Q47" s="71">
+      <c r="Q47" s="69">
         <v>300434066489180</v>
       </c>
       <c r="R47" s="47" t="s">
@@ -5873,19 +5917,19 @@
       <c r="S47" s="52">
         <v>45462.84778935185</v>
       </c>
-      <c r="T47" s="68">
+      <c r="T47" s="66">
         <v>38.315800000000003</v>
       </c>
-      <c r="U47" s="68">
+      <c r="U47" s="66">
         <v>-63.012493999999997</v>
       </c>
       <c r="V47" s="52">
         <v>45463.528101851851</v>
       </c>
-      <c r="W47" s="68">
+      <c r="W47" s="66">
         <v>38.311391</v>
       </c>
-      <c r="X47" s="68">
+      <c r="X47" s="66">
         <v>-62.918548000000001</v>
       </c>
       <c r="Y47" s="49">
@@ -5902,196 +5946,359 @@
         <v>132</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="65">
+    <row r="48" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="64">
         <v>30</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="64" t="s">
         <v>139</v>
       </c>
-      <c r="C48" s="65">
+      <c r="C48" s="64">
+        <v>4</v>
+      </c>
+      <c r="D48" s="64">
+        <v>1</v>
+      </c>
+      <c r="E48" s="70">
+        <v>45597</v>
+      </c>
+      <c r="F48" s="79"/>
+      <c r="G48" s="79"/>
+      <c r="H48" s="74"/>
+      <c r="I48" s="79"/>
+      <c r="J48" s="80"/>
+      <c r="K48" s="71"/>
+      <c r="L48" s="71"/>
+      <c r="M48" s="64"/>
+      <c r="N48" s="64"/>
+      <c r="O48" s="64"/>
+      <c r="P48" s="64"/>
+      <c r="Q48" s="63"/>
+      <c r="R48" s="63"/>
+      <c r="S48" s="75"/>
+      <c r="T48" s="64"/>
+      <c r="U48" s="64"/>
+      <c r="W48" s="64"/>
+      <c r="X48" s="64"/>
+      <c r="Y48" s="76">
+        <f t="shared" ref="Y48:Y52" si="12">(V48-S48)*1440/60</f>
+        <v>0</v>
+      </c>
+      <c r="Z48" s="77"/>
+      <c r="AA48" s="77"/>
+      <c r="AB48" s="64"/>
+      <c r="AC48" s="64"/>
+      <c r="AD48" s="64"/>
+    </row>
+    <row r="49" spans="1:30" s="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="44">
+        <v>31</v>
+      </c>
+      <c r="B49" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C49" s="44">
         <v>5</v>
       </c>
-      <c r="D48" s="65">
+      <c r="D49" s="44">
         <v>1</v>
       </c>
-      <c r="E48" s="81"/>
-      <c r="F48" s="82"/>
-      <c r="G48" s="82"/>
-      <c r="H48" s="76"/>
-      <c r="I48" s="82"/>
-      <c r="J48" s="83"/>
-      <c r="K48" s="73"/>
-      <c r="L48" s="73"/>
-      <c r="M48" s="65"/>
-      <c r="N48" s="65"/>
-      <c r="O48" s="65"/>
-      <c r="P48" s="65"/>
-      <c r="Q48" s="64"/>
-      <c r="R48" s="64"/>
-      <c r="S48" s="77"/>
-      <c r="T48" s="65"/>
-      <c r="U48" s="65"/>
-      <c r="W48" s="65"/>
-      <c r="X48" s="65"/>
-      <c r="Y48" s="78"/>
-      <c r="Z48" s="79"/>
-      <c r="AA48" s="79"/>
-      <c r="AB48" s="65"/>
-      <c r="AC48" s="65"/>
-      <c r="AD48" s="65"/>
-    </row>
-    <row r="49" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="20">
-        <v>30</v>
-      </c>
-      <c r="B49" s="65" t="s">
-        <v>139</v>
-      </c>
-      <c r="C49" s="20">
+      <c r="E49" s="68">
+        <v>45780</v>
+      </c>
+      <c r="F49" s="88">
+        <v>0.50486111111111109</v>
+      </c>
+      <c r="G49" s="89" t="s">
+        <v>141</v>
+      </c>
+      <c r="H49" s="44">
+        <v>20.020324074074075</v>
+      </c>
+      <c r="I49" s="90">
+        <v>-156.00538</v>
+      </c>
+      <c r="J49" s="45">
+        <v>45782</v>
+      </c>
+      <c r="K49" s="46">
+        <v>0.5</v>
+      </c>
+      <c r="L49" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="M49" s="44">
+        <v>20.222373999999999</v>
+      </c>
+      <c r="N49" s="44">
+        <v>-155.94340500000001</v>
+      </c>
+      <c r="O49" s="44">
+        <v>3</v>
+      </c>
+      <c r="P49" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q49" s="47">
+        <v>300434066482170</v>
+      </c>
+      <c r="R49" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="S49" s="52">
+        <v>45780.951365740744</v>
+      </c>
+      <c r="T49" s="91">
+        <v>20.032706000000001</v>
+      </c>
+      <c r="U49" s="91">
+        <v>-155.999832</v>
+      </c>
+      <c r="V49" s="52">
+        <v>45781.875567129631</v>
+      </c>
+      <c r="W49" s="91">
+        <v>20.074359999999999</v>
+      </c>
+      <c r="X49" s="91">
+        <v>-155.953611</v>
+      </c>
+      <c r="Y49" s="49">
+        <f t="shared" si="12"/>
+        <v>22.180833333288319</v>
+      </c>
+      <c r="Z49" s="50"/>
+      <c r="AA49" s="50"/>
+      <c r="AB49" s="44"/>
+      <c r="AC49" s="44"/>
+      <c r="AD49" s="44" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="50" spans="1:30" s="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="44">
+        <v>31</v>
+      </c>
+      <c r="B50" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" s="44">
         <v>5</v>
       </c>
-      <c r="D49" s="20">
+      <c r="D50" s="44">
         <v>2</v>
       </c>
-      <c r="E49" s="24"/>
-      <c r="F49" s="66"/>
-      <c r="G49" s="66"/>
-      <c r="H49" s="24"/>
-      <c r="I49" s="61"/>
-      <c r="J49" s="20"/>
-      <c r="K49" s="22"/>
-      <c r="L49" s="22"/>
-      <c r="M49" s="20"/>
-      <c r="N49" s="20"/>
-      <c r="O49" s="20"/>
-      <c r="P49" s="20"/>
-      <c r="Q49" s="23"/>
-      <c r="R49" s="23"/>
-      <c r="S49" s="24"/>
-      <c r="T49" s="20"/>
-      <c r="U49" s="20"/>
-      <c r="V49" s="24"/>
-      <c r="W49" s="20"/>
-      <c r="X49" s="20"/>
-      <c r="Y49" s="25"/>
-      <c r="Z49" s="26"/>
-      <c r="AA49" s="26"/>
-      <c r="AB49" s="20"/>
-      <c r="AC49" s="20"/>
-      <c r="AD49" s="20"/>
-    </row>
-    <row r="50" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="20">
-        <v>31</v>
-      </c>
-      <c r="B50" s="65" t="s">
-        <v>139</v>
-      </c>
-      <c r="C50" s="20">
+      <c r="E50" s="68">
+        <v>45780</v>
+      </c>
+      <c r="F50" s="88">
+        <v>0.50486111111111109</v>
+      </c>
+      <c r="G50" s="89" t="s">
+        <v>141</v>
+      </c>
+      <c r="H50" s="44">
+        <v>20.020324074074075</v>
+      </c>
+      <c r="I50" s="90">
+        <v>-156.00538</v>
+      </c>
+      <c r="J50" s="45">
+        <v>45782</v>
+      </c>
+      <c r="K50" s="46">
+        <v>0.5</v>
+      </c>
+      <c r="L50" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="M50" s="44">
+        <v>20.222373999999999</v>
+      </c>
+      <c r="N50" s="44">
+        <v>-155.94340500000001</v>
+      </c>
+      <c r="O50" s="44">
+        <v>3</v>
+      </c>
+      <c r="P50" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q50" s="47">
+        <v>300434066482170</v>
+      </c>
+      <c r="R50" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="S50" s="52">
+        <v>45782.028784722221</v>
+      </c>
+      <c r="T50" s="91">
+        <v>20.127566000000002</v>
+      </c>
+      <c r="U50" s="91">
+        <v>-155.93448900000001</v>
+      </c>
+      <c r="V50" s="52">
+        <v>45782.880578703705</v>
+      </c>
+      <c r="W50" s="91">
+        <v>20.216946</v>
+      </c>
+      <c r="X50" s="91">
+        <v>-155.941529</v>
+      </c>
+      <c r="Y50" s="49">
+        <f t="shared" si="12"/>
+        <v>20.443055555631872</v>
+      </c>
+      <c r="Z50" s="50"/>
+      <c r="AA50" s="50"/>
+      <c r="AB50" s="44"/>
+      <c r="AC50" s="44"/>
+      <c r="AD50" s="44" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="1:30" s="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="64">
+        <v>32</v>
+      </c>
+      <c r="B51" s="64" t="s">
+        <v>140</v>
+      </c>
+      <c r="C51" s="64">
         <v>5</v>
       </c>
-      <c r="D50" s="20">
+      <c r="D51" s="64">
         <v>1</v>
       </c>
-      <c r="E50" s="21"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="21"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="20"/>
-      <c r="N50" s="20"/>
-      <c r="O50" s="20"/>
-      <c r="P50" s="20"/>
-      <c r="Q50" s="23"/>
-      <c r="R50" s="23"/>
-      <c r="S50" s="24"/>
-      <c r="T50" s="20"/>
-      <c r="U50" s="20"/>
-      <c r="V50" s="24"/>
-      <c r="W50" s="20"/>
-      <c r="X50" s="20"/>
-      <c r="Y50" s="25"/>
-      <c r="Z50" s="26"/>
-      <c r="AA50" s="26"/>
-      <c r="AB50" s="20"/>
-      <c r="AC50" s="20"/>
-      <c r="AD50" s="20"/>
-    </row>
-    <row r="51" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="20">
-        <v>32</v>
-      </c>
-      <c r="B51" s="65" t="s">
-        <v>139</v>
-      </c>
-      <c r="C51" s="20">
+      <c r="E51" s="72">
+        <v>45784</v>
+      </c>
+      <c r="F51" s="71"/>
+      <c r="G51" s="71" t="s">
+        <v>144</v>
+      </c>
+      <c r="H51" s="64">
+        <v>19.97148</v>
+      </c>
+      <c r="I51" s="64">
+        <v>-156.08585299999999</v>
+      </c>
+      <c r="J51" s="72"/>
+      <c r="K51" s="71"/>
+      <c r="L51" s="71" t="s">
+        <v>145</v>
+      </c>
+      <c r="M51" s="64"/>
+      <c r="N51" s="64"/>
+      <c r="O51" s="64">
+        <v>3</v>
+      </c>
+      <c r="P51" s="64" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q51" s="63">
+        <v>300434066482170</v>
+      </c>
+      <c r="R51" s="63" t="s">
+        <v>37</v>
+      </c>
+      <c r="S51" s="74">
+        <v>45784.854861111111</v>
+      </c>
+      <c r="T51" s="92">
+        <v>19.972162000000001</v>
+      </c>
+      <c r="U51" s="92">
+        <v>-156.08393000000001</v>
+      </c>
+      <c r="V51" s="74">
+        <v>45785.979861111111</v>
+      </c>
+      <c r="W51" s="92">
+        <v>19.971561000000001</v>
+      </c>
+      <c r="X51" s="92">
+        <v>-156.05051</v>
+      </c>
+      <c r="Y51" s="76">
+        <f t="shared" si="12"/>
+        <v>27</v>
+      </c>
+      <c r="Z51" s="77"/>
+      <c r="AA51" s="77"/>
+      <c r="AB51" s="64"/>
+      <c r="AC51" s="64"/>
+      <c r="AD51" s="64"/>
+    </row>
+    <row r="52" spans="1:30" s="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="44">
+        <v>33</v>
+      </c>
+      <c r="B52" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C52" s="44">
         <v>5</v>
       </c>
-      <c r="D51" s="20">
+      <c r="D52" s="44">
         <v>1</v>
       </c>
-      <c r="E51" s="21"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="22"/>
-      <c r="L51" s="22"/>
-      <c r="M51" s="20"/>
-      <c r="N51" s="20"/>
-      <c r="O51" s="20"/>
-      <c r="P51" s="20"/>
-      <c r="Q51" s="23"/>
-      <c r="R51" s="23"/>
-      <c r="S51" s="24"/>
-      <c r="T51" s="20"/>
-      <c r="U51" s="20"/>
-      <c r="V51" s="24"/>
-      <c r="W51" s="20"/>
-      <c r="X51" s="20"/>
-      <c r="Y51" s="25"/>
-      <c r="Z51" s="26"/>
-      <c r="AA51" s="26"/>
-      <c r="AB51" s="20"/>
-      <c r="AC51" s="20"/>
-      <c r="AD51" s="20"/>
-    </row>
-    <row r="52" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="20"/>
-      <c r="B52" s="20"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="21"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="21"/>
-      <c r="K52" s="22"/>
-      <c r="L52" s="22"/>
-      <c r="M52" s="20"/>
-      <c r="N52" s="20"/>
-      <c r="O52" s="20"/>
-      <c r="P52" s="20"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
-      <c r="S52" s="24"/>
-      <c r="T52" s="20"/>
-      <c r="U52" s="20"/>
-      <c r="V52" s="24"/>
-      <c r="W52" s="20"/>
-      <c r="X52" s="20"/>
-      <c r="Y52" s="25"/>
-      <c r="Z52" s="26"/>
-      <c r="AA52" s="26"/>
-      <c r="AB52" s="20"/>
-      <c r="AC52" s="20"/>
-      <c r="AD52" s="20"/>
+      <c r="E52" s="45"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46" t="s">
+        <v>146</v>
+      </c>
+      <c r="H52" s="44"/>
+      <c r="I52" s="44"/>
+      <c r="J52" s="45"/>
+      <c r="K52" s="46"/>
+      <c r="L52" s="46" t="s">
+        <v>147</v>
+      </c>
+      <c r="M52" s="44"/>
+      <c r="N52" s="44"/>
+      <c r="O52" s="44">
+        <v>3</v>
+      </c>
+      <c r="P52" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q52" s="47">
+        <v>300434066482170</v>
+      </c>
+      <c r="R52" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="S52" s="52">
+        <v>45788.225694444445</v>
+      </c>
+      <c r="T52" s="91">
+        <v>19.937816000000002</v>
+      </c>
+      <c r="U52" s="91">
+        <v>-155.78363999999999</v>
+      </c>
+      <c r="V52" s="52">
+        <v>45789.118055555555</v>
+      </c>
+      <c r="W52" s="91">
+        <v>20.028275000000001</v>
+      </c>
+      <c r="X52" s="91">
+        <v>-155.99986999999999</v>
+      </c>
+      <c r="Y52" s="49">
+        <f t="shared" si="12"/>
+        <v>21.416666666627862</v>
+      </c>
+      <c r="Z52" s="50"/>
+      <c r="AA52" s="50"/>
+      <c r="AB52" s="44"/>
+      <c r="AC52" s="44"/>
+      <c r="AD52" s="44"/>
     </row>
     <row r="53" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="20"/>
@@ -46830,11 +47037,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="86" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
       <c r="D1" s="9" t="s">
         <v>53</v>
       </c>

</xml_diff>